<commit_message>
Add relationship validation reports
</commit_message>
<xml_diff>
--- a/data/exports/duplicate_candidates.xlsx
+++ b/data/exports/duplicate_candidates.xlsx
@@ -7420,7 +7420,7 @@
     </row>
     <row r="2" spans="1:18">
       <c r="A2">
-        <v>5863</v>
+        <v>6645</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
@@ -7476,7 +7476,7 @@
     </row>
     <row r="3" spans="1:18">
       <c r="A3">
-        <v>5775</v>
+        <v>6557</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
@@ -7526,7 +7526,7 @@
     </row>
     <row r="4" spans="1:18">
       <c r="A4">
-        <v>5740</v>
+        <v>6522</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -7582,7 +7582,7 @@
     </row>
     <row r="5" spans="1:18">
       <c r="A5">
-        <v>5630</v>
+        <v>6412</v>
       </c>
       <c r="B5" t="s">
         <v>21</v>
@@ -7638,7 +7638,7 @@
     </row>
     <row r="6" spans="1:18">
       <c r="A6">
-        <v>5648</v>
+        <v>6430</v>
       </c>
       <c r="B6" t="s">
         <v>22</v>
@@ -7694,7 +7694,7 @@
     </row>
     <row r="7" spans="1:18">
       <c r="A7">
-        <v>5693</v>
+        <v>6475</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
@@ -7744,7 +7744,7 @@
     </row>
     <row r="8" spans="1:18">
       <c r="A8">
-        <v>5705</v>
+        <v>6487</v>
       </c>
       <c r="B8" t="s">
         <v>24</v>
@@ -7800,7 +7800,7 @@
     </row>
     <row r="9" spans="1:18">
       <c r="A9">
-        <v>5673</v>
+        <v>6455</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>
@@ -7856,7 +7856,7 @@
     </row>
     <row r="10" spans="1:18">
       <c r="A10">
-        <v>5811</v>
+        <v>6593</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
@@ -7897,7 +7897,7 @@
     </row>
     <row r="11" spans="1:18">
       <c r="A11">
-        <v>5790</v>
+        <v>6572</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
@@ -7953,7 +7953,7 @@
     </row>
     <row r="12" spans="1:18">
       <c r="A12">
-        <v>5748</v>
+        <v>6530</v>
       </c>
       <c r="B12" t="s">
         <v>28</v>
@@ -8009,7 +8009,7 @@
     </row>
     <row r="13" spans="1:18">
       <c r="A13">
-        <v>5853</v>
+        <v>6635</v>
       </c>
       <c r="B13" t="s">
         <v>29</v>
@@ -8062,7 +8062,7 @@
     </row>
     <row r="14" spans="1:18">
       <c r="A14">
-        <v>5854</v>
+        <v>6636</v>
       </c>
       <c r="B14" t="s">
         <v>29</v>
@@ -8115,7 +8115,7 @@
     </row>
     <row r="15" spans="1:18">
       <c r="A15">
-        <v>5855</v>
+        <v>6637</v>
       </c>
       <c r="B15" t="s">
         <v>29</v>
@@ -8168,7 +8168,7 @@
     </row>
     <row r="16" spans="1:18">
       <c r="A16">
-        <v>5856</v>
+        <v>6638</v>
       </c>
       <c r="B16" t="s">
         <v>30</v>
@@ -8218,7 +8218,7 @@
     </row>
     <row r="17" spans="1:18">
       <c r="A17">
-        <v>5857</v>
+        <v>6639</v>
       </c>
       <c r="B17" t="s">
         <v>30</v>
@@ -8268,7 +8268,7 @@
     </row>
     <row r="18" spans="1:18">
       <c r="A18">
-        <v>5858</v>
+        <v>6640</v>
       </c>
       <c r="B18" t="s">
         <v>31</v>
@@ -8318,7 +8318,7 @@
     </row>
     <row r="19" spans="1:18">
       <c r="A19">
-        <v>5738</v>
+        <v>6520</v>
       </c>
       <c r="B19" t="s">
         <v>32</v>
@@ -8374,7 +8374,7 @@
     </row>
     <row r="20" spans="1:18">
       <c r="A20">
-        <v>5777</v>
+        <v>6559</v>
       </c>
       <c r="B20" t="s">
         <v>33</v>
@@ -8424,7 +8424,7 @@
     </row>
     <row r="21" spans="1:18">
       <c r="A21">
-        <v>5903</v>
+        <v>6685</v>
       </c>
       <c r="B21" t="s">
         <v>34</v>
@@ -8480,7 +8480,7 @@
     </row>
     <row r="22" spans="1:18">
       <c r="A22">
-        <v>5820</v>
+        <v>6602</v>
       </c>
       <c r="B22" t="s">
         <v>35</v>
@@ -8533,7 +8533,7 @@
     </row>
     <row r="23" spans="1:18">
       <c r="A23">
-        <v>5821</v>
+        <v>6603</v>
       </c>
       <c r="B23" t="s">
         <v>35</v>
@@ -8586,7 +8586,7 @@
     </row>
     <row r="24" spans="1:18">
       <c r="A24">
-        <v>5830</v>
+        <v>6612</v>
       </c>
       <c r="B24" t="s">
         <v>36</v>
@@ -8642,7 +8642,7 @@
     </row>
     <row r="25" spans="1:18">
       <c r="A25">
-        <v>5804</v>
+        <v>6586</v>
       </c>
       <c r="B25" t="s">
         <v>37</v>
@@ -8695,7 +8695,7 @@
     </row>
     <row r="26" spans="1:18">
       <c r="A26">
-        <v>5805</v>
+        <v>6587</v>
       </c>
       <c r="B26" t="s">
         <v>37</v>
@@ -8751,7 +8751,7 @@
     </row>
     <row r="27" spans="1:18">
       <c r="A27">
-        <v>5807</v>
+        <v>6589</v>
       </c>
       <c r="B27" t="s">
         <v>38</v>
@@ -8804,7 +8804,7 @@
     </row>
     <row r="28" spans="1:18">
       <c r="A28">
-        <v>5694</v>
+        <v>6476</v>
       </c>
       <c r="B28" t="s">
         <v>39</v>
@@ -8860,7 +8860,7 @@
     </row>
     <row r="29" spans="1:18">
       <c r="A29">
-        <v>5802</v>
+        <v>6584</v>
       </c>
       <c r="B29" t="s">
         <v>40</v>
@@ -8901,7 +8901,7 @@
     </row>
     <row r="30" spans="1:18">
       <c r="A30">
-        <v>5803</v>
+        <v>6585</v>
       </c>
       <c r="B30" t="s">
         <v>40</v>
@@ -8945,7 +8945,7 @@
     </row>
     <row r="31" spans="1:18">
       <c r="A31">
-        <v>5806</v>
+        <v>6588</v>
       </c>
       <c r="B31" t="s">
         <v>41</v>
@@ -8986,7 +8986,7 @@
     </row>
     <row r="32" spans="1:18">
       <c r="A32">
-        <v>5907</v>
+        <v>6689</v>
       </c>
       <c r="B32" t="s">
         <v>42</v>
@@ -9042,7 +9042,7 @@
     </row>
     <row r="33" spans="1:18">
       <c r="A33">
-        <v>5728</v>
+        <v>6510</v>
       </c>
       <c r="B33" t="s">
         <v>43</v>
@@ -9098,7 +9098,7 @@
     </row>
     <row r="34" spans="1:18">
       <c r="A34">
-        <v>5729</v>
+        <v>6511</v>
       </c>
       <c r="B34" t="s">
         <v>44</v>
@@ -9139,7 +9139,7 @@
     </row>
     <row r="35" spans="1:18">
       <c r="A35">
-        <v>5769</v>
+        <v>6551</v>
       </c>
       <c r="B35" t="s">
         <v>45</v>
@@ -9195,7 +9195,7 @@
     </row>
     <row r="36" spans="1:18">
       <c r="A36">
-        <v>5755</v>
+        <v>6537</v>
       </c>
       <c r="B36" t="s">
         <v>46</v>
@@ -9248,7 +9248,7 @@
     </row>
     <row r="37" spans="1:18">
       <c r="A37">
-        <v>5756</v>
+        <v>6538</v>
       </c>
       <c r="B37" t="s">
         <v>46</v>
@@ -9304,7 +9304,7 @@
     </row>
     <row r="38" spans="1:18">
       <c r="A38">
-        <v>5758</v>
+        <v>6540</v>
       </c>
       <c r="B38" t="s">
         <v>47</v>
@@ -9357,7 +9357,7 @@
     </row>
     <row r="39" spans="1:18">
       <c r="A39">
-        <v>5761</v>
+        <v>6543</v>
       </c>
       <c r="B39" t="s">
         <v>48</v>
@@ -9404,7 +9404,7 @@
     </row>
     <row r="40" spans="1:18">
       <c r="A40">
-        <v>5762</v>
+        <v>6544</v>
       </c>
       <c r="B40" t="s">
         <v>48</v>
@@ -9454,7 +9454,7 @@
     </row>
     <row r="41" spans="1:18">
       <c r="A41">
-        <v>5801</v>
+        <v>6583</v>
       </c>
       <c r="B41" t="s">
         <v>49</v>
@@ -9501,7 +9501,7 @@
     </row>
     <row r="42" spans="1:18">
       <c r="A42">
-        <v>5816</v>
+        <v>6598</v>
       </c>
       <c r="B42" t="s">
         <v>50</v>
@@ -9554,7 +9554,7 @@
     </row>
     <row r="43" spans="1:18">
       <c r="A43">
-        <v>5817</v>
+        <v>6599</v>
       </c>
       <c r="B43" t="s">
         <v>50</v>
@@ -9607,7 +9607,7 @@
     </row>
     <row r="44" spans="1:18">
       <c r="A44">
-        <v>5828</v>
+        <v>6610</v>
       </c>
       <c r="B44" t="s">
         <v>51</v>
@@ -9663,7 +9663,7 @@
     </row>
     <row r="45" spans="1:18">
       <c r="A45">
-        <v>5661</v>
+        <v>6443</v>
       </c>
       <c r="B45" t="s">
         <v>52</v>
@@ -9713,7 +9713,7 @@
     </row>
     <row r="46" spans="1:18">
       <c r="A46">
-        <v>5926</v>
+        <v>6708</v>
       </c>
       <c r="B46" t="s">
         <v>53</v>
@@ -9769,7 +9769,7 @@
     </row>
     <row r="47" spans="1:18">
       <c r="A47">
-        <v>5641</v>
+        <v>6423</v>
       </c>
       <c r="B47" t="s">
         <v>54</v>
@@ -9822,7 +9822,7 @@
     </row>
     <row r="48" spans="1:18">
       <c r="A48">
-        <v>5792</v>
+        <v>6574</v>
       </c>
       <c r="B48" t="s">
         <v>55</v>
@@ -9875,7 +9875,7 @@
     </row>
     <row r="49" spans="1:18">
       <c r="A49">
-        <v>5826</v>
+        <v>6608</v>
       </c>
       <c r="B49" t="s">
         <v>56</v>
@@ -9931,7 +9931,7 @@
     </row>
     <row r="50" spans="1:18">
       <c r="A50">
-        <v>5640</v>
+        <v>6422</v>
       </c>
       <c r="B50" t="s">
         <v>57</v>
@@ -9978,7 +9978,7 @@
     </row>
     <row r="51" spans="1:18">
       <c r="A51">
-        <v>5891</v>
+        <v>6673</v>
       </c>
       <c r="B51" t="s">
         <v>58</v>
@@ -10028,7 +10028,7 @@
     </row>
     <row r="52" spans="1:18">
       <c r="A52">
-        <v>5739</v>
+        <v>6521</v>
       </c>
       <c r="B52" t="s">
         <v>59</v>
@@ -10084,7 +10084,7 @@
     </row>
     <row r="53" spans="1:18">
       <c r="A53">
-        <v>5840</v>
+        <v>6622</v>
       </c>
       <c r="B53" t="s">
         <v>60</v>
@@ -10137,7 +10137,7 @@
     </row>
     <row r="54" spans="1:18">
       <c r="A54">
-        <v>5845</v>
+        <v>6627</v>
       </c>
       <c r="B54" t="s">
         <v>61</v>
@@ -10190,7 +10190,7 @@
     </row>
     <row r="55" spans="1:18">
       <c r="A55">
-        <v>5920</v>
+        <v>6702</v>
       </c>
       <c r="B55" t="s">
         <v>62</v>
@@ -10243,7 +10243,7 @@
     </row>
     <row r="56" spans="1:18">
       <c r="A56">
-        <v>5643</v>
+        <v>6425</v>
       </c>
       <c r="B56" t="s">
         <v>63</v>
@@ -10287,7 +10287,7 @@
     </row>
     <row r="57" spans="1:18">
       <c r="A57">
-        <v>5751</v>
+        <v>6533</v>
       </c>
       <c r="B57" t="s">
         <v>64</v>
@@ -10343,7 +10343,7 @@
     </row>
     <row r="58" spans="1:18">
       <c r="A58">
-        <v>5843</v>
+        <v>6625</v>
       </c>
       <c r="B58" t="s">
         <v>65</v>
@@ -10396,7 +10396,7 @@
     </row>
     <row r="59" spans="1:18">
       <c r="A59">
-        <v>5675</v>
+        <v>6457</v>
       </c>
       <c r="B59" t="s">
         <v>66</v>
@@ -10449,7 +10449,7 @@
     </row>
     <row r="60" spans="1:18">
       <c r="A60">
-        <v>5598</v>
+        <v>6380</v>
       </c>
       <c r="B60" t="s">
         <v>67</v>
@@ -10502,7 +10502,7 @@
     </row>
     <row r="61" spans="1:18">
       <c r="A61">
-        <v>5864</v>
+        <v>6646</v>
       </c>
       <c r="B61" t="s">
         <v>68</v>
@@ -10555,7 +10555,7 @@
     </row>
     <row r="62" spans="1:18">
       <c r="A62">
-        <v>5852</v>
+        <v>6634</v>
       </c>
       <c r="B62" t="s">
         <v>69</v>
@@ -10608,7 +10608,7 @@
     </row>
     <row r="63" spans="1:18">
       <c r="A63">
-        <v>5766</v>
+        <v>6548</v>
       </c>
       <c r="B63" t="s">
         <v>70</v>
@@ -10664,7 +10664,7 @@
     </row>
     <row r="64" spans="1:18">
       <c r="A64">
-        <v>5730</v>
+        <v>6512</v>
       </c>
       <c r="B64" t="s">
         <v>71</v>
@@ -10717,7 +10717,7 @@
     </row>
     <row r="65" spans="1:18">
       <c r="A65">
-        <v>5718</v>
+        <v>6500</v>
       </c>
       <c r="B65" t="s">
         <v>72</v>
@@ -10764,7 +10764,7 @@
     </row>
     <row r="66" spans="1:18">
       <c r="A66">
-        <v>5742</v>
+        <v>6524</v>
       </c>
       <c r="B66" t="s">
         <v>73</v>
@@ -10820,7 +10820,7 @@
     </row>
     <row r="67" spans="1:18">
       <c r="A67">
-        <v>5682</v>
+        <v>6464</v>
       </c>
       <c r="B67" t="s">
         <v>74</v>
@@ -10870,7 +10870,7 @@
     </row>
     <row r="68" spans="1:18">
       <c r="A68">
-        <v>5938</v>
+        <v>6720</v>
       </c>
       <c r="B68" t="s">
         <v>75</v>
@@ -10920,7 +10920,7 @@
     </row>
     <row r="69" spans="1:18">
       <c r="A69">
-        <v>5736</v>
+        <v>6518</v>
       </c>
       <c r="B69" t="s">
         <v>76</v>
@@ -10976,7 +10976,7 @@
     </row>
     <row r="70" spans="1:18">
       <c r="A70">
-        <v>5933</v>
+        <v>6715</v>
       </c>
       <c r="B70" t="s">
         <v>77</v>
@@ -11032,7 +11032,7 @@
     </row>
     <row r="71" spans="1:18">
       <c r="A71">
-        <v>5763</v>
+        <v>6545</v>
       </c>
       <c r="B71" t="s">
         <v>78</v>
@@ -11079,7 +11079,7 @@
     </row>
     <row r="72" spans="1:18">
       <c r="A72">
-        <v>5764</v>
+        <v>6546</v>
       </c>
       <c r="B72" t="s">
         <v>78</v>
@@ -11129,7 +11129,7 @@
     </row>
     <row r="73" spans="1:18">
       <c r="A73">
-        <v>5813</v>
+        <v>6595</v>
       </c>
       <c r="B73" t="s">
         <v>79</v>
@@ -11176,7 +11176,7 @@
     </row>
     <row r="74" spans="1:18">
       <c r="A74">
-        <v>5860</v>
+        <v>6642</v>
       </c>
       <c r="B74" t="s">
         <v>80</v>
@@ -11220,7 +11220,7 @@
     </row>
     <row r="75" spans="1:18">
       <c r="A75">
-        <v>5927</v>
+        <v>6709</v>
       </c>
       <c r="B75" t="s">
         <v>81</v>
@@ -11273,7 +11273,7 @@
     </row>
     <row r="76" spans="1:18">
       <c r="A76">
-        <v>5786</v>
+        <v>6568</v>
       </c>
       <c r="B76" t="s">
         <v>82</v>
@@ -11329,7 +11329,7 @@
     </row>
     <row r="77" spans="1:18">
       <c r="A77">
-        <v>5600</v>
+        <v>6382</v>
       </c>
       <c r="B77" t="s">
         <v>83</v>
@@ -11382,7 +11382,7 @@
     </row>
     <row r="78" spans="1:18">
       <c r="A78">
-        <v>5824</v>
+        <v>6606</v>
       </c>
       <c r="B78" t="s">
         <v>84</v>
@@ -11435,7 +11435,7 @@
     </row>
     <row r="79" spans="1:18">
       <c r="A79">
-        <v>5825</v>
+        <v>6607</v>
       </c>
       <c r="B79" t="s">
         <v>84</v>
@@ -11488,7 +11488,7 @@
     </row>
     <row r="80" spans="1:18">
       <c r="A80">
-        <v>5833</v>
+        <v>6615</v>
       </c>
       <c r="B80" t="s">
         <v>85</v>
@@ -11544,7 +11544,7 @@
     </row>
     <row r="81" spans="1:18">
       <c r="A81">
-        <v>5788</v>
+        <v>6570</v>
       </c>
       <c r="B81" t="s">
         <v>86</v>
@@ -11600,7 +11600,7 @@
     </row>
     <row r="82" spans="1:18">
       <c r="A82">
-        <v>5773</v>
+        <v>6555</v>
       </c>
       <c r="B82" t="s">
         <v>87</v>
@@ -11656,7 +11656,7 @@
     </row>
     <row r="83" spans="1:18">
       <c r="A83">
-        <v>5697</v>
+        <v>6479</v>
       </c>
       <c r="B83" t="s">
         <v>88</v>
@@ -11712,7 +11712,7 @@
     </row>
     <row r="84" spans="1:18">
       <c r="A84">
-        <v>5698</v>
+        <v>6480</v>
       </c>
       <c r="B84" t="s">
         <v>88</v>
@@ -11768,7 +11768,7 @@
     </row>
     <row r="85" spans="1:18">
       <c r="A85">
-        <v>5715</v>
+        <v>6497</v>
       </c>
       <c r="B85" t="s">
         <v>89</v>
@@ -11824,7 +11824,7 @@
     </row>
     <row r="86" spans="1:18">
       <c r="A86">
-        <v>5901</v>
+        <v>6683</v>
       </c>
       <c r="B86" t="s">
         <v>90</v>
@@ -11880,7 +11880,7 @@
     </row>
     <row r="87" spans="1:18">
       <c r="A87">
-        <v>5709</v>
+        <v>6491</v>
       </c>
       <c r="B87" t="s">
         <v>91</v>
@@ -11936,7 +11936,7 @@
     </row>
     <row r="88" spans="1:18">
       <c r="A88">
-        <v>5862</v>
+        <v>6644</v>
       </c>
       <c r="B88" t="s">
         <v>92</v>
@@ -11992,7 +11992,7 @@
     </row>
     <row r="89" spans="1:18">
       <c r="A89">
-        <v>5623</v>
+        <v>6405</v>
       </c>
       <c r="B89" t="s">
         <v>93</v>
@@ -12048,7 +12048,7 @@
     </row>
     <row r="90" spans="1:18">
       <c r="A90">
-        <v>5624</v>
+        <v>6406</v>
       </c>
       <c r="B90" t="s">
         <v>93</v>
@@ -12104,7 +12104,7 @@
     </row>
     <row r="91" spans="1:18">
       <c r="A91">
-        <v>5631</v>
+        <v>6413</v>
       </c>
       <c r="B91" t="s">
         <v>94</v>
@@ -12157,7 +12157,7 @@
     </row>
     <row r="92" spans="1:18">
       <c r="A92">
-        <v>5771</v>
+        <v>6553</v>
       </c>
       <c r="B92" t="s">
         <v>95</v>
@@ -12210,7 +12210,7 @@
     </row>
     <row r="93" spans="1:18">
       <c r="A93">
-        <v>5619</v>
+        <v>6401</v>
       </c>
       <c r="B93" t="s">
         <v>96</v>
@@ -12254,7 +12254,7 @@
     </row>
     <row r="94" spans="1:18">
       <c r="A94">
-        <v>5867</v>
+        <v>6649</v>
       </c>
       <c r="B94" t="s">
         <v>97</v>
@@ -12310,7 +12310,7 @@
     </row>
     <row r="95" spans="1:18">
       <c r="A95">
-        <v>5679</v>
+        <v>6461</v>
       </c>
       <c r="B95" t="s">
         <v>98</v>
@@ -12363,7 +12363,7 @@
     </row>
     <row r="96" spans="1:18">
       <c r="A96">
-        <v>5848</v>
+        <v>6630</v>
       </c>
       <c r="B96" t="s">
         <v>99</v>
@@ -12416,7 +12416,7 @@
     </row>
     <row r="97" spans="1:18">
       <c r="A97">
-        <v>5923</v>
+        <v>6705</v>
       </c>
       <c r="B97" t="s">
         <v>100</v>
@@ -12469,7 +12469,7 @@
     </row>
     <row r="98" spans="1:18">
       <c r="A98">
-        <v>5683</v>
+        <v>6465</v>
       </c>
       <c r="B98" t="s">
         <v>101</v>
@@ -12525,7 +12525,7 @@
     </row>
     <row r="99" spans="1:18">
       <c r="A99">
-        <v>5638</v>
+        <v>6420</v>
       </c>
       <c r="B99" t="s">
         <v>102</v>
@@ -12569,7 +12569,7 @@
     </row>
     <row r="100" spans="1:18">
       <c r="A100">
-        <v>5639</v>
+        <v>6421</v>
       </c>
       <c r="B100" t="s">
         <v>102</v>
@@ -12613,7 +12613,7 @@
     </row>
     <row r="101" spans="1:18">
       <c r="A101">
-        <v>5701</v>
+        <v>6483</v>
       </c>
       <c r="B101" t="s">
         <v>103</v>
@@ -12657,7 +12657,7 @@
     </row>
     <row r="102" spans="1:18">
       <c r="A102">
-        <v>5934</v>
+        <v>6716</v>
       </c>
       <c r="B102" t="s">
         <v>104</v>
@@ -12698,7 +12698,7 @@
     </row>
     <row r="103" spans="1:18">
       <c r="A103">
-        <v>5809</v>
+        <v>6591</v>
       </c>
       <c r="B103" t="s">
         <v>105</v>
@@ -12739,7 +12739,7 @@
     </row>
     <row r="104" spans="1:18">
       <c r="A104">
-        <v>5656</v>
+        <v>6438</v>
       </c>
       <c r="B104" t="s">
         <v>106</v>
@@ -12789,7 +12789,7 @@
     </row>
     <row r="105" spans="1:18">
       <c r="A105">
-        <v>5609</v>
+        <v>6391</v>
       </c>
       <c r="B105" t="s">
         <v>107</v>
@@ -12842,7 +12842,7 @@
     </row>
     <row r="106" spans="1:18">
       <c r="A106">
-        <v>5913</v>
+        <v>6695</v>
       </c>
       <c r="B106" t="s">
         <v>108</v>
@@ -12892,7 +12892,7 @@
     </row>
     <row r="107" spans="1:18">
       <c r="A107">
-        <v>5837</v>
+        <v>6619</v>
       </c>
       <c r="B107" t="s">
         <v>109</v>
@@ -12945,7 +12945,7 @@
     </row>
     <row r="108" spans="1:18">
       <c r="A108">
-        <v>5889</v>
+        <v>6671</v>
       </c>
       <c r="B108" t="s">
         <v>110</v>
@@ -12992,7 +12992,7 @@
     </row>
     <row r="109" spans="1:18">
       <c r="A109">
-        <v>5841</v>
+        <v>6623</v>
       </c>
       <c r="B109" t="s">
         <v>111</v>
@@ -13045,7 +13045,7 @@
     </row>
     <row r="110" spans="1:18">
       <c r="A110">
-        <v>5859</v>
+        <v>6641</v>
       </c>
       <c r="B110" t="s">
         <v>112</v>
@@ -13083,7 +13083,7 @@
     </row>
     <row r="111" spans="1:18">
       <c r="A111">
-        <v>5722</v>
+        <v>6504</v>
       </c>
       <c r="B111" t="s">
         <v>113</v>
@@ -13139,7 +13139,7 @@
     </row>
     <row r="112" spans="1:18">
       <c r="A112">
-        <v>5636</v>
+        <v>6418</v>
       </c>
       <c r="B112" t="s">
         <v>114</v>
@@ -13189,7 +13189,7 @@
     </row>
     <row r="113" spans="1:18">
       <c r="A113">
-        <v>5637</v>
+        <v>6419</v>
       </c>
       <c r="B113" t="s">
         <v>114</v>
@@ -13239,7 +13239,7 @@
     </row>
     <row r="114" spans="1:18">
       <c r="A114">
-        <v>5700</v>
+        <v>6482</v>
       </c>
       <c r="B114" t="s">
         <v>115</v>
@@ -13289,7 +13289,7 @@
     </row>
     <row r="115" spans="1:18">
       <c r="A115">
-        <v>5626</v>
+        <v>6408</v>
       </c>
       <c r="B115" t="s">
         <v>116</v>
@@ -13333,7 +13333,7 @@
     </row>
     <row r="116" spans="1:18">
       <c r="A116">
-        <v>5627</v>
+        <v>6409</v>
       </c>
       <c r="B116" t="s">
         <v>116</v>
@@ -13377,7 +13377,7 @@
     </row>
     <row r="117" spans="1:18">
       <c r="A117">
-        <v>5699</v>
+        <v>6481</v>
       </c>
       <c r="B117" t="s">
         <v>117</v>
@@ -13421,7 +13421,7 @@
     </row>
     <row r="118" spans="1:18">
       <c r="A118">
-        <v>5885</v>
+        <v>6667</v>
       </c>
       <c r="B118" t="s">
         <v>118</v>
@@ -13471,7 +13471,7 @@
     </row>
     <row r="119" spans="1:18">
       <c r="A119">
-        <v>5663</v>
+        <v>6445</v>
       </c>
       <c r="B119" t="s">
         <v>119</v>
@@ -13521,7 +13521,7 @@
     </row>
     <row r="120" spans="1:18">
       <c r="A120">
-        <v>5674</v>
+        <v>6456</v>
       </c>
       <c r="B120" t="s">
         <v>120</v>
@@ -13577,7 +13577,7 @@
     </row>
     <row r="121" spans="1:18">
       <c r="A121">
-        <v>5687</v>
+        <v>6469</v>
       </c>
       <c r="B121" t="s">
         <v>121</v>
@@ -13615,7 +13615,7 @@
     </row>
     <row r="122" spans="1:18">
       <c r="A122">
-        <v>5778</v>
+        <v>6560</v>
       </c>
       <c r="B122" t="s">
         <v>122</v>
@@ -13671,7 +13671,7 @@
     </row>
     <row r="123" spans="1:18">
       <c r="A123">
-        <v>5781</v>
+        <v>6563</v>
       </c>
       <c r="B123" t="s">
         <v>123</v>
@@ -13727,7 +13727,7 @@
     </row>
     <row r="124" spans="1:18">
       <c r="A124">
-        <v>5835</v>
+        <v>6617</v>
       </c>
       <c r="B124" t="s">
         <v>124</v>
@@ -13780,7 +13780,7 @@
     </row>
     <row r="125" spans="1:18">
       <c r="A125">
-        <v>5888</v>
+        <v>6670</v>
       </c>
       <c r="B125" t="s">
         <v>125</v>
@@ -13830,7 +13830,7 @@
     </row>
     <row r="126" spans="1:18">
       <c r="A126">
-        <v>5836</v>
+        <v>6618</v>
       </c>
       <c r="B126" t="s">
         <v>126</v>
@@ -13883,7 +13883,7 @@
     </row>
     <row r="127" spans="1:18">
       <c r="A127">
-        <v>5613</v>
+        <v>6395</v>
       </c>
       <c r="B127" t="s">
         <v>127</v>
@@ -13936,7 +13936,7 @@
     </row>
     <row r="128" spans="1:18">
       <c r="A128">
-        <v>5662</v>
+        <v>6444</v>
       </c>
       <c r="B128" t="s">
         <v>128</v>
@@ -13980,7 +13980,7 @@
     </row>
     <row r="129" spans="1:18">
       <c r="A129">
-        <v>5900</v>
+        <v>6682</v>
       </c>
       <c r="B129" t="s">
         <v>129</v>
@@ -14036,7 +14036,7 @@
     </row>
     <row r="130" spans="1:18">
       <c r="A130">
-        <v>5735</v>
+        <v>6517</v>
       </c>
       <c r="B130" t="s">
         <v>130</v>
@@ -14092,7 +14092,7 @@
     </row>
     <row r="131" spans="1:18">
       <c r="A131">
-        <v>5743</v>
+        <v>6525</v>
       </c>
       <c r="B131" t="s">
         <v>131</v>
@@ -14148,7 +14148,7 @@
     </row>
     <row r="132" spans="1:18">
       <c r="A132">
-        <v>5721</v>
+        <v>6503</v>
       </c>
       <c r="B132" t="s">
         <v>132</v>
@@ -14204,7 +14204,7 @@
     </row>
     <row r="133" spans="1:18">
       <c r="A133">
-        <v>5849</v>
+        <v>6631</v>
       </c>
       <c r="B133" t="s">
         <v>133</v>
@@ -14257,7 +14257,7 @@
     </row>
     <row r="134" spans="1:18">
       <c r="A134">
-        <v>5719</v>
+        <v>6501</v>
       </c>
       <c r="B134" t="s">
         <v>134</v>
@@ -14313,7 +14313,7 @@
     </row>
     <row r="135" spans="1:18">
       <c r="A135">
-        <v>5880</v>
+        <v>6662</v>
       </c>
       <c r="B135" t="s">
         <v>135</v>
@@ -14369,7 +14369,7 @@
     </row>
     <row r="136" spans="1:18">
       <c r="A136">
-        <v>5665</v>
+        <v>6447</v>
       </c>
       <c r="B136" t="s">
         <v>136</v>
@@ -14413,7 +14413,7 @@
     </row>
     <row r="137" spans="1:18">
       <c r="A137">
-        <v>5892</v>
+        <v>6674</v>
       </c>
       <c r="B137" t="s">
         <v>137</v>
@@ -14463,7 +14463,7 @@
     </row>
     <row r="138" spans="1:18">
       <c r="A138">
-        <v>5660</v>
+        <v>6442</v>
       </c>
       <c r="B138" t="s">
         <v>138</v>
@@ -14513,7 +14513,7 @@
     </row>
     <row r="139" spans="1:18">
       <c r="A139">
-        <v>5680</v>
+        <v>6462</v>
       </c>
       <c r="B139" t="s">
         <v>139</v>
@@ -14569,7 +14569,7 @@
     </row>
     <row r="140" spans="1:18">
       <c r="A140">
-        <v>5770</v>
+        <v>6552</v>
       </c>
       <c r="B140" t="s">
         <v>140</v>
@@ -14625,7 +14625,7 @@
     </row>
     <row r="141" spans="1:18">
       <c r="A141">
-        <v>5659</v>
+        <v>6441</v>
       </c>
       <c r="B141" t="s">
         <v>141</v>
@@ -14663,7 +14663,7 @@
     </row>
     <row r="142" spans="1:18">
       <c r="A142">
-        <v>5925</v>
+        <v>6707</v>
       </c>
       <c r="B142" t="s">
         <v>142</v>
@@ -14716,7 +14716,7 @@
     </row>
     <row r="143" spans="1:18">
       <c r="A143">
-        <v>5686</v>
+        <v>6468</v>
       </c>
       <c r="B143" t="s">
         <v>143</v>
@@ -14769,7 +14769,7 @@
     </row>
     <row r="144" spans="1:18">
       <c r="A144">
-        <v>5616</v>
+        <v>6398</v>
       </c>
       <c r="B144" t="s">
         <v>144</v>
@@ -14822,7 +14822,7 @@
     </row>
     <row r="145" spans="1:18">
       <c r="A145">
-        <v>5783</v>
+        <v>6565</v>
       </c>
       <c r="B145" t="s">
         <v>145</v>
@@ -14878,7 +14878,7 @@
     </row>
     <row r="146" spans="1:18">
       <c r="A146">
-        <v>5784</v>
+        <v>6566</v>
       </c>
       <c r="B146" t="s">
         <v>145</v>
@@ -14934,7 +14934,7 @@
     </row>
     <row r="147" spans="1:18">
       <c r="A147">
-        <v>5785</v>
+        <v>6567</v>
       </c>
       <c r="B147" t="s">
         <v>146</v>
@@ -14990,7 +14990,7 @@
     </row>
     <row r="148" spans="1:18">
       <c r="A148">
-        <v>5910</v>
+        <v>6692</v>
       </c>
       <c r="B148" t="s">
         <v>147</v>
@@ -15046,7 +15046,7 @@
     </row>
     <row r="149" spans="1:18">
       <c r="A149">
-        <v>5882</v>
+        <v>6664</v>
       </c>
       <c r="B149" t="s">
         <v>148</v>
@@ -15102,7 +15102,7 @@
     </row>
     <row r="150" spans="1:18">
       <c r="A150">
-        <v>5798</v>
+        <v>6580</v>
       </c>
       <c r="B150" t="s">
         <v>149</v>
@@ -15155,7 +15155,7 @@
     </row>
     <row r="151" spans="1:18">
       <c r="A151">
-        <v>5713</v>
+        <v>6495</v>
       </c>
       <c r="B151" t="s">
         <v>150</v>
@@ -15211,7 +15211,7 @@
     </row>
     <row r="152" spans="1:18">
       <c r="A152">
-        <v>5711</v>
+        <v>6493</v>
       </c>
       <c r="B152" t="s">
         <v>151</v>
@@ -15267,7 +15267,7 @@
     </row>
     <row r="153" spans="1:18">
       <c r="A153">
-        <v>5844</v>
+        <v>6626</v>
       </c>
       <c r="B153" t="s">
         <v>152</v>
@@ -15320,7 +15320,7 @@
     </row>
     <row r="154" spans="1:18">
       <c r="A154">
-        <v>5690</v>
+        <v>6472</v>
       </c>
       <c r="B154" t="s">
         <v>153</v>
@@ -15376,7 +15376,7 @@
     </row>
     <row r="155" spans="1:18">
       <c r="A155">
-        <v>5902</v>
+        <v>6684</v>
       </c>
       <c r="B155" t="s">
         <v>154</v>
@@ -15432,7 +15432,7 @@
     </row>
     <row r="156" spans="1:18">
       <c r="A156">
-        <v>5776</v>
+        <v>6558</v>
       </c>
       <c r="B156" t="s">
         <v>155</v>
@@ -15482,7 +15482,7 @@
     </row>
     <row r="157" spans="1:18">
       <c r="A157">
-        <v>5710</v>
+        <v>6492</v>
       </c>
       <c r="B157" t="s">
         <v>156</v>
@@ -15538,7 +15538,7 @@
     </row>
     <row r="158" spans="1:18">
       <c r="A158">
-        <v>5810</v>
+        <v>6592</v>
       </c>
       <c r="B158" t="s">
         <v>157</v>
@@ -15579,7 +15579,7 @@
     </row>
     <row r="159" spans="1:18">
       <c r="A159">
-        <v>5831</v>
+        <v>6613</v>
       </c>
       <c r="B159" t="s">
         <v>158</v>
@@ -15629,7 +15629,7 @@
     </row>
     <row r="160" spans="1:18">
       <c r="A160">
-        <v>5941</v>
+        <v>6723</v>
       </c>
       <c r="B160" t="s">
         <v>159</v>
@@ -15685,7 +15685,7 @@
     </row>
     <row r="161" spans="1:18">
       <c r="A161">
-        <v>5625</v>
+        <v>6407</v>
       </c>
       <c r="B161" t="s">
         <v>160</v>
@@ -15741,7 +15741,7 @@
     </row>
     <row r="162" spans="1:18">
       <c r="A162">
-        <v>5808</v>
+        <v>6590</v>
       </c>
       <c r="B162" t="s">
         <v>161</v>
@@ -15794,7 +15794,7 @@
     </row>
     <row r="163" spans="1:18">
       <c r="A163">
-        <v>5842</v>
+        <v>6624</v>
       </c>
       <c r="B163" t="s">
         <v>162</v>
@@ -15847,7 +15847,7 @@
     </row>
     <row r="164" spans="1:18">
       <c r="A164">
-        <v>5655</v>
+        <v>6437</v>
       </c>
       <c r="B164" t="s">
         <v>163</v>
@@ -15885,7 +15885,7 @@
     </row>
     <row r="165" spans="1:18">
       <c r="A165">
-        <v>5899</v>
+        <v>6681</v>
       </c>
       <c r="B165" t="s">
         <v>164</v>
@@ -15941,7 +15941,7 @@
     </row>
     <row r="166" spans="1:18">
       <c r="A166">
-        <v>5681</v>
+        <v>6463</v>
       </c>
       <c r="B166" t="s">
         <v>165</v>
@@ -15997,7 +15997,7 @@
     </row>
     <row r="167" spans="1:18">
       <c r="A167">
-        <v>5688</v>
+        <v>6470</v>
       </c>
       <c r="B167" t="s">
         <v>166</v>
@@ -16050,7 +16050,7 @@
     </row>
     <row r="168" spans="1:18">
       <c r="A168">
-        <v>5676</v>
+        <v>6458</v>
       </c>
       <c r="B168" t="s">
         <v>167</v>
@@ -16103,7 +16103,7 @@
     </row>
     <row r="169" spans="1:18">
       <c r="A169">
-        <v>5723</v>
+        <v>6505</v>
       </c>
       <c r="B169" t="s">
         <v>168</v>
@@ -16147,7 +16147,7 @@
     </row>
     <row r="170" spans="1:18">
       <c r="A170">
-        <v>5617</v>
+        <v>6399</v>
       </c>
       <c r="B170" t="s">
         <v>169</v>
@@ -16203,7 +16203,7 @@
     </row>
     <row r="171" spans="1:18">
       <c r="A171">
-        <v>5905</v>
+        <v>6687</v>
       </c>
       <c r="B171" t="s">
         <v>170</v>
@@ -16259,7 +16259,7 @@
     </row>
     <row r="172" spans="1:18">
       <c r="A172">
-        <v>5794</v>
+        <v>6576</v>
       </c>
       <c r="B172" t="s">
         <v>171</v>
@@ -16312,7 +16312,7 @@
     </row>
     <row r="173" spans="1:18">
       <c r="A173">
-        <v>5912</v>
+        <v>6694</v>
       </c>
       <c r="B173" t="s">
         <v>172</v>
@@ -16368,7 +16368,7 @@
     </row>
     <row r="174" spans="1:18">
       <c r="A174">
-        <v>5915</v>
+        <v>6697</v>
       </c>
       <c r="B174" t="s">
         <v>173</v>
@@ -16421,7 +16421,7 @@
     </row>
     <row r="175" spans="1:18">
       <c r="A175">
-        <v>5747</v>
+        <v>6529</v>
       </c>
       <c r="B175" t="s">
         <v>174</v>
@@ -16471,7 +16471,7 @@
     </row>
     <row r="176" spans="1:18">
       <c r="A176">
-        <v>5726</v>
+        <v>6508</v>
       </c>
       <c r="B176" t="s">
         <v>175</v>
@@ -16527,7 +16527,7 @@
     </row>
     <row r="177" spans="1:18">
       <c r="A177">
-        <v>5908</v>
+        <v>6690</v>
       </c>
       <c r="B177" t="s">
         <v>176</v>
@@ -16571,7 +16571,7 @@
     </row>
     <row r="178" spans="1:18">
       <c r="A178">
-        <v>5838</v>
+        <v>6620</v>
       </c>
       <c r="B178" t="s">
         <v>177</v>
@@ -16627,7 +16627,7 @@
     </row>
     <row r="179" spans="1:18">
       <c r="A179">
-        <v>5909</v>
+        <v>6691</v>
       </c>
       <c r="B179" t="s">
         <v>178</v>
@@ -16683,7 +16683,7 @@
     </row>
     <row r="180" spans="1:18">
       <c r="A180">
-        <v>5707</v>
+        <v>6489</v>
       </c>
       <c r="B180" t="s">
         <v>179</v>
@@ -16739,7 +16739,7 @@
     </row>
     <row r="181" spans="1:18">
       <c r="A181">
-        <v>5608</v>
+        <v>6390</v>
       </c>
       <c r="B181" t="s">
         <v>180</v>
@@ -16789,7 +16789,7 @@
     </row>
     <row r="182" spans="1:18">
       <c r="A182">
-        <v>5605</v>
+        <v>6387</v>
       </c>
       <c r="B182" t="s">
         <v>181</v>
@@ -16842,7 +16842,7 @@
     </row>
     <row r="183" spans="1:18">
       <c r="A183">
-        <v>5601</v>
+        <v>6383</v>
       </c>
       <c r="B183" t="s">
         <v>182</v>
@@ -16892,7 +16892,7 @@
     </row>
     <row r="184" spans="1:18">
       <c r="A184">
-        <v>5670</v>
+        <v>6452</v>
       </c>
       <c r="B184" t="s">
         <v>183</v>
@@ -16942,7 +16942,7 @@
     </row>
     <row r="185" spans="1:18">
       <c r="A185">
-        <v>5930</v>
+        <v>6712</v>
       </c>
       <c r="B185" t="s">
         <v>184</v>
@@ -16998,7 +16998,7 @@
     </row>
     <row r="186" spans="1:18">
       <c r="A186">
-        <v>5744</v>
+        <v>6526</v>
       </c>
       <c r="B186" t="s">
         <v>185</v>
@@ -17054,7 +17054,7 @@
     </row>
     <row r="187" spans="1:18">
       <c r="A187">
-        <v>5745</v>
+        <v>6527</v>
       </c>
       <c r="B187" t="s">
         <v>186</v>
@@ -17110,7 +17110,7 @@
     </row>
     <row r="188" spans="1:18">
       <c r="A188">
-        <v>5935</v>
+        <v>6717</v>
       </c>
       <c r="B188" t="s">
         <v>187</v>
@@ -17166,7 +17166,7 @@
     </row>
     <row r="189" spans="1:18">
       <c r="A189">
-        <v>5633</v>
+        <v>6415</v>
       </c>
       <c r="B189" t="s">
         <v>188</v>
@@ -17219,7 +17219,7 @@
     </row>
     <row r="190" spans="1:18">
       <c r="A190">
-        <v>5634</v>
+        <v>6416</v>
       </c>
       <c r="B190" t="s">
         <v>188</v>
@@ -17272,7 +17272,7 @@
     </row>
     <row r="191" spans="1:18">
       <c r="A191">
-        <v>5883</v>
+        <v>6665</v>
       </c>
       <c r="B191" t="s">
         <v>189</v>
@@ -17328,7 +17328,7 @@
     </row>
     <row r="192" spans="1:18">
       <c r="A192">
-        <v>5878</v>
+        <v>6660</v>
       </c>
       <c r="B192" t="s">
         <v>190</v>
@@ -17384,7 +17384,7 @@
     </row>
     <row r="193" spans="1:18">
       <c r="A193">
-        <v>5746</v>
+        <v>6528</v>
       </c>
       <c r="B193" t="s">
         <v>191</v>
@@ -17440,7 +17440,7 @@
     </row>
     <row r="194" spans="1:18">
       <c r="A194">
-        <v>5865</v>
+        <v>6647</v>
       </c>
       <c r="B194" t="s">
         <v>192</v>
@@ -17493,7 +17493,7 @@
     </row>
     <row r="195" spans="1:18">
       <c r="A195">
-        <v>5866</v>
+        <v>6648</v>
       </c>
       <c r="B195" t="s">
         <v>192</v>
@@ -17546,7 +17546,7 @@
     </row>
     <row r="196" spans="1:18">
       <c r="A196">
-        <v>5911</v>
+        <v>6693</v>
       </c>
       <c r="B196" t="s">
         <v>193</v>
@@ -17596,7 +17596,7 @@
     </row>
     <row r="197" spans="1:18">
       <c r="A197">
-        <v>5779</v>
+        <v>6561</v>
       </c>
       <c r="B197" t="s">
         <v>194</v>
@@ -17652,7 +17652,7 @@
     </row>
     <row r="198" spans="1:18">
       <c r="A198">
-        <v>5937</v>
+        <v>6719</v>
       </c>
       <c r="B198" t="s">
         <v>195</v>
@@ -17708,7 +17708,7 @@
     </row>
     <row r="199" spans="1:18">
       <c r="A199">
-        <v>5914</v>
+        <v>6696</v>
       </c>
       <c r="B199" t="s">
         <v>196</v>
@@ -17761,7 +17761,7 @@
     </row>
     <row r="200" spans="1:18">
       <c r="A200">
-        <v>5620</v>
+        <v>6402</v>
       </c>
       <c r="B200" t="s">
         <v>197</v>
@@ -17817,7 +17817,7 @@
     </row>
     <row r="201" spans="1:18">
       <c r="A201">
-        <v>5621</v>
+        <v>6403</v>
       </c>
       <c r="B201" t="s">
         <v>197</v>
@@ -17873,7 +17873,7 @@
     </row>
     <row r="202" spans="1:18">
       <c r="A202">
-        <v>5622</v>
+        <v>6404</v>
       </c>
       <c r="B202" t="s">
         <v>197</v>
@@ -17929,7 +17929,7 @@
     </row>
     <row r="203" spans="1:18">
       <c r="A203">
-        <v>5695</v>
+        <v>6477</v>
       </c>
       <c r="B203" t="s">
         <v>198</v>
@@ -17985,7 +17985,7 @@
     </row>
     <row r="204" spans="1:18">
       <c r="A204">
-        <v>5696</v>
+        <v>6478</v>
       </c>
       <c r="B204" t="s">
         <v>198</v>
@@ -18041,7 +18041,7 @@
     </row>
     <row r="205" spans="1:18">
       <c r="A205">
-        <v>5714</v>
+        <v>6496</v>
       </c>
       <c r="B205" t="s">
         <v>199</v>
@@ -18097,7 +18097,7 @@
     </row>
     <row r="206" spans="1:18">
       <c r="A206">
-        <v>5607</v>
+        <v>6389</v>
       </c>
       <c r="B206" t="s">
         <v>200</v>
@@ -18144,7 +18144,7 @@
     </row>
     <row r="207" spans="1:18">
       <c r="A207">
-        <v>5921</v>
+        <v>6703</v>
       </c>
       <c r="B207" t="s">
         <v>201</v>
@@ -18200,7 +18200,7 @@
     </row>
     <row r="208" spans="1:18">
       <c r="A208">
-        <v>5922</v>
+        <v>6704</v>
       </c>
       <c r="B208" t="s">
         <v>201</v>
@@ -18256,7 +18256,7 @@
     </row>
     <row r="209" spans="1:18">
       <c r="A209">
-        <v>5924</v>
+        <v>6706</v>
       </c>
       <c r="B209" t="s">
         <v>202</v>
@@ -18312,7 +18312,7 @@
     </row>
     <row r="210" spans="1:18">
       <c r="A210">
-        <v>5668</v>
+        <v>6450</v>
       </c>
       <c r="B210" t="s">
         <v>203</v>
@@ -18362,7 +18362,7 @@
     </row>
     <row r="211" spans="1:18">
       <c r="A211">
-        <v>5932</v>
+        <v>6714</v>
       </c>
       <c r="B211" t="s">
         <v>204</v>
@@ -18388,7 +18388,7 @@
     </row>
     <row r="212" spans="1:18">
       <c r="A212">
-        <v>5733</v>
+        <v>6515</v>
       </c>
       <c r="B212" t="s">
         <v>205</v>
@@ -18444,7 +18444,7 @@
     </row>
     <row r="213" spans="1:18">
       <c r="A213">
-        <v>5678</v>
+        <v>6460</v>
       </c>
       <c r="B213" t="s">
         <v>206</v>
@@ -18500,7 +18500,7 @@
     </row>
     <row r="214" spans="1:18">
       <c r="A214">
-        <v>5671</v>
+        <v>6453</v>
       </c>
       <c r="B214" t="s">
         <v>207</v>
@@ -18550,7 +18550,7 @@
     </row>
     <row r="215" spans="1:18">
       <c r="A215">
-        <v>5689</v>
+        <v>6471</v>
       </c>
       <c r="B215" t="s">
         <v>208</v>
@@ -18603,7 +18603,7 @@
     </row>
     <row r="216" spans="1:18">
       <c r="A216">
-        <v>5876</v>
+        <v>6658</v>
       </c>
       <c r="B216" t="s">
         <v>209</v>
@@ -18659,7 +18659,7 @@
     </row>
     <row r="217" spans="1:18">
       <c r="A217">
-        <v>5677</v>
+        <v>6459</v>
       </c>
       <c r="B217" t="s">
         <v>210</v>
@@ -18715,7 +18715,7 @@
     </row>
     <row r="218" spans="1:18">
       <c r="A218">
-        <v>5664</v>
+        <v>6446</v>
       </c>
       <c r="B218" t="s">
         <v>211</v>
@@ -18765,7 +18765,7 @@
     </row>
     <row r="219" spans="1:18">
       <c r="A219">
-        <v>5604</v>
+        <v>6386</v>
       </c>
       <c r="B219" t="s">
         <v>212</v>
@@ -18818,7 +18818,7 @@
     </row>
     <row r="220" spans="1:18">
       <c r="A220">
-        <v>5916</v>
+        <v>6698</v>
       </c>
       <c r="B220" t="s">
         <v>213</v>
@@ -18871,7 +18871,7 @@
     </row>
     <row r="221" spans="1:18">
       <c r="A221">
-        <v>5897</v>
+        <v>6679</v>
       </c>
       <c r="B221" t="s">
         <v>214</v>
@@ -18927,7 +18927,7 @@
     </row>
     <row r="222" spans="1:18">
       <c r="A222">
-        <v>5704</v>
+        <v>6486</v>
       </c>
       <c r="B222" t="s">
         <v>215</v>
@@ -18983,7 +18983,7 @@
     </row>
     <row r="223" spans="1:18">
       <c r="A223">
-        <v>5727</v>
+        <v>6509</v>
       </c>
       <c r="B223" t="s">
         <v>216</v>
@@ -19039,7 +19039,7 @@
     </row>
     <row r="224" spans="1:18">
       <c r="A224">
-        <v>5782</v>
+        <v>6564</v>
       </c>
       <c r="B224" t="s">
         <v>217</v>
@@ -19095,7 +19095,7 @@
     </row>
     <row r="225" spans="1:18">
       <c r="A225">
-        <v>5929</v>
+        <v>6711</v>
       </c>
       <c r="B225" t="s">
         <v>218</v>
@@ -19151,7 +19151,7 @@
     </row>
     <row r="226" spans="1:18">
       <c r="A226">
-        <v>5654</v>
+        <v>6436</v>
       </c>
       <c r="B226" t="s">
         <v>219</v>
@@ -19201,7 +19201,7 @@
     </row>
     <row r="227" spans="1:18">
       <c r="A227">
-        <v>5767</v>
+        <v>6549</v>
       </c>
       <c r="B227" t="s">
         <v>220</v>
@@ -19257,7 +19257,7 @@
     </row>
     <row r="228" spans="1:18">
       <c r="A228">
-        <v>5614</v>
+        <v>6396</v>
       </c>
       <c r="B228" t="s">
         <v>221</v>
@@ -19310,7 +19310,7 @@
     </row>
     <row r="229" spans="1:18">
       <c r="A229">
-        <v>5706</v>
+        <v>6488</v>
       </c>
       <c r="B229" t="s">
         <v>222</v>
@@ -19366,7 +19366,7 @@
     </row>
     <row r="230" spans="1:18">
       <c r="A230">
-        <v>5647</v>
+        <v>6429</v>
       </c>
       <c r="B230" t="s">
         <v>223</v>
@@ -19419,7 +19419,7 @@
     </row>
     <row r="231" spans="1:18">
       <c r="A231">
-        <v>5645</v>
+        <v>6427</v>
       </c>
       <c r="B231" t="s">
         <v>224</v>
@@ -19475,7 +19475,7 @@
     </row>
     <row r="232" spans="1:18">
       <c r="A232">
-        <v>5642</v>
+        <v>6424</v>
       </c>
       <c r="B232" t="s">
         <v>225</v>
@@ -19528,7 +19528,7 @@
     </row>
     <row r="233" spans="1:18">
       <c r="A233">
-        <v>5599</v>
+        <v>6381</v>
       </c>
       <c r="B233" t="s">
         <v>226</v>
@@ -19581,7 +19581,7 @@
     </row>
     <row r="234" spans="1:18">
       <c r="A234">
-        <v>5839</v>
+        <v>6621</v>
       </c>
       <c r="B234" t="s">
         <v>227</v>
@@ -19634,7 +19634,7 @@
     </row>
     <row r="235" spans="1:18">
       <c r="A235">
-        <v>5672</v>
+        <v>6454</v>
       </c>
       <c r="B235" t="s">
         <v>228</v>
@@ -19672,7 +19672,7 @@
     </row>
     <row r="236" spans="1:18">
       <c r="A236">
-        <v>5667</v>
+        <v>6449</v>
       </c>
       <c r="B236" t="s">
         <v>229</v>
@@ -19725,7 +19725,7 @@
     </row>
     <row r="237" spans="1:18">
       <c r="A237">
-        <v>5774</v>
+        <v>6556</v>
       </c>
       <c r="B237" t="s">
         <v>230</v>
@@ -19775,7 +19775,7 @@
     </row>
     <row r="238" spans="1:18">
       <c r="A238">
-        <v>5669</v>
+        <v>6451</v>
       </c>
       <c r="B238" t="s">
         <v>231</v>
@@ -19825,7 +19825,7 @@
     </row>
     <row r="239" spans="1:18">
       <c r="A239">
-        <v>5610</v>
+        <v>6392</v>
       </c>
       <c r="B239" t="s">
         <v>232</v>
@@ -19878,7 +19878,7 @@
     </row>
     <row r="240" spans="1:18">
       <c r="A240">
-        <v>5611</v>
+        <v>6393</v>
       </c>
       <c r="B240" t="s">
         <v>232</v>
@@ -19931,7 +19931,7 @@
     </row>
     <row r="241" spans="1:18">
       <c r="A241">
-        <v>5712</v>
+        <v>6494</v>
       </c>
       <c r="B241" t="s">
         <v>233</v>
@@ -19987,7 +19987,7 @@
     </row>
     <row r="242" spans="1:18">
       <c r="A242">
-        <v>5615</v>
+        <v>6397</v>
       </c>
       <c r="B242" t="s">
         <v>234</v>
@@ -20040,7 +20040,7 @@
     </row>
     <row r="243" spans="1:18">
       <c r="A243">
-        <v>5894</v>
+        <v>6676</v>
       </c>
       <c r="B243" t="s">
         <v>235</v>
@@ -20096,7 +20096,7 @@
     </row>
     <row r="244" spans="1:18">
       <c r="A244">
-        <v>5649</v>
+        <v>6431</v>
       </c>
       <c r="B244" t="s">
         <v>236</v>
@@ -20146,7 +20146,7 @@
     </row>
     <row r="245" spans="1:18">
       <c r="A245">
-        <v>5644</v>
+        <v>6426</v>
       </c>
       <c r="B245" t="s">
         <v>237</v>
@@ -20202,7 +20202,7 @@
     </row>
     <row r="246" spans="1:18">
       <c r="A246">
-        <v>5896</v>
+        <v>6678</v>
       </c>
       <c r="B246" t="s">
         <v>238</v>
@@ -20258,7 +20258,7 @@
     </row>
     <row r="247" spans="1:18">
       <c r="A247">
-        <v>5895</v>
+        <v>6677</v>
       </c>
       <c r="B247" t="s">
         <v>239</v>
@@ -20314,7 +20314,7 @@
     </row>
     <row r="248" spans="1:18">
       <c r="A248">
-        <v>5618</v>
+        <v>6400</v>
       </c>
       <c r="B248" t="s">
         <v>240</v>
@@ -20370,7 +20370,7 @@
     </row>
     <row r="249" spans="1:18">
       <c r="A249">
-        <v>5692</v>
+        <v>6474</v>
       </c>
       <c r="B249" t="s">
         <v>241</v>
@@ -20420,7 +20420,7 @@
     </row>
     <row r="250" spans="1:18">
       <c r="A250">
-        <v>5752</v>
+        <v>6534</v>
       </c>
       <c r="B250" t="s">
         <v>242</v>
@@ -20470,7 +20470,7 @@
     </row>
     <row r="251" spans="1:18">
       <c r="A251">
-        <v>5846</v>
+        <v>6628</v>
       </c>
       <c r="B251" t="s">
         <v>243</v>
@@ -20523,7 +20523,7 @@
     </row>
     <row r="252" spans="1:18">
       <c r="A252">
-        <v>5795</v>
+        <v>6577</v>
       </c>
       <c r="B252" t="s">
         <v>244</v>
@@ -20567,7 +20567,7 @@
     </row>
     <row r="253" spans="1:18">
       <c r="A253">
-        <v>5753</v>
+        <v>6535</v>
       </c>
       <c r="B253" t="s">
         <v>245</v>
@@ -20620,7 +20620,7 @@
     </row>
     <row r="254" spans="1:18">
       <c r="A254">
-        <v>5754</v>
+        <v>6536</v>
       </c>
       <c r="B254" t="s">
         <v>245</v>
@@ -20676,7 +20676,7 @@
     </row>
     <row r="255" spans="1:18">
       <c r="A255">
-        <v>5757</v>
+        <v>6539</v>
       </c>
       <c r="B255" t="s">
         <v>246</v>
@@ -20729,7 +20729,7 @@
     </row>
     <row r="256" spans="1:18">
       <c r="A256">
-        <v>5716</v>
+        <v>6498</v>
       </c>
       <c r="B256" t="s">
         <v>247</v>
@@ -20773,7 +20773,7 @@
     </row>
     <row r="257" spans="1:18">
       <c r="A257">
-        <v>5628</v>
+        <v>6410</v>
       </c>
       <c r="B257" t="s">
         <v>248</v>
@@ -20826,7 +20826,7 @@
     </row>
     <row r="258" spans="1:18">
       <c r="A258">
-        <v>5629</v>
+        <v>6411</v>
       </c>
       <c r="B258" t="s">
         <v>248</v>
@@ -20879,7 +20879,7 @@
     </row>
     <row r="259" spans="1:18">
       <c r="A259">
-        <v>5635</v>
+        <v>6417</v>
       </c>
       <c r="B259" t="s">
         <v>249</v>
@@ -20935,7 +20935,7 @@
     </row>
     <row r="260" spans="1:18">
       <c r="A260">
-        <v>5868</v>
+        <v>6650</v>
       </c>
       <c r="B260" t="s">
         <v>250</v>
@@ -20991,7 +20991,7 @@
     </row>
     <row r="261" spans="1:18">
       <c r="A261">
-        <v>5869</v>
+        <v>6651</v>
       </c>
       <c r="B261" t="s">
         <v>250</v>
@@ -21047,7 +21047,7 @@
     </row>
     <row r="262" spans="1:18">
       <c r="A262">
-        <v>5870</v>
+        <v>6652</v>
       </c>
       <c r="B262" t="s">
         <v>250</v>
@@ -21103,7 +21103,7 @@
     </row>
     <row r="263" spans="1:18">
       <c r="A263">
-        <v>5874</v>
+        <v>6656</v>
       </c>
       <c r="B263" t="s">
         <v>251</v>
@@ -21159,7 +21159,7 @@
     </row>
     <row r="264" spans="1:18">
       <c r="A264">
-        <v>5872</v>
+        <v>6654</v>
       </c>
       <c r="B264" t="s">
         <v>252</v>
@@ -21215,7 +21215,7 @@
     </row>
     <row r="265" spans="1:18">
       <c r="A265">
-        <v>5873</v>
+        <v>6655</v>
       </c>
       <c r="B265" t="s">
         <v>252</v>
@@ -21271,7 +21271,7 @@
     </row>
     <row r="266" spans="1:18">
       <c r="A266">
-        <v>5780</v>
+        <v>6562</v>
       </c>
       <c r="B266" t="s">
         <v>253</v>
@@ -21327,7 +21327,7 @@
     </row>
     <row r="267" spans="1:18">
       <c r="A267">
-        <v>5708</v>
+        <v>6490</v>
       </c>
       <c r="B267" t="s">
         <v>254</v>
@@ -21383,7 +21383,7 @@
     </row>
     <row r="268" spans="1:18">
       <c r="A268">
-        <v>5691</v>
+        <v>6473</v>
       </c>
       <c r="B268" t="s">
         <v>255</v>
@@ -21439,7 +21439,7 @@
     </row>
     <row r="269" spans="1:18">
       <c r="A269">
-        <v>5684</v>
+        <v>6466</v>
       </c>
       <c r="B269" t="s">
         <v>256</v>
@@ -21495,7 +21495,7 @@
     </row>
     <row r="270" spans="1:18">
       <c r="A270">
-        <v>5632</v>
+        <v>6414</v>
       </c>
       <c r="B270" t="s">
         <v>257</v>
@@ -21548,7 +21548,7 @@
     </row>
     <row r="271" spans="1:18">
       <c r="A271">
-        <v>5887</v>
+        <v>6669</v>
       </c>
       <c r="B271" t="s">
         <v>258</v>
@@ -21598,7 +21598,7 @@
     </row>
     <row r="272" spans="1:18">
       <c r="A272">
-        <v>5877</v>
+        <v>6659</v>
       </c>
       <c r="B272" t="s">
         <v>259</v>
@@ -21654,7 +21654,7 @@
     </row>
     <row r="273" spans="1:18">
       <c r="A273">
-        <v>5702</v>
+        <v>6484</v>
       </c>
       <c r="B273" t="s">
         <v>260</v>
@@ -21692,7 +21692,7 @@
     </row>
     <row r="274" spans="1:18">
       <c r="A274">
-        <v>5703</v>
+        <v>6485</v>
       </c>
       <c r="B274" t="s">
         <v>260</v>
@@ -21730,7 +21730,7 @@
     </row>
     <row r="275" spans="1:18">
       <c r="A275">
-        <v>5717</v>
+        <v>6499</v>
       </c>
       <c r="B275" t="s">
         <v>261</v>
@@ -21768,7 +21768,7 @@
     </row>
     <row r="276" spans="1:18">
       <c r="A276">
-        <v>5850</v>
+        <v>6632</v>
       </c>
       <c r="B276" t="s">
         <v>262</v>
@@ -21821,7 +21821,7 @@
     </row>
     <row r="277" spans="1:18">
       <c r="A277">
-        <v>5875</v>
+        <v>6657</v>
       </c>
       <c r="B277" t="s">
         <v>263</v>
@@ -21877,7 +21877,7 @@
     </row>
     <row r="278" spans="1:18">
       <c r="A278">
-        <v>5657</v>
+        <v>6439</v>
       </c>
       <c r="B278" t="s">
         <v>264</v>
@@ -21927,7 +21927,7 @@
     </row>
     <row r="279" spans="1:18">
       <c r="A279">
-        <v>5666</v>
+        <v>6448</v>
       </c>
       <c r="B279" t="s">
         <v>265</v>
@@ -21971,7 +21971,7 @@
     </row>
     <row r="280" spans="1:18">
       <c r="A280">
-        <v>5917</v>
+        <v>6699</v>
       </c>
       <c r="B280" t="s">
         <v>266</v>
@@ -22024,7 +22024,7 @@
     </row>
     <row r="281" spans="1:18">
       <c r="A281">
-        <v>5658</v>
+        <v>6440</v>
       </c>
       <c r="B281" t="s">
         <v>267</v>
@@ -22074,7 +22074,7 @@
     </row>
     <row r="282" spans="1:18">
       <c r="A282">
-        <v>5737</v>
+        <v>6519</v>
       </c>
       <c r="B282" t="s">
         <v>268</v>
@@ -22130,7 +22130,7 @@
     </row>
     <row r="283" spans="1:18">
       <c r="A283">
-        <v>5732</v>
+        <v>6514</v>
       </c>
       <c r="B283" t="s">
         <v>269</v>
@@ -22186,7 +22186,7 @@
     </row>
     <row r="284" spans="1:18">
       <c r="A284">
-        <v>5847</v>
+        <v>6629</v>
       </c>
       <c r="B284" t="s">
         <v>270</v>
@@ -22239,7 +22239,7 @@
     </row>
     <row r="285" spans="1:18">
       <c r="A285">
-        <v>5606</v>
+        <v>6388</v>
       </c>
       <c r="B285" t="s">
         <v>271</v>
@@ -22292,7 +22292,7 @@
     </row>
     <row r="286" spans="1:18">
       <c r="A286">
-        <v>5731</v>
+        <v>6513</v>
       </c>
       <c r="B286" t="s">
         <v>272</v>
@@ -22345,7 +22345,7 @@
     </row>
     <row r="287" spans="1:18">
       <c r="A287">
-        <v>5765</v>
+        <v>6547</v>
       </c>
       <c r="B287" t="s">
         <v>273</v>
@@ -22401,7 +22401,7 @@
     </row>
     <row r="288" spans="1:18">
       <c r="A288">
-        <v>5793</v>
+        <v>6575</v>
       </c>
       <c r="B288" t="s">
         <v>274</v>
@@ -22454,7 +22454,7 @@
     </row>
     <row r="289" spans="1:18">
       <c r="A289">
-        <v>5720</v>
+        <v>6502</v>
       </c>
       <c r="B289" t="s">
         <v>275</v>
@@ -22510,7 +22510,7 @@
     </row>
     <row r="290" spans="1:18">
       <c r="A290">
-        <v>5940</v>
+        <v>6722</v>
       </c>
       <c r="B290" t="s">
         <v>276</v>
@@ -22566,7 +22566,7 @@
     </row>
     <row r="291" spans="1:18">
       <c r="A291">
-        <v>5881</v>
+        <v>6663</v>
       </c>
       <c r="B291" t="s">
         <v>277</v>
@@ -22622,7 +22622,7 @@
     </row>
     <row r="292" spans="1:18">
       <c r="A292">
-        <v>5879</v>
+        <v>6661</v>
       </c>
       <c r="B292" t="s">
         <v>278</v>
@@ -22678,7 +22678,7 @@
     </row>
     <row r="293" spans="1:18">
       <c r="A293">
-        <v>5834</v>
+        <v>6616</v>
       </c>
       <c r="B293" t="s">
         <v>279</v>
@@ -22731,7 +22731,7 @@
     </row>
     <row r="294" spans="1:18">
       <c r="A294">
-        <v>5597</v>
+        <v>6379</v>
       </c>
       <c r="B294" t="s">
         <v>280</v>
@@ -22772,7 +22772,7 @@
     </row>
     <row r="295" spans="1:18">
       <c r="A295">
-        <v>5890</v>
+        <v>6672</v>
       </c>
       <c r="B295" t="s">
         <v>281</v>
@@ -22822,7 +22822,7 @@
     </row>
     <row r="296" spans="1:18">
       <c r="A296">
-        <v>5646</v>
+        <v>6428</v>
       </c>
       <c r="B296" t="s">
         <v>282</v>
@@ -22878,7 +22878,7 @@
     </row>
     <row r="297" spans="1:18">
       <c r="A297">
-        <v>5650</v>
+        <v>6432</v>
       </c>
       <c r="B297" t="s">
         <v>283</v>
@@ -22934,7 +22934,7 @@
     </row>
     <row r="298" spans="1:18">
       <c r="A298">
-        <v>5772</v>
+        <v>6554</v>
       </c>
       <c r="B298" t="s">
         <v>284</v>
@@ -22990,7 +22990,7 @@
     </row>
     <row r="299" spans="1:18">
       <c r="A299">
-        <v>5724</v>
+        <v>6506</v>
       </c>
       <c r="B299" t="s">
         <v>285</v>
@@ -23034,7 +23034,7 @@
     </row>
     <row r="300" spans="1:18">
       <c r="A300">
-        <v>5906</v>
+        <v>6688</v>
       </c>
       <c r="B300" t="s">
         <v>286</v>
@@ -23090,7 +23090,7 @@
     </row>
     <row r="301" spans="1:18">
       <c r="A301">
-        <v>5904</v>
+        <v>6686</v>
       </c>
       <c r="B301" t="s">
         <v>287</v>
@@ -23146,7 +23146,7 @@
     </row>
     <row r="302" spans="1:18">
       <c r="A302">
-        <v>5939</v>
+        <v>6721</v>
       </c>
       <c r="B302" t="s">
         <v>288</v>
@@ -23199,7 +23199,7 @@
     </row>
     <row r="303" spans="1:18">
       <c r="A303">
-        <v>5931</v>
+        <v>6713</v>
       </c>
       <c r="B303" t="s">
         <v>289</v>
@@ -23255,7 +23255,7 @@
     </row>
     <row r="304" spans="1:18">
       <c r="A304">
-        <v>5651</v>
+        <v>6433</v>
       </c>
       <c r="B304" t="s">
         <v>290</v>
@@ -23311,7 +23311,7 @@
     </row>
     <row r="305" spans="1:18">
       <c r="A305">
-        <v>5919</v>
+        <v>6701</v>
       </c>
       <c r="B305" t="s">
         <v>291</v>
@@ -23367,7 +23367,7 @@
     </row>
     <row r="306" spans="1:18">
       <c r="A306">
-        <v>5612</v>
+        <v>6394</v>
       </c>
       <c r="B306" t="s">
         <v>292</v>
@@ -23417,7 +23417,7 @@
     </row>
     <row r="307" spans="1:18">
       <c r="A307">
-        <v>5812</v>
+        <v>6594</v>
       </c>
       <c r="B307" t="s">
         <v>293</v>
@@ -23458,7 +23458,7 @@
     </row>
     <row r="308" spans="1:18">
       <c r="A308">
-        <v>5898</v>
+        <v>6680</v>
       </c>
       <c r="B308" t="s">
         <v>294</v>
@@ -23514,7 +23514,7 @@
     </row>
     <row r="309" spans="1:18">
       <c r="A309">
-        <v>5886</v>
+        <v>6668</v>
       </c>
       <c r="B309" t="s">
         <v>295</v>
@@ -23564,7 +23564,7 @@
     </row>
     <row r="310" spans="1:18">
       <c r="A310">
-        <v>5685</v>
+        <v>6467</v>
       </c>
       <c r="B310" t="s">
         <v>296</v>
@@ -23620,7 +23620,7 @@
     </row>
     <row r="311" spans="1:18">
       <c r="A311">
-        <v>5750</v>
+        <v>6532</v>
       </c>
       <c r="B311" t="s">
         <v>297</v>
@@ -23673,7 +23673,7 @@
     </row>
     <row r="312" spans="1:18">
       <c r="A312">
-        <v>5871</v>
+        <v>6653</v>
       </c>
       <c r="B312" t="s">
         <v>298</v>
@@ -23717,7 +23717,7 @@
     </row>
     <row r="313" spans="1:18">
       <c r="A313">
-        <v>5734</v>
+        <v>6516</v>
       </c>
       <c r="B313" t="s">
         <v>299</v>
@@ -23773,7 +23773,7 @@
     </row>
     <row r="314" spans="1:18">
       <c r="A314">
-        <v>5861</v>
+        <v>6643</v>
       </c>
       <c r="B314" t="s">
         <v>300</v>
@@ -23829,7 +23829,7 @@
     </row>
     <row r="315" spans="1:18">
       <c r="A315">
-        <v>5602</v>
+        <v>6384</v>
       </c>
       <c r="B315" t="s">
         <v>301</v>
@@ -23879,7 +23879,7 @@
     </row>
     <row r="316" spans="1:18">
       <c r="A316">
-        <v>5603</v>
+        <v>6385</v>
       </c>
       <c r="B316" t="s">
         <v>301</v>
@@ -23929,7 +23929,7 @@
     </row>
     <row r="317" spans="1:18">
       <c r="A317">
-        <v>5884</v>
+        <v>6666</v>
       </c>
       <c r="B317" t="s">
         <v>302</v>
@@ -23979,7 +23979,7 @@
     </row>
     <row r="318" spans="1:18">
       <c r="A318">
-        <v>5942</v>
+        <v>6724</v>
       </c>
       <c r="B318" t="s">
         <v>303</v>
@@ -24032,7 +24032,7 @@
     </row>
     <row r="319" spans="1:18">
       <c r="A319">
-        <v>5893</v>
+        <v>6675</v>
       </c>
       <c r="B319" t="s">
         <v>304</v>
@@ -24076,7 +24076,7 @@
     </row>
     <row r="320" spans="1:18">
       <c r="A320">
-        <v>5796</v>
+        <v>6578</v>
       </c>
       <c r="B320" t="s">
         <v>305</v>
@@ -24123,7 +24123,7 @@
     </row>
     <row r="321" spans="1:18">
       <c r="A321">
-        <v>5797</v>
+        <v>6579</v>
       </c>
       <c r="B321" t="s">
         <v>305</v>
@@ -24173,7 +24173,7 @@
     </row>
     <row r="322" spans="1:18">
       <c r="A322">
-        <v>5799</v>
+        <v>6581</v>
       </c>
       <c r="B322" t="s">
         <v>306</v>
@@ -24220,7 +24220,7 @@
     </row>
     <row r="323" spans="1:18">
       <c r="A323">
-        <v>5787</v>
+        <v>6569</v>
       </c>
       <c r="B323" t="s">
         <v>307</v>
@@ -24276,7 +24276,7 @@
     </row>
     <row r="324" spans="1:18">
       <c r="A324">
-        <v>5768</v>
+        <v>6550</v>
       </c>
       <c r="B324" t="s">
         <v>308</v>
@@ -24332,7 +24332,7 @@
     </row>
     <row r="325" spans="1:18">
       <c r="A325">
-        <v>5814</v>
+        <v>6596</v>
       </c>
       <c r="B325" t="s">
         <v>309</v>
@@ -24385,7 +24385,7 @@
     </row>
     <row r="326" spans="1:18">
       <c r="A326">
-        <v>5815</v>
+        <v>6597</v>
       </c>
       <c r="B326" t="s">
         <v>309</v>
@@ -24438,7 +24438,7 @@
     </row>
     <row r="327" spans="1:18">
       <c r="A327">
-        <v>5827</v>
+        <v>6609</v>
       </c>
       <c r="B327" t="s">
         <v>310</v>
@@ -24494,7 +24494,7 @@
     </row>
     <row r="328" spans="1:18">
       <c r="A328">
-        <v>5759</v>
+        <v>6541</v>
       </c>
       <c r="B328" t="s">
         <v>311</v>
@@ -24541,7 +24541,7 @@
     </row>
     <row r="329" spans="1:18">
       <c r="A329">
-        <v>5760</v>
+        <v>6542</v>
       </c>
       <c r="B329" t="s">
         <v>311</v>
@@ -24591,7 +24591,7 @@
     </row>
     <row r="330" spans="1:18">
       <c r="A330">
-        <v>5800</v>
+        <v>6582</v>
       </c>
       <c r="B330" t="s">
         <v>312</v>
@@ -24638,7 +24638,7 @@
     </row>
     <row r="331" spans="1:18">
       <c r="A331">
-        <v>5818</v>
+        <v>6600</v>
       </c>
       <c r="B331" t="s">
         <v>313</v>
@@ -24691,7 +24691,7 @@
     </row>
     <row r="332" spans="1:18">
       <c r="A332">
-        <v>5819</v>
+        <v>6601</v>
       </c>
       <c r="B332" t="s">
         <v>313</v>
@@ -24744,7 +24744,7 @@
     </row>
     <row r="333" spans="1:18">
       <c r="A333">
-        <v>5822</v>
+        <v>6604</v>
       </c>
       <c r="B333" t="s">
         <v>314</v>
@@ -24785,7 +24785,7 @@
     </row>
     <row r="334" spans="1:18">
       <c r="A334">
-        <v>5823</v>
+        <v>6605</v>
       </c>
       <c r="B334" t="s">
         <v>314</v>
@@ -24826,7 +24826,7 @@
     </row>
     <row r="335" spans="1:18">
       <c r="A335">
-        <v>5829</v>
+        <v>6611</v>
       </c>
       <c r="B335" t="s">
         <v>315</v>
@@ -24882,7 +24882,7 @@
     </row>
     <row r="336" spans="1:18">
       <c r="A336">
-        <v>5832</v>
+        <v>6614</v>
       </c>
       <c r="B336" t="s">
         <v>316</v>
@@ -24926,7 +24926,7 @@
     </row>
     <row r="337" spans="1:18">
       <c r="A337">
-        <v>5741</v>
+        <v>6523</v>
       </c>
       <c r="B337" t="s">
         <v>317</v>
@@ -24982,7 +24982,7 @@
     </row>
     <row r="338" spans="1:18">
       <c r="A338">
-        <v>5851</v>
+        <v>6633</v>
       </c>
       <c r="B338" t="s">
         <v>318</v>
@@ -25035,7 +25035,7 @@
     </row>
     <row r="339" spans="1:18">
       <c r="A339">
-        <v>5749</v>
+        <v>6531</v>
       </c>
       <c r="B339" t="s">
         <v>319</v>
@@ -25091,7 +25091,7 @@
     </row>
     <row r="340" spans="1:18">
       <c r="A340">
-        <v>5791</v>
+        <v>6573</v>
       </c>
       <c r="B340" t="s">
         <v>320</v>
@@ -25135,7 +25135,7 @@
     </row>
     <row r="341" spans="1:18">
       <c r="A341">
-        <v>5936</v>
+        <v>6718</v>
       </c>
       <c r="B341" t="s">
         <v>321</v>
@@ -25191,7 +25191,7 @@
     </row>
     <row r="342" spans="1:18">
       <c r="A342">
-        <v>5725</v>
+        <v>6507</v>
       </c>
       <c r="B342" t="s">
         <v>322</v>
@@ -25247,7 +25247,7 @@
     </row>
     <row r="343" spans="1:18">
       <c r="A343">
-        <v>5918</v>
+        <v>6700</v>
       </c>
       <c r="B343" t="s">
         <v>323</v>
@@ -25300,7 +25300,7 @@
     </row>
     <row r="344" spans="1:18">
       <c r="A344">
-        <v>5789</v>
+        <v>6571</v>
       </c>
       <c r="B344" t="s">
         <v>324</v>
@@ -25356,7 +25356,7 @@
     </row>
     <row r="345" spans="1:18">
       <c r="A345">
-        <v>5652</v>
+        <v>6434</v>
       </c>
       <c r="B345" t="s">
         <v>325</v>
@@ -25412,7 +25412,7 @@
     </row>
     <row r="346" spans="1:18">
       <c r="A346">
-        <v>5928</v>
+        <v>6710</v>
       </c>
       <c r="B346" t="s">
         <v>326</v>
@@ -25462,7 +25462,7 @@
     </row>
     <row r="347" spans="1:18">
       <c r="A347">
-        <v>5653</v>
+        <v>6435</v>
       </c>
       <c r="B347" t="s">
         <v>327</v>
@@ -25512,7 +25512,7 @@
     </row>
     <row r="348" spans="1:18">
       <c r="A348">
-        <v>5943</v>
+        <v>6725</v>
       </c>
       <c r="B348" t="s">
         <v>328</v>
@@ -25562,7 +25562,7 @@
     </row>
     <row r="349" spans="1:18">
       <c r="A349">
-        <v>5944</v>
+        <v>6726</v>
       </c>
       <c r="B349" t="s">
         <v>329</v>
@@ -25618,7 +25618,7 @@
     </row>
     <row r="350" spans="1:18">
       <c r="A350">
-        <v>5945</v>
+        <v>6727</v>
       </c>
       <c r="B350" t="s">
         <v>330</v>
@@ -25665,7 +25665,7 @@
     </row>
     <row r="351" spans="1:18">
       <c r="A351">
-        <v>5946</v>
+        <v>6728</v>
       </c>
       <c r="B351" t="s">
         <v>331</v>
@@ -25718,7 +25718,7 @@
     </row>
     <row r="352" spans="1:18">
       <c r="A352">
-        <v>5948</v>
+        <v>6730</v>
       </c>
       <c r="B352" t="s">
         <v>332</v>
@@ -25771,7 +25771,7 @@
     </row>
     <row r="353" spans="1:18">
       <c r="A353">
-        <v>5947</v>
+        <v>6729</v>
       </c>
       <c r="B353" t="s">
         <v>333</v>
@@ -25815,7 +25815,7 @@
     </row>
     <row r="354" spans="1:18">
       <c r="A354">
-        <v>5949</v>
+        <v>6731</v>
       </c>
       <c r="B354" t="s">
         <v>334</v>
@@ -25871,7 +25871,7 @@
     </row>
     <row r="355" spans="1:18">
       <c r="A355">
-        <v>5950</v>
+        <v>6732</v>
       </c>
       <c r="B355" t="s">
         <v>335</v>
@@ -25909,7 +25909,7 @@
     </row>
     <row r="356" spans="1:18">
       <c r="A356">
-        <v>5955</v>
+        <v>6737</v>
       </c>
       <c r="B356" t="s">
         <v>336</v>
@@ -25962,7 +25962,7 @@
     </row>
     <row r="357" spans="1:18">
       <c r="A357">
-        <v>5954</v>
+        <v>6736</v>
       </c>
       <c r="B357" t="s">
         <v>337</v>
@@ -26012,7 +26012,7 @@
     </row>
     <row r="358" spans="1:18">
       <c r="A358">
-        <v>5952</v>
+        <v>6734</v>
       </c>
       <c r="B358" t="s">
         <v>338</v>
@@ -26068,7 +26068,7 @@
     </row>
     <row r="359" spans="1:18">
       <c r="A359">
-        <v>5953</v>
+        <v>6735</v>
       </c>
       <c r="B359" t="s">
         <v>339</v>
@@ -26118,7 +26118,7 @@
     </row>
     <row r="360" spans="1:18">
       <c r="A360">
-        <v>5951</v>
+        <v>6733</v>
       </c>
       <c r="B360" t="s">
         <v>340</v>
@@ -26168,7 +26168,7 @@
     </row>
     <row r="361" spans="1:18">
       <c r="A361">
-        <v>5958</v>
+        <v>6740</v>
       </c>
       <c r="B361" t="s">
         <v>341</v>
@@ -26212,7 +26212,7 @@
     </row>
     <row r="362" spans="1:18">
       <c r="A362">
-        <v>5957</v>
+        <v>6739</v>
       </c>
       <c r="B362" t="s">
         <v>342</v>
@@ -26262,7 +26262,7 @@
     </row>
     <row r="363" spans="1:18">
       <c r="A363">
-        <v>5956</v>
+        <v>6738</v>
       </c>
       <c r="B363" t="s">
         <v>343</v>
@@ -26300,7 +26300,7 @@
     </row>
     <row r="364" spans="1:18">
       <c r="A364">
-        <v>5965</v>
+        <v>6747</v>
       </c>
       <c r="B364" t="s">
         <v>344</v>
@@ -26335,7 +26335,7 @@
     </row>
     <row r="365" spans="1:18">
       <c r="A365">
-        <v>5959</v>
+        <v>6741</v>
       </c>
       <c r="B365" t="s">
         <v>345</v>
@@ -26379,7 +26379,7 @@
     </row>
     <row r="366" spans="1:18">
       <c r="A366">
-        <v>5960</v>
+        <v>6742</v>
       </c>
       <c r="B366" t="s">
         <v>346</v>
@@ -26432,7 +26432,7 @@
     </row>
     <row r="367" spans="1:18">
       <c r="A367">
-        <v>5966</v>
+        <v>6748</v>
       </c>
       <c r="B367" t="s">
         <v>347</v>
@@ -26485,7 +26485,7 @@
     </row>
     <row r="368" spans="1:18">
       <c r="A368">
-        <v>5967</v>
+        <v>6749</v>
       </c>
       <c r="B368" t="s">
         <v>348</v>
@@ -26523,7 +26523,7 @@
     </row>
     <row r="369" spans="1:18">
       <c r="A369">
-        <v>5964</v>
+        <v>6746</v>
       </c>
       <c r="B369" t="s">
         <v>349</v>
@@ -26579,7 +26579,7 @@
     </row>
     <row r="370" spans="1:18">
       <c r="A370">
-        <v>5961</v>
+        <v>6743</v>
       </c>
       <c r="B370" t="s">
         <v>350</v>
@@ -26626,7 +26626,7 @@
     </row>
     <row r="371" spans="1:18">
       <c r="A371">
-        <v>5962</v>
+        <v>6744</v>
       </c>
       <c r="B371" t="s">
         <v>255</v>
@@ -26679,7 +26679,7 @@
     </row>
     <row r="372" spans="1:18">
       <c r="A372">
-        <v>5963</v>
+        <v>6745</v>
       </c>
       <c r="B372" t="s">
         <v>351</v>
@@ -26732,7 +26732,7 @@
     </row>
     <row r="373" spans="1:18">
       <c r="A373">
-        <v>5968</v>
+        <v>6750</v>
       </c>
       <c r="B373" t="s">
         <v>352</v>
@@ -26782,7 +26782,7 @@
     </row>
     <row r="374" spans="1:18">
       <c r="A374">
-        <v>5971</v>
+        <v>6753</v>
       </c>
       <c r="B374" t="s">
         <v>353</v>
@@ -26832,7 +26832,7 @@
     </row>
     <row r="375" spans="1:18">
       <c r="A375">
-        <v>5970</v>
+        <v>6752</v>
       </c>
       <c r="B375" t="s">
         <v>354</v>
@@ -26888,7 +26888,7 @@
     </row>
     <row r="376" spans="1:18">
       <c r="A376">
-        <v>5972</v>
+        <v>6754</v>
       </c>
       <c r="B376" t="s">
         <v>355</v>
@@ -26938,7 +26938,7 @@
     </row>
     <row r="377" spans="1:18">
       <c r="A377">
-        <v>5969</v>
+        <v>6751</v>
       </c>
       <c r="B377" t="s">
         <v>356</v>
@@ -26976,7 +26976,7 @@
     </row>
     <row r="378" spans="1:18">
       <c r="A378">
-        <v>5975</v>
+        <v>6757</v>
       </c>
       <c r="B378" t="s">
         <v>357</v>
@@ -27020,7 +27020,7 @@
     </row>
     <row r="379" spans="1:18">
       <c r="A379">
-        <v>5974</v>
+        <v>6756</v>
       </c>
       <c r="B379" t="s">
         <v>244</v>
@@ -27061,7 +27061,7 @@
     </row>
     <row r="380" spans="1:18">
       <c r="A380">
-        <v>5973</v>
+        <v>6755</v>
       </c>
       <c r="B380" t="s">
         <v>358</v>
@@ -27117,7 +27117,7 @@
     </row>
     <row r="381" spans="1:18">
       <c r="A381">
-        <v>5978</v>
+        <v>6760</v>
       </c>
       <c r="B381" t="s">
         <v>359</v>
@@ -27167,7 +27167,7 @@
     </row>
     <row r="382" spans="1:18">
       <c r="A382">
-        <v>5977</v>
+        <v>6759</v>
       </c>
       <c r="B382" t="s">
         <v>360</v>
@@ -27223,7 +27223,7 @@
     </row>
     <row r="383" spans="1:18">
       <c r="A383">
-        <v>5979</v>
+        <v>6761</v>
       </c>
       <c r="B383" t="s">
         <v>361</v>
@@ -27273,7 +27273,7 @@
     </row>
     <row r="384" spans="1:18">
       <c r="A384">
-        <v>5976</v>
+        <v>6758</v>
       </c>
       <c r="B384" t="s">
         <v>333</v>
@@ -27317,7 +27317,7 @@
     </row>
     <row r="385" spans="1:18">
       <c r="A385">
-        <v>5981</v>
+        <v>6763</v>
       </c>
       <c r="B385" t="s">
         <v>346</v>
@@ -27370,7 +27370,7 @@
     </row>
     <row r="386" spans="1:18">
       <c r="A386">
-        <v>5985</v>
+        <v>6767</v>
       </c>
       <c r="B386" t="s">
         <v>362</v>
@@ -27414,7 +27414,7 @@
     </row>
     <row r="387" spans="1:18">
       <c r="A387">
-        <v>5980</v>
+        <v>6762</v>
       </c>
       <c r="B387" t="s">
         <v>363</v>
@@ -27458,7 +27458,7 @@
     </row>
     <row r="388" spans="1:18">
       <c r="A388">
-        <v>5984</v>
+        <v>6766</v>
       </c>
       <c r="B388" t="s">
         <v>364</v>
@@ -27493,7 +27493,7 @@
     </row>
     <row r="389" spans="1:18">
       <c r="A389">
-        <v>5983</v>
+        <v>6765</v>
       </c>
       <c r="B389" t="s">
         <v>357</v>
@@ -27531,7 +27531,7 @@
     </row>
     <row r="390" spans="1:18">
       <c r="A390">
-        <v>5982</v>
+        <v>6764</v>
       </c>
       <c r="B390" t="s">
         <v>365</v>
@@ -27572,7 +27572,7 @@
     </row>
     <row r="391" spans="1:18">
       <c r="A391">
-        <v>5986</v>
+        <v>6768</v>
       </c>
       <c r="B391" t="s">
         <v>366</v>
@@ -27625,7 +27625,7 @@
     </row>
     <row r="392" spans="1:18">
       <c r="A392">
-        <v>5987</v>
+        <v>6769</v>
       </c>
       <c r="B392" t="s">
         <v>367</v>

</xml_diff>

<commit_message>
Refresh generated review exports
</commit_message>
<xml_diff>
--- a/data/exports/duplicate_candidates.xlsx
+++ b/data/exports/duplicate_candidates.xlsx
@@ -7420,7 +7420,7 @@
     </row>
     <row r="2" spans="1:18">
       <c r="A2">
-        <v>6645</v>
+        <v>7036</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
@@ -7476,7 +7476,7 @@
     </row>
     <row r="3" spans="1:18">
       <c r="A3">
-        <v>6557</v>
+        <v>6948</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
@@ -7526,7 +7526,7 @@
     </row>
     <row r="4" spans="1:18">
       <c r="A4">
-        <v>6522</v>
+        <v>6913</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -7582,7 +7582,7 @@
     </row>
     <row r="5" spans="1:18">
       <c r="A5">
-        <v>6412</v>
+        <v>6803</v>
       </c>
       <c r="B5" t="s">
         <v>21</v>
@@ -7638,7 +7638,7 @@
     </row>
     <row r="6" spans="1:18">
       <c r="A6">
-        <v>6430</v>
+        <v>6821</v>
       </c>
       <c r="B6" t="s">
         <v>22</v>
@@ -7694,7 +7694,7 @@
     </row>
     <row r="7" spans="1:18">
       <c r="A7">
-        <v>6475</v>
+        <v>6866</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
@@ -7744,7 +7744,7 @@
     </row>
     <row r="8" spans="1:18">
       <c r="A8">
-        <v>6487</v>
+        <v>6878</v>
       </c>
       <c r="B8" t="s">
         <v>24</v>
@@ -7800,7 +7800,7 @@
     </row>
     <row r="9" spans="1:18">
       <c r="A9">
-        <v>6455</v>
+        <v>6846</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>
@@ -7856,7 +7856,7 @@
     </row>
     <row r="10" spans="1:18">
       <c r="A10">
-        <v>6593</v>
+        <v>6984</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
@@ -7897,7 +7897,7 @@
     </row>
     <row r="11" spans="1:18">
       <c r="A11">
-        <v>6572</v>
+        <v>6963</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
@@ -7953,7 +7953,7 @@
     </row>
     <row r="12" spans="1:18">
       <c r="A12">
-        <v>6530</v>
+        <v>6921</v>
       </c>
       <c r="B12" t="s">
         <v>28</v>
@@ -8009,7 +8009,7 @@
     </row>
     <row r="13" spans="1:18">
       <c r="A13">
-        <v>6635</v>
+        <v>7026</v>
       </c>
       <c r="B13" t="s">
         <v>29</v>
@@ -8062,7 +8062,7 @@
     </row>
     <row r="14" spans="1:18">
       <c r="A14">
-        <v>6636</v>
+        <v>7027</v>
       </c>
       <c r="B14" t="s">
         <v>29</v>
@@ -8115,7 +8115,7 @@
     </row>
     <row r="15" spans="1:18">
       <c r="A15">
-        <v>6637</v>
+        <v>7028</v>
       </c>
       <c r="B15" t="s">
         <v>29</v>
@@ -8168,7 +8168,7 @@
     </row>
     <row r="16" spans="1:18">
       <c r="A16">
-        <v>6638</v>
+        <v>7029</v>
       </c>
       <c r="B16" t="s">
         <v>30</v>
@@ -8218,7 +8218,7 @@
     </row>
     <row r="17" spans="1:18">
       <c r="A17">
-        <v>6639</v>
+        <v>7030</v>
       </c>
       <c r="B17" t="s">
         <v>30</v>
@@ -8268,7 +8268,7 @@
     </row>
     <row r="18" spans="1:18">
       <c r="A18">
-        <v>6640</v>
+        <v>7031</v>
       </c>
       <c r="B18" t="s">
         <v>31</v>
@@ -8318,7 +8318,7 @@
     </row>
     <row r="19" spans="1:18">
       <c r="A19">
-        <v>6520</v>
+        <v>6911</v>
       </c>
       <c r="B19" t="s">
         <v>32</v>
@@ -8374,7 +8374,7 @@
     </row>
     <row r="20" spans="1:18">
       <c r="A20">
-        <v>6559</v>
+        <v>6950</v>
       </c>
       <c r="B20" t="s">
         <v>33</v>
@@ -8424,7 +8424,7 @@
     </row>
     <row r="21" spans="1:18">
       <c r="A21">
-        <v>6685</v>
+        <v>7076</v>
       </c>
       <c r="B21" t="s">
         <v>34</v>
@@ -8480,7 +8480,7 @@
     </row>
     <row r="22" spans="1:18">
       <c r="A22">
-        <v>6602</v>
+        <v>6993</v>
       </c>
       <c r="B22" t="s">
         <v>35</v>
@@ -8533,7 +8533,7 @@
     </row>
     <row r="23" spans="1:18">
       <c r="A23">
-        <v>6603</v>
+        <v>6994</v>
       </c>
       <c r="B23" t="s">
         <v>35</v>
@@ -8586,7 +8586,7 @@
     </row>
     <row r="24" spans="1:18">
       <c r="A24">
-        <v>6612</v>
+        <v>7003</v>
       </c>
       <c r="B24" t="s">
         <v>36</v>
@@ -8642,7 +8642,7 @@
     </row>
     <row r="25" spans="1:18">
       <c r="A25">
-        <v>6586</v>
+        <v>6977</v>
       </c>
       <c r="B25" t="s">
         <v>37</v>
@@ -8695,7 +8695,7 @@
     </row>
     <row r="26" spans="1:18">
       <c r="A26">
-        <v>6587</v>
+        <v>6978</v>
       </c>
       <c r="B26" t="s">
         <v>37</v>
@@ -8751,7 +8751,7 @@
     </row>
     <row r="27" spans="1:18">
       <c r="A27">
-        <v>6589</v>
+        <v>6980</v>
       </c>
       <c r="B27" t="s">
         <v>38</v>
@@ -8804,7 +8804,7 @@
     </row>
     <row r="28" spans="1:18">
       <c r="A28">
-        <v>6476</v>
+        <v>6867</v>
       </c>
       <c r="B28" t="s">
         <v>39</v>
@@ -8860,7 +8860,7 @@
     </row>
     <row r="29" spans="1:18">
       <c r="A29">
-        <v>6584</v>
+        <v>6975</v>
       </c>
       <c r="B29" t="s">
         <v>40</v>
@@ -8901,7 +8901,7 @@
     </row>
     <row r="30" spans="1:18">
       <c r="A30">
-        <v>6585</v>
+        <v>6976</v>
       </c>
       <c r="B30" t="s">
         <v>40</v>
@@ -8945,7 +8945,7 @@
     </row>
     <row r="31" spans="1:18">
       <c r="A31">
-        <v>6588</v>
+        <v>6979</v>
       </c>
       <c r="B31" t="s">
         <v>41</v>
@@ -8986,7 +8986,7 @@
     </row>
     <row r="32" spans="1:18">
       <c r="A32">
-        <v>6689</v>
+        <v>7080</v>
       </c>
       <c r="B32" t="s">
         <v>42</v>
@@ -9042,7 +9042,7 @@
     </row>
     <row r="33" spans="1:18">
       <c r="A33">
-        <v>6510</v>
+        <v>6901</v>
       </c>
       <c r="B33" t="s">
         <v>43</v>
@@ -9098,7 +9098,7 @@
     </row>
     <row r="34" spans="1:18">
       <c r="A34">
-        <v>6511</v>
+        <v>6902</v>
       </c>
       <c r="B34" t="s">
         <v>44</v>
@@ -9139,7 +9139,7 @@
     </row>
     <row r="35" spans="1:18">
       <c r="A35">
-        <v>6551</v>
+        <v>6942</v>
       </c>
       <c r="B35" t="s">
         <v>45</v>
@@ -9195,7 +9195,7 @@
     </row>
     <row r="36" spans="1:18">
       <c r="A36">
-        <v>6537</v>
+        <v>6928</v>
       </c>
       <c r="B36" t="s">
         <v>46</v>
@@ -9248,7 +9248,7 @@
     </row>
     <row r="37" spans="1:18">
       <c r="A37">
-        <v>6538</v>
+        <v>6929</v>
       </c>
       <c r="B37" t="s">
         <v>46</v>
@@ -9304,7 +9304,7 @@
     </row>
     <row r="38" spans="1:18">
       <c r="A38">
-        <v>6540</v>
+        <v>6931</v>
       </c>
       <c r="B38" t="s">
         <v>47</v>
@@ -9357,7 +9357,7 @@
     </row>
     <row r="39" spans="1:18">
       <c r="A39">
-        <v>6543</v>
+        <v>6934</v>
       </c>
       <c r="B39" t="s">
         <v>48</v>
@@ -9404,7 +9404,7 @@
     </row>
     <row r="40" spans="1:18">
       <c r="A40">
-        <v>6544</v>
+        <v>6935</v>
       </c>
       <c r="B40" t="s">
         <v>48</v>
@@ -9454,7 +9454,7 @@
     </row>
     <row r="41" spans="1:18">
       <c r="A41">
-        <v>6583</v>
+        <v>6974</v>
       </c>
       <c r="B41" t="s">
         <v>49</v>
@@ -9501,7 +9501,7 @@
     </row>
     <row r="42" spans="1:18">
       <c r="A42">
-        <v>6598</v>
+        <v>6989</v>
       </c>
       <c r="B42" t="s">
         <v>50</v>
@@ -9554,7 +9554,7 @@
     </row>
     <row r="43" spans="1:18">
       <c r="A43">
-        <v>6599</v>
+        <v>6990</v>
       </c>
       <c r="B43" t="s">
         <v>50</v>
@@ -9607,7 +9607,7 @@
     </row>
     <row r="44" spans="1:18">
       <c r="A44">
-        <v>6610</v>
+        <v>7001</v>
       </c>
       <c r="B44" t="s">
         <v>51</v>
@@ -9663,7 +9663,7 @@
     </row>
     <row r="45" spans="1:18">
       <c r="A45">
-        <v>6443</v>
+        <v>6834</v>
       </c>
       <c r="B45" t="s">
         <v>52</v>
@@ -9713,7 +9713,7 @@
     </row>
     <row r="46" spans="1:18">
       <c r="A46">
-        <v>6708</v>
+        <v>7099</v>
       </c>
       <c r="B46" t="s">
         <v>53</v>
@@ -9769,7 +9769,7 @@
     </row>
     <row r="47" spans="1:18">
       <c r="A47">
-        <v>6423</v>
+        <v>6814</v>
       </c>
       <c r="B47" t="s">
         <v>54</v>
@@ -9822,7 +9822,7 @@
     </row>
     <row r="48" spans="1:18">
       <c r="A48">
-        <v>6574</v>
+        <v>6965</v>
       </c>
       <c r="B48" t="s">
         <v>55</v>
@@ -9875,7 +9875,7 @@
     </row>
     <row r="49" spans="1:18">
       <c r="A49">
-        <v>6608</v>
+        <v>6999</v>
       </c>
       <c r="B49" t="s">
         <v>56</v>
@@ -9931,7 +9931,7 @@
     </row>
     <row r="50" spans="1:18">
       <c r="A50">
-        <v>6422</v>
+        <v>6813</v>
       </c>
       <c r="B50" t="s">
         <v>57</v>
@@ -9978,7 +9978,7 @@
     </row>
     <row r="51" spans="1:18">
       <c r="A51">
-        <v>6673</v>
+        <v>7064</v>
       </c>
       <c r="B51" t="s">
         <v>58</v>
@@ -10028,7 +10028,7 @@
     </row>
     <row r="52" spans="1:18">
       <c r="A52">
-        <v>6521</v>
+        <v>6912</v>
       </c>
       <c r="B52" t="s">
         <v>59</v>
@@ -10084,7 +10084,7 @@
     </row>
     <row r="53" spans="1:18">
       <c r="A53">
-        <v>6622</v>
+        <v>7013</v>
       </c>
       <c r="B53" t="s">
         <v>60</v>
@@ -10137,7 +10137,7 @@
     </row>
     <row r="54" spans="1:18">
       <c r="A54">
-        <v>6627</v>
+        <v>7018</v>
       </c>
       <c r="B54" t="s">
         <v>61</v>
@@ -10190,7 +10190,7 @@
     </row>
     <row r="55" spans="1:18">
       <c r="A55">
-        <v>6702</v>
+        <v>7093</v>
       </c>
       <c r="B55" t="s">
         <v>62</v>
@@ -10243,7 +10243,7 @@
     </row>
     <row r="56" spans="1:18">
       <c r="A56">
-        <v>6425</v>
+        <v>6816</v>
       </c>
       <c r="B56" t="s">
         <v>63</v>
@@ -10287,7 +10287,7 @@
     </row>
     <row r="57" spans="1:18">
       <c r="A57">
-        <v>6533</v>
+        <v>6924</v>
       </c>
       <c r="B57" t="s">
         <v>64</v>
@@ -10343,7 +10343,7 @@
     </row>
     <row r="58" spans="1:18">
       <c r="A58">
-        <v>6625</v>
+        <v>7016</v>
       </c>
       <c r="B58" t="s">
         <v>65</v>
@@ -10396,7 +10396,7 @@
     </row>
     <row r="59" spans="1:18">
       <c r="A59">
-        <v>6457</v>
+        <v>6848</v>
       </c>
       <c r="B59" t="s">
         <v>66</v>
@@ -10449,7 +10449,7 @@
     </row>
     <row r="60" spans="1:18">
       <c r="A60">
-        <v>6380</v>
+        <v>6771</v>
       </c>
       <c r="B60" t="s">
         <v>67</v>
@@ -10502,7 +10502,7 @@
     </row>
     <row r="61" spans="1:18">
       <c r="A61">
-        <v>6646</v>
+        <v>7037</v>
       </c>
       <c r="B61" t="s">
         <v>68</v>
@@ -10555,7 +10555,7 @@
     </row>
     <row r="62" spans="1:18">
       <c r="A62">
-        <v>6634</v>
+        <v>7025</v>
       </c>
       <c r="B62" t="s">
         <v>69</v>
@@ -10608,7 +10608,7 @@
     </row>
     <row r="63" spans="1:18">
       <c r="A63">
-        <v>6548</v>
+        <v>6939</v>
       </c>
       <c r="B63" t="s">
         <v>70</v>
@@ -10664,7 +10664,7 @@
     </row>
     <row r="64" spans="1:18">
       <c r="A64">
-        <v>6512</v>
+        <v>6903</v>
       </c>
       <c r="B64" t="s">
         <v>71</v>
@@ -10717,7 +10717,7 @@
     </row>
     <row r="65" spans="1:18">
       <c r="A65">
-        <v>6500</v>
+        <v>6891</v>
       </c>
       <c r="B65" t="s">
         <v>72</v>
@@ -10764,7 +10764,7 @@
     </row>
     <row r="66" spans="1:18">
       <c r="A66">
-        <v>6524</v>
+        <v>6915</v>
       </c>
       <c r="B66" t="s">
         <v>73</v>
@@ -10820,7 +10820,7 @@
     </row>
     <row r="67" spans="1:18">
       <c r="A67">
-        <v>6464</v>
+        <v>6855</v>
       </c>
       <c r="B67" t="s">
         <v>74</v>
@@ -10870,7 +10870,7 @@
     </row>
     <row r="68" spans="1:18">
       <c r="A68">
-        <v>6720</v>
+        <v>7111</v>
       </c>
       <c r="B68" t="s">
         <v>75</v>
@@ -10920,7 +10920,7 @@
     </row>
     <row r="69" spans="1:18">
       <c r="A69">
-        <v>6518</v>
+        <v>6909</v>
       </c>
       <c r="B69" t="s">
         <v>76</v>
@@ -10976,7 +10976,7 @@
     </row>
     <row r="70" spans="1:18">
       <c r="A70">
-        <v>6715</v>
+        <v>7106</v>
       </c>
       <c r="B70" t="s">
         <v>77</v>
@@ -11032,7 +11032,7 @@
     </row>
     <row r="71" spans="1:18">
       <c r="A71">
-        <v>6545</v>
+        <v>6936</v>
       </c>
       <c r="B71" t="s">
         <v>78</v>
@@ -11079,7 +11079,7 @@
     </row>
     <row r="72" spans="1:18">
       <c r="A72">
-        <v>6546</v>
+        <v>6937</v>
       </c>
       <c r="B72" t="s">
         <v>78</v>
@@ -11129,7 +11129,7 @@
     </row>
     <row r="73" spans="1:18">
       <c r="A73">
-        <v>6595</v>
+        <v>6986</v>
       </c>
       <c r="B73" t="s">
         <v>79</v>
@@ -11176,7 +11176,7 @@
     </row>
     <row r="74" spans="1:18">
       <c r="A74">
-        <v>6642</v>
+        <v>7033</v>
       </c>
       <c r="B74" t="s">
         <v>80</v>
@@ -11220,7 +11220,7 @@
     </row>
     <row r="75" spans="1:18">
       <c r="A75">
-        <v>6709</v>
+        <v>7100</v>
       </c>
       <c r="B75" t="s">
         <v>81</v>
@@ -11273,7 +11273,7 @@
     </row>
     <row r="76" spans="1:18">
       <c r="A76">
-        <v>6568</v>
+        <v>6959</v>
       </c>
       <c r="B76" t="s">
         <v>82</v>
@@ -11329,7 +11329,7 @@
     </row>
     <row r="77" spans="1:18">
       <c r="A77">
-        <v>6382</v>
+        <v>6773</v>
       </c>
       <c r="B77" t="s">
         <v>83</v>
@@ -11382,7 +11382,7 @@
     </row>
     <row r="78" spans="1:18">
       <c r="A78">
-        <v>6606</v>
+        <v>6997</v>
       </c>
       <c r="B78" t="s">
         <v>84</v>
@@ -11435,7 +11435,7 @@
     </row>
     <row r="79" spans="1:18">
       <c r="A79">
-        <v>6607</v>
+        <v>6998</v>
       </c>
       <c r="B79" t="s">
         <v>84</v>
@@ -11488,7 +11488,7 @@
     </row>
     <row r="80" spans="1:18">
       <c r="A80">
-        <v>6615</v>
+        <v>7006</v>
       </c>
       <c r="B80" t="s">
         <v>85</v>
@@ -11544,7 +11544,7 @@
     </row>
     <row r="81" spans="1:18">
       <c r="A81">
-        <v>6570</v>
+        <v>6961</v>
       </c>
       <c r="B81" t="s">
         <v>86</v>
@@ -11600,7 +11600,7 @@
     </row>
     <row r="82" spans="1:18">
       <c r="A82">
-        <v>6555</v>
+        <v>6946</v>
       </c>
       <c r="B82" t="s">
         <v>87</v>
@@ -11656,7 +11656,7 @@
     </row>
     <row r="83" spans="1:18">
       <c r="A83">
-        <v>6479</v>
+        <v>6870</v>
       </c>
       <c r="B83" t="s">
         <v>88</v>
@@ -11712,7 +11712,7 @@
     </row>
     <row r="84" spans="1:18">
       <c r="A84">
-        <v>6480</v>
+        <v>6871</v>
       </c>
       <c r="B84" t="s">
         <v>88</v>
@@ -11768,7 +11768,7 @@
     </row>
     <row r="85" spans="1:18">
       <c r="A85">
-        <v>6497</v>
+        <v>6888</v>
       </c>
       <c r="B85" t="s">
         <v>89</v>
@@ -11824,7 +11824,7 @@
     </row>
     <row r="86" spans="1:18">
       <c r="A86">
-        <v>6683</v>
+        <v>7074</v>
       </c>
       <c r="B86" t="s">
         <v>90</v>
@@ -11880,7 +11880,7 @@
     </row>
     <row r="87" spans="1:18">
       <c r="A87">
-        <v>6491</v>
+        <v>6882</v>
       </c>
       <c r="B87" t="s">
         <v>91</v>
@@ -11936,7 +11936,7 @@
     </row>
     <row r="88" spans="1:18">
       <c r="A88">
-        <v>6644</v>
+        <v>7035</v>
       </c>
       <c r="B88" t="s">
         <v>92</v>
@@ -11992,7 +11992,7 @@
     </row>
     <row r="89" spans="1:18">
       <c r="A89">
-        <v>6405</v>
+        <v>6796</v>
       </c>
       <c r="B89" t="s">
         <v>93</v>
@@ -12048,7 +12048,7 @@
     </row>
     <row r="90" spans="1:18">
       <c r="A90">
-        <v>6406</v>
+        <v>6797</v>
       </c>
       <c r="B90" t="s">
         <v>93</v>
@@ -12104,7 +12104,7 @@
     </row>
     <row r="91" spans="1:18">
       <c r="A91">
-        <v>6413</v>
+        <v>6804</v>
       </c>
       <c r="B91" t="s">
         <v>94</v>
@@ -12157,7 +12157,7 @@
     </row>
     <row r="92" spans="1:18">
       <c r="A92">
-        <v>6553</v>
+        <v>6944</v>
       </c>
       <c r="B92" t="s">
         <v>95</v>
@@ -12210,7 +12210,7 @@
     </row>
     <row r="93" spans="1:18">
       <c r="A93">
-        <v>6401</v>
+        <v>6792</v>
       </c>
       <c r="B93" t="s">
         <v>96</v>
@@ -12254,7 +12254,7 @@
     </row>
     <row r="94" spans="1:18">
       <c r="A94">
-        <v>6649</v>
+        <v>7040</v>
       </c>
       <c r="B94" t="s">
         <v>97</v>
@@ -12310,7 +12310,7 @@
     </row>
     <row r="95" spans="1:18">
       <c r="A95">
-        <v>6461</v>
+        <v>6852</v>
       </c>
       <c r="B95" t="s">
         <v>98</v>
@@ -12363,7 +12363,7 @@
     </row>
     <row r="96" spans="1:18">
       <c r="A96">
-        <v>6630</v>
+        <v>7021</v>
       </c>
       <c r="B96" t="s">
         <v>99</v>
@@ -12416,7 +12416,7 @@
     </row>
     <row r="97" spans="1:18">
       <c r="A97">
-        <v>6705</v>
+        <v>7096</v>
       </c>
       <c r="B97" t="s">
         <v>100</v>
@@ -12469,7 +12469,7 @@
     </row>
     <row r="98" spans="1:18">
       <c r="A98">
-        <v>6465</v>
+        <v>6856</v>
       </c>
       <c r="B98" t="s">
         <v>101</v>
@@ -12525,7 +12525,7 @@
     </row>
     <row r="99" spans="1:18">
       <c r="A99">
-        <v>6420</v>
+        <v>6811</v>
       </c>
       <c r="B99" t="s">
         <v>102</v>
@@ -12569,7 +12569,7 @@
     </row>
     <row r="100" spans="1:18">
       <c r="A100">
-        <v>6421</v>
+        <v>6812</v>
       </c>
       <c r="B100" t="s">
         <v>102</v>
@@ -12613,7 +12613,7 @@
     </row>
     <row r="101" spans="1:18">
       <c r="A101">
-        <v>6483</v>
+        <v>6874</v>
       </c>
       <c r="B101" t="s">
         <v>103</v>
@@ -12657,7 +12657,7 @@
     </row>
     <row r="102" spans="1:18">
       <c r="A102">
-        <v>6716</v>
+        <v>7107</v>
       </c>
       <c r="B102" t="s">
         <v>104</v>
@@ -12698,7 +12698,7 @@
     </row>
     <row r="103" spans="1:18">
       <c r="A103">
-        <v>6591</v>
+        <v>6982</v>
       </c>
       <c r="B103" t="s">
         <v>105</v>
@@ -12739,7 +12739,7 @@
     </row>
     <row r="104" spans="1:18">
       <c r="A104">
-        <v>6438</v>
+        <v>6829</v>
       </c>
       <c r="B104" t="s">
         <v>106</v>
@@ -12789,7 +12789,7 @@
     </row>
     <row r="105" spans="1:18">
       <c r="A105">
-        <v>6391</v>
+        <v>6782</v>
       </c>
       <c r="B105" t="s">
         <v>107</v>
@@ -12842,7 +12842,7 @@
     </row>
     <row r="106" spans="1:18">
       <c r="A106">
-        <v>6695</v>
+        <v>7086</v>
       </c>
       <c r="B106" t="s">
         <v>108</v>
@@ -12892,7 +12892,7 @@
     </row>
     <row r="107" spans="1:18">
       <c r="A107">
-        <v>6619</v>
+        <v>7010</v>
       </c>
       <c r="B107" t="s">
         <v>109</v>
@@ -12945,7 +12945,7 @@
     </row>
     <row r="108" spans="1:18">
       <c r="A108">
-        <v>6671</v>
+        <v>7062</v>
       </c>
       <c r="B108" t="s">
         <v>110</v>
@@ -12992,7 +12992,7 @@
     </row>
     <row r="109" spans="1:18">
       <c r="A109">
-        <v>6623</v>
+        <v>7014</v>
       </c>
       <c r="B109" t="s">
         <v>111</v>
@@ -13045,7 +13045,7 @@
     </row>
     <row r="110" spans="1:18">
       <c r="A110">
-        <v>6641</v>
+        <v>7032</v>
       </c>
       <c r="B110" t="s">
         <v>112</v>
@@ -13083,7 +13083,7 @@
     </row>
     <row r="111" spans="1:18">
       <c r="A111">
-        <v>6504</v>
+        <v>6895</v>
       </c>
       <c r="B111" t="s">
         <v>113</v>
@@ -13139,7 +13139,7 @@
     </row>
     <row r="112" spans="1:18">
       <c r="A112">
-        <v>6418</v>
+        <v>6809</v>
       </c>
       <c r="B112" t="s">
         <v>114</v>
@@ -13189,7 +13189,7 @@
     </row>
     <row r="113" spans="1:18">
       <c r="A113">
-        <v>6419</v>
+        <v>6810</v>
       </c>
       <c r="B113" t="s">
         <v>114</v>
@@ -13239,7 +13239,7 @@
     </row>
     <row r="114" spans="1:18">
       <c r="A114">
-        <v>6482</v>
+        <v>6873</v>
       </c>
       <c r="B114" t="s">
         <v>115</v>
@@ -13289,7 +13289,7 @@
     </row>
     <row r="115" spans="1:18">
       <c r="A115">
-        <v>6408</v>
+        <v>6799</v>
       </c>
       <c r="B115" t="s">
         <v>116</v>
@@ -13333,7 +13333,7 @@
     </row>
     <row r="116" spans="1:18">
       <c r="A116">
-        <v>6409</v>
+        <v>6800</v>
       </c>
       <c r="B116" t="s">
         <v>116</v>
@@ -13377,7 +13377,7 @@
     </row>
     <row r="117" spans="1:18">
       <c r="A117">
-        <v>6481</v>
+        <v>6872</v>
       </c>
       <c r="B117" t="s">
         <v>117</v>
@@ -13421,7 +13421,7 @@
     </row>
     <row r="118" spans="1:18">
       <c r="A118">
-        <v>6667</v>
+        <v>7058</v>
       </c>
       <c r="B118" t="s">
         <v>118</v>
@@ -13471,7 +13471,7 @@
     </row>
     <row r="119" spans="1:18">
       <c r="A119">
-        <v>6445</v>
+        <v>6836</v>
       </c>
       <c r="B119" t="s">
         <v>119</v>
@@ -13521,7 +13521,7 @@
     </row>
     <row r="120" spans="1:18">
       <c r="A120">
-        <v>6456</v>
+        <v>6847</v>
       </c>
       <c r="B120" t="s">
         <v>120</v>
@@ -13577,7 +13577,7 @@
     </row>
     <row r="121" spans="1:18">
       <c r="A121">
-        <v>6469</v>
+        <v>6860</v>
       </c>
       <c r="B121" t="s">
         <v>121</v>
@@ -13615,7 +13615,7 @@
     </row>
     <row r="122" spans="1:18">
       <c r="A122">
-        <v>6560</v>
+        <v>6951</v>
       </c>
       <c r="B122" t="s">
         <v>122</v>
@@ -13671,7 +13671,7 @@
     </row>
     <row r="123" spans="1:18">
       <c r="A123">
-        <v>6563</v>
+        <v>6954</v>
       </c>
       <c r="B123" t="s">
         <v>123</v>
@@ -13727,7 +13727,7 @@
     </row>
     <row r="124" spans="1:18">
       <c r="A124">
-        <v>6617</v>
+        <v>7008</v>
       </c>
       <c r="B124" t="s">
         <v>124</v>
@@ -13780,7 +13780,7 @@
     </row>
     <row r="125" spans="1:18">
       <c r="A125">
-        <v>6670</v>
+        <v>7061</v>
       </c>
       <c r="B125" t="s">
         <v>125</v>
@@ -13830,7 +13830,7 @@
     </row>
     <row r="126" spans="1:18">
       <c r="A126">
-        <v>6618</v>
+        <v>7009</v>
       </c>
       <c r="B126" t="s">
         <v>126</v>
@@ -13883,7 +13883,7 @@
     </row>
     <row r="127" spans="1:18">
       <c r="A127">
-        <v>6395</v>
+        <v>6786</v>
       </c>
       <c r="B127" t="s">
         <v>127</v>
@@ -13936,7 +13936,7 @@
     </row>
     <row r="128" spans="1:18">
       <c r="A128">
-        <v>6444</v>
+        <v>6835</v>
       </c>
       <c r="B128" t="s">
         <v>128</v>
@@ -13980,7 +13980,7 @@
     </row>
     <row r="129" spans="1:18">
       <c r="A129">
-        <v>6682</v>
+        <v>7073</v>
       </c>
       <c r="B129" t="s">
         <v>129</v>
@@ -14036,7 +14036,7 @@
     </row>
     <row r="130" spans="1:18">
       <c r="A130">
-        <v>6517</v>
+        <v>6908</v>
       </c>
       <c r="B130" t="s">
         <v>130</v>
@@ -14092,7 +14092,7 @@
     </row>
     <row r="131" spans="1:18">
       <c r="A131">
-        <v>6525</v>
+        <v>6916</v>
       </c>
       <c r="B131" t="s">
         <v>131</v>
@@ -14148,7 +14148,7 @@
     </row>
     <row r="132" spans="1:18">
       <c r="A132">
-        <v>6503</v>
+        <v>6894</v>
       </c>
       <c r="B132" t="s">
         <v>132</v>
@@ -14204,7 +14204,7 @@
     </row>
     <row r="133" spans="1:18">
       <c r="A133">
-        <v>6631</v>
+        <v>7022</v>
       </c>
       <c r="B133" t="s">
         <v>133</v>
@@ -14257,7 +14257,7 @@
     </row>
     <row r="134" spans="1:18">
       <c r="A134">
-        <v>6501</v>
+        <v>6892</v>
       </c>
       <c r="B134" t="s">
         <v>134</v>
@@ -14313,7 +14313,7 @@
     </row>
     <row r="135" spans="1:18">
       <c r="A135">
-        <v>6662</v>
+        <v>7053</v>
       </c>
       <c r="B135" t="s">
         <v>135</v>
@@ -14369,7 +14369,7 @@
     </row>
     <row r="136" spans="1:18">
       <c r="A136">
-        <v>6447</v>
+        <v>6838</v>
       </c>
       <c r="B136" t="s">
         <v>136</v>
@@ -14413,7 +14413,7 @@
     </row>
     <row r="137" spans="1:18">
       <c r="A137">
-        <v>6674</v>
+        <v>7065</v>
       </c>
       <c r="B137" t="s">
         <v>137</v>
@@ -14463,7 +14463,7 @@
     </row>
     <row r="138" spans="1:18">
       <c r="A138">
-        <v>6442</v>
+        <v>6833</v>
       </c>
       <c r="B138" t="s">
         <v>138</v>
@@ -14513,7 +14513,7 @@
     </row>
     <row r="139" spans="1:18">
       <c r="A139">
-        <v>6462</v>
+        <v>6853</v>
       </c>
       <c r="B139" t="s">
         <v>139</v>
@@ -14569,7 +14569,7 @@
     </row>
     <row r="140" spans="1:18">
       <c r="A140">
-        <v>6552</v>
+        <v>6943</v>
       </c>
       <c r="B140" t="s">
         <v>140</v>
@@ -14625,7 +14625,7 @@
     </row>
     <row r="141" spans="1:18">
       <c r="A141">
-        <v>6441</v>
+        <v>6832</v>
       </c>
       <c r="B141" t="s">
         <v>141</v>
@@ -14663,7 +14663,7 @@
     </row>
     <row r="142" spans="1:18">
       <c r="A142">
-        <v>6707</v>
+        <v>7098</v>
       </c>
       <c r="B142" t="s">
         <v>142</v>
@@ -14716,7 +14716,7 @@
     </row>
     <row r="143" spans="1:18">
       <c r="A143">
-        <v>6468</v>
+        <v>6859</v>
       </c>
       <c r="B143" t="s">
         <v>143</v>
@@ -14769,7 +14769,7 @@
     </row>
     <row r="144" spans="1:18">
       <c r="A144">
-        <v>6398</v>
+        <v>6789</v>
       </c>
       <c r="B144" t="s">
         <v>144</v>
@@ -14822,7 +14822,7 @@
     </row>
     <row r="145" spans="1:18">
       <c r="A145">
-        <v>6565</v>
+        <v>6956</v>
       </c>
       <c r="B145" t="s">
         <v>145</v>
@@ -14878,7 +14878,7 @@
     </row>
     <row r="146" spans="1:18">
       <c r="A146">
-        <v>6566</v>
+        <v>6957</v>
       </c>
       <c r="B146" t="s">
         <v>145</v>
@@ -14934,7 +14934,7 @@
     </row>
     <row r="147" spans="1:18">
       <c r="A147">
-        <v>6567</v>
+        <v>6958</v>
       </c>
       <c r="B147" t="s">
         <v>146</v>
@@ -14990,7 +14990,7 @@
     </row>
     <row r="148" spans="1:18">
       <c r="A148">
-        <v>6692</v>
+        <v>7083</v>
       </c>
       <c r="B148" t="s">
         <v>147</v>
@@ -15046,7 +15046,7 @@
     </row>
     <row r="149" spans="1:18">
       <c r="A149">
-        <v>6664</v>
+        <v>7055</v>
       </c>
       <c r="B149" t="s">
         <v>148</v>
@@ -15102,7 +15102,7 @@
     </row>
     <row r="150" spans="1:18">
       <c r="A150">
-        <v>6580</v>
+        <v>6971</v>
       </c>
       <c r="B150" t="s">
         <v>149</v>
@@ -15155,7 +15155,7 @@
     </row>
     <row r="151" spans="1:18">
       <c r="A151">
-        <v>6495</v>
+        <v>6886</v>
       </c>
       <c r="B151" t="s">
         <v>150</v>
@@ -15211,7 +15211,7 @@
     </row>
     <row r="152" spans="1:18">
       <c r="A152">
-        <v>6493</v>
+        <v>6884</v>
       </c>
       <c r="B152" t="s">
         <v>151</v>
@@ -15267,7 +15267,7 @@
     </row>
     <row r="153" spans="1:18">
       <c r="A153">
-        <v>6626</v>
+        <v>7017</v>
       </c>
       <c r="B153" t="s">
         <v>152</v>
@@ -15320,7 +15320,7 @@
     </row>
     <row r="154" spans="1:18">
       <c r="A154">
-        <v>6472</v>
+        <v>6863</v>
       </c>
       <c r="B154" t="s">
         <v>153</v>
@@ -15376,7 +15376,7 @@
     </row>
     <row r="155" spans="1:18">
       <c r="A155">
-        <v>6684</v>
+        <v>7075</v>
       </c>
       <c r="B155" t="s">
         <v>154</v>
@@ -15432,7 +15432,7 @@
     </row>
     <row r="156" spans="1:18">
       <c r="A156">
-        <v>6558</v>
+        <v>6949</v>
       </c>
       <c r="B156" t="s">
         <v>155</v>
@@ -15482,7 +15482,7 @@
     </row>
     <row r="157" spans="1:18">
       <c r="A157">
-        <v>6492</v>
+        <v>6883</v>
       </c>
       <c r="B157" t="s">
         <v>156</v>
@@ -15538,7 +15538,7 @@
     </row>
     <row r="158" spans="1:18">
       <c r="A158">
-        <v>6592</v>
+        <v>6983</v>
       </c>
       <c r="B158" t="s">
         <v>157</v>
@@ -15579,7 +15579,7 @@
     </row>
     <row r="159" spans="1:18">
       <c r="A159">
-        <v>6613</v>
+        <v>7004</v>
       </c>
       <c r="B159" t="s">
         <v>158</v>
@@ -15629,7 +15629,7 @@
     </row>
     <row r="160" spans="1:18">
       <c r="A160">
-        <v>6723</v>
+        <v>7114</v>
       </c>
       <c r="B160" t="s">
         <v>159</v>
@@ -15685,7 +15685,7 @@
     </row>
     <row r="161" spans="1:18">
       <c r="A161">
-        <v>6407</v>
+        <v>6798</v>
       </c>
       <c r="B161" t="s">
         <v>160</v>
@@ -15741,7 +15741,7 @@
     </row>
     <row r="162" spans="1:18">
       <c r="A162">
-        <v>6590</v>
+        <v>6981</v>
       </c>
       <c r="B162" t="s">
         <v>161</v>
@@ -15794,7 +15794,7 @@
     </row>
     <row r="163" spans="1:18">
       <c r="A163">
-        <v>6624</v>
+        <v>7015</v>
       </c>
       <c r="B163" t="s">
         <v>162</v>
@@ -15847,7 +15847,7 @@
     </row>
     <row r="164" spans="1:18">
       <c r="A164">
-        <v>6437</v>
+        <v>6828</v>
       </c>
       <c r="B164" t="s">
         <v>163</v>
@@ -15885,7 +15885,7 @@
     </row>
     <row r="165" spans="1:18">
       <c r="A165">
-        <v>6681</v>
+        <v>7072</v>
       </c>
       <c r="B165" t="s">
         <v>164</v>
@@ -15941,7 +15941,7 @@
     </row>
     <row r="166" spans="1:18">
       <c r="A166">
-        <v>6463</v>
+        <v>6854</v>
       </c>
       <c r="B166" t="s">
         <v>165</v>
@@ -15997,7 +15997,7 @@
     </row>
     <row r="167" spans="1:18">
       <c r="A167">
-        <v>6470</v>
+        <v>6861</v>
       </c>
       <c r="B167" t="s">
         <v>166</v>
@@ -16050,7 +16050,7 @@
     </row>
     <row r="168" spans="1:18">
       <c r="A168">
-        <v>6458</v>
+        <v>6849</v>
       </c>
       <c r="B168" t="s">
         <v>167</v>
@@ -16103,7 +16103,7 @@
     </row>
     <row r="169" spans="1:18">
       <c r="A169">
-        <v>6505</v>
+        <v>6896</v>
       </c>
       <c r="B169" t="s">
         <v>168</v>
@@ -16147,7 +16147,7 @@
     </row>
     <row r="170" spans="1:18">
       <c r="A170">
-        <v>6399</v>
+        <v>6790</v>
       </c>
       <c r="B170" t="s">
         <v>169</v>
@@ -16203,7 +16203,7 @@
     </row>
     <row r="171" spans="1:18">
       <c r="A171">
-        <v>6687</v>
+        <v>7078</v>
       </c>
       <c r="B171" t="s">
         <v>170</v>
@@ -16259,7 +16259,7 @@
     </row>
     <row r="172" spans="1:18">
       <c r="A172">
-        <v>6576</v>
+        <v>6967</v>
       </c>
       <c r="B172" t="s">
         <v>171</v>
@@ -16312,7 +16312,7 @@
     </row>
     <row r="173" spans="1:18">
       <c r="A173">
-        <v>6694</v>
+        <v>7085</v>
       </c>
       <c r="B173" t="s">
         <v>172</v>
@@ -16368,7 +16368,7 @@
     </row>
     <row r="174" spans="1:18">
       <c r="A174">
-        <v>6697</v>
+        <v>7088</v>
       </c>
       <c r="B174" t="s">
         <v>173</v>
@@ -16421,7 +16421,7 @@
     </row>
     <row r="175" spans="1:18">
       <c r="A175">
-        <v>6529</v>
+        <v>6920</v>
       </c>
       <c r="B175" t="s">
         <v>174</v>
@@ -16471,7 +16471,7 @@
     </row>
     <row r="176" spans="1:18">
       <c r="A176">
-        <v>6508</v>
+        <v>6899</v>
       </c>
       <c r="B176" t="s">
         <v>175</v>
@@ -16527,7 +16527,7 @@
     </row>
     <row r="177" spans="1:18">
       <c r="A177">
-        <v>6690</v>
+        <v>7081</v>
       </c>
       <c r="B177" t="s">
         <v>176</v>
@@ -16571,7 +16571,7 @@
     </row>
     <row r="178" spans="1:18">
       <c r="A178">
-        <v>6620</v>
+        <v>7011</v>
       </c>
       <c r="B178" t="s">
         <v>177</v>
@@ -16627,7 +16627,7 @@
     </row>
     <row r="179" spans="1:18">
       <c r="A179">
-        <v>6691</v>
+        <v>7082</v>
       </c>
       <c r="B179" t="s">
         <v>178</v>
@@ -16683,7 +16683,7 @@
     </row>
     <row r="180" spans="1:18">
       <c r="A180">
-        <v>6489</v>
+        <v>6880</v>
       </c>
       <c r="B180" t="s">
         <v>179</v>
@@ -16739,7 +16739,7 @@
     </row>
     <row r="181" spans="1:18">
       <c r="A181">
-        <v>6390</v>
+        <v>6781</v>
       </c>
       <c r="B181" t="s">
         <v>180</v>
@@ -16789,7 +16789,7 @@
     </row>
     <row r="182" spans="1:18">
       <c r="A182">
-        <v>6387</v>
+        <v>6778</v>
       </c>
       <c r="B182" t="s">
         <v>181</v>
@@ -16842,7 +16842,7 @@
     </row>
     <row r="183" spans="1:18">
       <c r="A183">
-        <v>6383</v>
+        <v>6774</v>
       </c>
       <c r="B183" t="s">
         <v>182</v>
@@ -16892,7 +16892,7 @@
     </row>
     <row r="184" spans="1:18">
       <c r="A184">
-        <v>6452</v>
+        <v>6843</v>
       </c>
       <c r="B184" t="s">
         <v>183</v>
@@ -16942,7 +16942,7 @@
     </row>
     <row r="185" spans="1:18">
       <c r="A185">
-        <v>6712</v>
+        <v>7103</v>
       </c>
       <c r="B185" t="s">
         <v>184</v>
@@ -16998,7 +16998,7 @@
     </row>
     <row r="186" spans="1:18">
       <c r="A186">
-        <v>6526</v>
+        <v>6917</v>
       </c>
       <c r="B186" t="s">
         <v>185</v>
@@ -17054,7 +17054,7 @@
     </row>
     <row r="187" spans="1:18">
       <c r="A187">
-        <v>6527</v>
+        <v>6918</v>
       </c>
       <c r="B187" t="s">
         <v>186</v>
@@ -17110,7 +17110,7 @@
     </row>
     <row r="188" spans="1:18">
       <c r="A188">
-        <v>6717</v>
+        <v>7108</v>
       </c>
       <c r="B188" t="s">
         <v>187</v>
@@ -17166,7 +17166,7 @@
     </row>
     <row r="189" spans="1:18">
       <c r="A189">
-        <v>6415</v>
+        <v>6806</v>
       </c>
       <c r="B189" t="s">
         <v>188</v>
@@ -17219,7 +17219,7 @@
     </row>
     <row r="190" spans="1:18">
       <c r="A190">
-        <v>6416</v>
+        <v>6807</v>
       </c>
       <c r="B190" t="s">
         <v>188</v>
@@ -17272,7 +17272,7 @@
     </row>
     <row r="191" spans="1:18">
       <c r="A191">
-        <v>6665</v>
+        <v>7056</v>
       </c>
       <c r="B191" t="s">
         <v>189</v>
@@ -17328,7 +17328,7 @@
     </row>
     <row r="192" spans="1:18">
       <c r="A192">
-        <v>6660</v>
+        <v>7051</v>
       </c>
       <c r="B192" t="s">
         <v>190</v>
@@ -17384,7 +17384,7 @@
     </row>
     <row r="193" spans="1:18">
       <c r="A193">
-        <v>6528</v>
+        <v>6919</v>
       </c>
       <c r="B193" t="s">
         <v>191</v>
@@ -17440,7 +17440,7 @@
     </row>
     <row r="194" spans="1:18">
       <c r="A194">
-        <v>6647</v>
+        <v>7038</v>
       </c>
       <c r="B194" t="s">
         <v>192</v>
@@ -17493,7 +17493,7 @@
     </row>
     <row r="195" spans="1:18">
       <c r="A195">
-        <v>6648</v>
+        <v>7039</v>
       </c>
       <c r="B195" t="s">
         <v>192</v>
@@ -17546,7 +17546,7 @@
     </row>
     <row r="196" spans="1:18">
       <c r="A196">
-        <v>6693</v>
+        <v>7084</v>
       </c>
       <c r="B196" t="s">
         <v>193</v>
@@ -17596,7 +17596,7 @@
     </row>
     <row r="197" spans="1:18">
       <c r="A197">
-        <v>6561</v>
+        <v>6952</v>
       </c>
       <c r="B197" t="s">
         <v>194</v>
@@ -17652,7 +17652,7 @@
     </row>
     <row r="198" spans="1:18">
       <c r="A198">
-        <v>6719</v>
+        <v>7110</v>
       </c>
       <c r="B198" t="s">
         <v>195</v>
@@ -17708,7 +17708,7 @@
     </row>
     <row r="199" spans="1:18">
       <c r="A199">
-        <v>6696</v>
+        <v>7087</v>
       </c>
       <c r="B199" t="s">
         <v>196</v>
@@ -17761,7 +17761,7 @@
     </row>
     <row r="200" spans="1:18">
       <c r="A200">
-        <v>6402</v>
+        <v>6793</v>
       </c>
       <c r="B200" t="s">
         <v>197</v>
@@ -17817,7 +17817,7 @@
     </row>
     <row r="201" spans="1:18">
       <c r="A201">
-        <v>6403</v>
+        <v>6794</v>
       </c>
       <c r="B201" t="s">
         <v>197</v>
@@ -17873,7 +17873,7 @@
     </row>
     <row r="202" spans="1:18">
       <c r="A202">
-        <v>6404</v>
+        <v>6795</v>
       </c>
       <c r="B202" t="s">
         <v>197</v>
@@ -17929,7 +17929,7 @@
     </row>
     <row r="203" spans="1:18">
       <c r="A203">
-        <v>6477</v>
+        <v>6868</v>
       </c>
       <c r="B203" t="s">
         <v>198</v>
@@ -17985,7 +17985,7 @@
     </row>
     <row r="204" spans="1:18">
       <c r="A204">
-        <v>6478</v>
+        <v>6869</v>
       </c>
       <c r="B204" t="s">
         <v>198</v>
@@ -18041,7 +18041,7 @@
     </row>
     <row r="205" spans="1:18">
       <c r="A205">
-        <v>6496</v>
+        <v>6887</v>
       </c>
       <c r="B205" t="s">
         <v>199</v>
@@ -18097,7 +18097,7 @@
     </row>
     <row r="206" spans="1:18">
       <c r="A206">
-        <v>6389</v>
+        <v>6780</v>
       </c>
       <c r="B206" t="s">
         <v>200</v>
@@ -18144,7 +18144,7 @@
     </row>
     <row r="207" spans="1:18">
       <c r="A207">
-        <v>6703</v>
+        <v>7094</v>
       </c>
       <c r="B207" t="s">
         <v>201</v>
@@ -18200,7 +18200,7 @@
     </row>
     <row r="208" spans="1:18">
       <c r="A208">
-        <v>6704</v>
+        <v>7095</v>
       </c>
       <c r="B208" t="s">
         <v>201</v>
@@ -18256,7 +18256,7 @@
     </row>
     <row r="209" spans="1:18">
       <c r="A209">
-        <v>6706</v>
+        <v>7097</v>
       </c>
       <c r="B209" t="s">
         <v>202</v>
@@ -18312,7 +18312,7 @@
     </row>
     <row r="210" spans="1:18">
       <c r="A210">
-        <v>6450</v>
+        <v>6841</v>
       </c>
       <c r="B210" t="s">
         <v>203</v>
@@ -18362,7 +18362,7 @@
     </row>
     <row r="211" spans="1:18">
       <c r="A211">
-        <v>6714</v>
+        <v>7105</v>
       </c>
       <c r="B211" t="s">
         <v>204</v>
@@ -18388,7 +18388,7 @@
     </row>
     <row r="212" spans="1:18">
       <c r="A212">
-        <v>6515</v>
+        <v>6906</v>
       </c>
       <c r="B212" t="s">
         <v>205</v>
@@ -18444,7 +18444,7 @@
     </row>
     <row r="213" spans="1:18">
       <c r="A213">
-        <v>6460</v>
+        <v>6851</v>
       </c>
       <c r="B213" t="s">
         <v>206</v>
@@ -18500,7 +18500,7 @@
     </row>
     <row r="214" spans="1:18">
       <c r="A214">
-        <v>6453</v>
+        <v>6844</v>
       </c>
       <c r="B214" t="s">
         <v>207</v>
@@ -18550,7 +18550,7 @@
     </row>
     <row r="215" spans="1:18">
       <c r="A215">
-        <v>6471</v>
+        <v>6862</v>
       </c>
       <c r="B215" t="s">
         <v>208</v>
@@ -18603,7 +18603,7 @@
     </row>
     <row r="216" spans="1:18">
       <c r="A216">
-        <v>6658</v>
+        <v>7049</v>
       </c>
       <c r="B216" t="s">
         <v>209</v>
@@ -18659,7 +18659,7 @@
     </row>
     <row r="217" spans="1:18">
       <c r="A217">
-        <v>6459</v>
+        <v>6850</v>
       </c>
       <c r="B217" t="s">
         <v>210</v>
@@ -18715,7 +18715,7 @@
     </row>
     <row r="218" spans="1:18">
       <c r="A218">
-        <v>6446</v>
+        <v>6837</v>
       </c>
       <c r="B218" t="s">
         <v>211</v>
@@ -18765,7 +18765,7 @@
     </row>
     <row r="219" spans="1:18">
       <c r="A219">
-        <v>6386</v>
+        <v>6777</v>
       </c>
       <c r="B219" t="s">
         <v>212</v>
@@ -18818,7 +18818,7 @@
     </row>
     <row r="220" spans="1:18">
       <c r="A220">
-        <v>6698</v>
+        <v>7089</v>
       </c>
       <c r="B220" t="s">
         <v>213</v>
@@ -18871,7 +18871,7 @@
     </row>
     <row r="221" spans="1:18">
       <c r="A221">
-        <v>6679</v>
+        <v>7070</v>
       </c>
       <c r="B221" t="s">
         <v>214</v>
@@ -18927,7 +18927,7 @@
     </row>
     <row r="222" spans="1:18">
       <c r="A222">
-        <v>6486</v>
+        <v>6877</v>
       </c>
       <c r="B222" t="s">
         <v>215</v>
@@ -18983,7 +18983,7 @@
     </row>
     <row r="223" spans="1:18">
       <c r="A223">
-        <v>6509</v>
+        <v>6900</v>
       </c>
       <c r="B223" t="s">
         <v>216</v>
@@ -19039,7 +19039,7 @@
     </row>
     <row r="224" spans="1:18">
       <c r="A224">
-        <v>6564</v>
+        <v>6955</v>
       </c>
       <c r="B224" t="s">
         <v>217</v>
@@ -19095,7 +19095,7 @@
     </row>
     <row r="225" spans="1:18">
       <c r="A225">
-        <v>6711</v>
+        <v>7102</v>
       </c>
       <c r="B225" t="s">
         <v>218</v>
@@ -19151,7 +19151,7 @@
     </row>
     <row r="226" spans="1:18">
       <c r="A226">
-        <v>6436</v>
+        <v>6827</v>
       </c>
       <c r="B226" t="s">
         <v>219</v>
@@ -19201,7 +19201,7 @@
     </row>
     <row r="227" spans="1:18">
       <c r="A227">
-        <v>6549</v>
+        <v>6940</v>
       </c>
       <c r="B227" t="s">
         <v>220</v>
@@ -19257,7 +19257,7 @@
     </row>
     <row r="228" spans="1:18">
       <c r="A228">
-        <v>6396</v>
+        <v>6787</v>
       </c>
       <c r="B228" t="s">
         <v>221</v>
@@ -19310,7 +19310,7 @@
     </row>
     <row r="229" spans="1:18">
       <c r="A229">
-        <v>6488</v>
+        <v>6879</v>
       </c>
       <c r="B229" t="s">
         <v>222</v>
@@ -19366,7 +19366,7 @@
     </row>
     <row r="230" spans="1:18">
       <c r="A230">
-        <v>6429</v>
+        <v>6820</v>
       </c>
       <c r="B230" t="s">
         <v>223</v>
@@ -19419,7 +19419,7 @@
     </row>
     <row r="231" spans="1:18">
       <c r="A231">
-        <v>6427</v>
+        <v>6818</v>
       </c>
       <c r="B231" t="s">
         <v>224</v>
@@ -19475,7 +19475,7 @@
     </row>
     <row r="232" spans="1:18">
       <c r="A232">
-        <v>6424</v>
+        <v>6815</v>
       </c>
       <c r="B232" t="s">
         <v>225</v>
@@ -19528,7 +19528,7 @@
     </row>
     <row r="233" spans="1:18">
       <c r="A233">
-        <v>6381</v>
+        <v>6772</v>
       </c>
       <c r="B233" t="s">
         <v>226</v>
@@ -19581,7 +19581,7 @@
     </row>
     <row r="234" spans="1:18">
       <c r="A234">
-        <v>6621</v>
+        <v>7012</v>
       </c>
       <c r="B234" t="s">
         <v>227</v>
@@ -19634,7 +19634,7 @@
     </row>
     <row r="235" spans="1:18">
       <c r="A235">
-        <v>6454</v>
+        <v>6845</v>
       </c>
       <c r="B235" t="s">
         <v>228</v>
@@ -19672,7 +19672,7 @@
     </row>
     <row r="236" spans="1:18">
       <c r="A236">
-        <v>6449</v>
+        <v>6840</v>
       </c>
       <c r="B236" t="s">
         <v>229</v>
@@ -19725,7 +19725,7 @@
     </row>
     <row r="237" spans="1:18">
       <c r="A237">
-        <v>6556</v>
+        <v>6947</v>
       </c>
       <c r="B237" t="s">
         <v>230</v>
@@ -19775,7 +19775,7 @@
     </row>
     <row r="238" spans="1:18">
       <c r="A238">
-        <v>6451</v>
+        <v>6842</v>
       </c>
       <c r="B238" t="s">
         <v>231</v>
@@ -19825,7 +19825,7 @@
     </row>
     <row r="239" spans="1:18">
       <c r="A239">
-        <v>6392</v>
+        <v>6783</v>
       </c>
       <c r="B239" t="s">
         <v>232</v>
@@ -19878,7 +19878,7 @@
     </row>
     <row r="240" spans="1:18">
       <c r="A240">
-        <v>6393</v>
+        <v>6784</v>
       </c>
       <c r="B240" t="s">
         <v>232</v>
@@ -19931,7 +19931,7 @@
     </row>
     <row r="241" spans="1:18">
       <c r="A241">
-        <v>6494</v>
+        <v>6885</v>
       </c>
       <c r="B241" t="s">
         <v>233</v>
@@ -19987,7 +19987,7 @@
     </row>
     <row r="242" spans="1:18">
       <c r="A242">
-        <v>6397</v>
+        <v>6788</v>
       </c>
       <c r="B242" t="s">
         <v>234</v>
@@ -20040,7 +20040,7 @@
     </row>
     <row r="243" spans="1:18">
       <c r="A243">
-        <v>6676</v>
+        <v>7067</v>
       </c>
       <c r="B243" t="s">
         <v>235</v>
@@ -20096,7 +20096,7 @@
     </row>
     <row r="244" spans="1:18">
       <c r="A244">
-        <v>6431</v>
+        <v>6822</v>
       </c>
       <c r="B244" t="s">
         <v>236</v>
@@ -20146,7 +20146,7 @@
     </row>
     <row r="245" spans="1:18">
       <c r="A245">
-        <v>6426</v>
+        <v>6817</v>
       </c>
       <c r="B245" t="s">
         <v>237</v>
@@ -20202,7 +20202,7 @@
     </row>
     <row r="246" spans="1:18">
       <c r="A246">
-        <v>6678</v>
+        <v>7069</v>
       </c>
       <c r="B246" t="s">
         <v>238</v>
@@ -20258,7 +20258,7 @@
     </row>
     <row r="247" spans="1:18">
       <c r="A247">
-        <v>6677</v>
+        <v>7068</v>
       </c>
       <c r="B247" t="s">
         <v>239</v>
@@ -20314,7 +20314,7 @@
     </row>
     <row r="248" spans="1:18">
       <c r="A248">
-        <v>6400</v>
+        <v>6791</v>
       </c>
       <c r="B248" t="s">
         <v>240</v>
@@ -20370,7 +20370,7 @@
     </row>
     <row r="249" spans="1:18">
       <c r="A249">
-        <v>6474</v>
+        <v>6865</v>
       </c>
       <c r="B249" t="s">
         <v>241</v>
@@ -20420,7 +20420,7 @@
     </row>
     <row r="250" spans="1:18">
       <c r="A250">
-        <v>6534</v>
+        <v>6925</v>
       </c>
       <c r="B250" t="s">
         <v>242</v>
@@ -20470,7 +20470,7 @@
     </row>
     <row r="251" spans="1:18">
       <c r="A251">
-        <v>6628</v>
+        <v>7019</v>
       </c>
       <c r="B251" t="s">
         <v>243</v>
@@ -20523,7 +20523,7 @@
     </row>
     <row r="252" spans="1:18">
       <c r="A252">
-        <v>6577</v>
+        <v>6968</v>
       </c>
       <c r="B252" t="s">
         <v>244</v>
@@ -20567,7 +20567,7 @@
     </row>
     <row r="253" spans="1:18">
       <c r="A253">
-        <v>6535</v>
+        <v>6926</v>
       </c>
       <c r="B253" t="s">
         <v>245</v>
@@ -20620,7 +20620,7 @@
     </row>
     <row r="254" spans="1:18">
       <c r="A254">
-        <v>6536</v>
+        <v>6927</v>
       </c>
       <c r="B254" t="s">
         <v>245</v>
@@ -20676,7 +20676,7 @@
     </row>
     <row r="255" spans="1:18">
       <c r="A255">
-        <v>6539</v>
+        <v>6930</v>
       </c>
       <c r="B255" t="s">
         <v>246</v>
@@ -20729,7 +20729,7 @@
     </row>
     <row r="256" spans="1:18">
       <c r="A256">
-        <v>6498</v>
+        <v>6889</v>
       </c>
       <c r="B256" t="s">
         <v>247</v>
@@ -20773,7 +20773,7 @@
     </row>
     <row r="257" spans="1:18">
       <c r="A257">
-        <v>6410</v>
+        <v>6801</v>
       </c>
       <c r="B257" t="s">
         <v>248</v>
@@ -20826,7 +20826,7 @@
     </row>
     <row r="258" spans="1:18">
       <c r="A258">
-        <v>6411</v>
+        <v>6802</v>
       </c>
       <c r="B258" t="s">
         <v>248</v>
@@ -20879,7 +20879,7 @@
     </row>
     <row r="259" spans="1:18">
       <c r="A259">
-        <v>6417</v>
+        <v>6808</v>
       </c>
       <c r="B259" t="s">
         <v>249</v>
@@ -20935,7 +20935,7 @@
     </row>
     <row r="260" spans="1:18">
       <c r="A260">
-        <v>6650</v>
+        <v>7041</v>
       </c>
       <c r="B260" t="s">
         <v>250</v>
@@ -20991,7 +20991,7 @@
     </row>
     <row r="261" spans="1:18">
       <c r="A261">
-        <v>6651</v>
+        <v>7042</v>
       </c>
       <c r="B261" t="s">
         <v>250</v>
@@ -21047,7 +21047,7 @@
     </row>
     <row r="262" spans="1:18">
       <c r="A262">
-        <v>6652</v>
+        <v>7043</v>
       </c>
       <c r="B262" t="s">
         <v>250</v>
@@ -21103,7 +21103,7 @@
     </row>
     <row r="263" spans="1:18">
       <c r="A263">
-        <v>6656</v>
+        <v>7047</v>
       </c>
       <c r="B263" t="s">
         <v>251</v>
@@ -21159,7 +21159,7 @@
     </row>
     <row r="264" spans="1:18">
       <c r="A264">
-        <v>6654</v>
+        <v>7045</v>
       </c>
       <c r="B264" t="s">
         <v>252</v>
@@ -21215,7 +21215,7 @@
     </row>
     <row r="265" spans="1:18">
       <c r="A265">
-        <v>6655</v>
+        <v>7046</v>
       </c>
       <c r="B265" t="s">
         <v>252</v>
@@ -21271,7 +21271,7 @@
     </row>
     <row r="266" spans="1:18">
       <c r="A266">
-        <v>6562</v>
+        <v>6953</v>
       </c>
       <c r="B266" t="s">
         <v>253</v>
@@ -21327,7 +21327,7 @@
     </row>
     <row r="267" spans="1:18">
       <c r="A267">
-        <v>6490</v>
+        <v>6881</v>
       </c>
       <c r="B267" t="s">
         <v>254</v>
@@ -21383,7 +21383,7 @@
     </row>
     <row r="268" spans="1:18">
       <c r="A268">
-        <v>6473</v>
+        <v>6864</v>
       </c>
       <c r="B268" t="s">
         <v>255</v>
@@ -21439,7 +21439,7 @@
     </row>
     <row r="269" spans="1:18">
       <c r="A269">
-        <v>6466</v>
+        <v>6857</v>
       </c>
       <c r="B269" t="s">
         <v>256</v>
@@ -21495,7 +21495,7 @@
     </row>
     <row r="270" spans="1:18">
       <c r="A270">
-        <v>6414</v>
+        <v>6805</v>
       </c>
       <c r="B270" t="s">
         <v>257</v>
@@ -21548,7 +21548,7 @@
     </row>
     <row r="271" spans="1:18">
       <c r="A271">
-        <v>6669</v>
+        <v>7060</v>
       </c>
       <c r="B271" t="s">
         <v>258</v>
@@ -21598,7 +21598,7 @@
     </row>
     <row r="272" spans="1:18">
       <c r="A272">
-        <v>6659</v>
+        <v>7050</v>
       </c>
       <c r="B272" t="s">
         <v>259</v>
@@ -21654,7 +21654,7 @@
     </row>
     <row r="273" spans="1:18">
       <c r="A273">
-        <v>6484</v>
+        <v>6875</v>
       </c>
       <c r="B273" t="s">
         <v>260</v>
@@ -21692,7 +21692,7 @@
     </row>
     <row r="274" spans="1:18">
       <c r="A274">
-        <v>6485</v>
+        <v>6876</v>
       </c>
       <c r="B274" t="s">
         <v>260</v>
@@ -21730,7 +21730,7 @@
     </row>
     <row r="275" spans="1:18">
       <c r="A275">
-        <v>6499</v>
+        <v>6890</v>
       </c>
       <c r="B275" t="s">
         <v>261</v>
@@ -21768,7 +21768,7 @@
     </row>
     <row r="276" spans="1:18">
       <c r="A276">
-        <v>6632</v>
+        <v>7023</v>
       </c>
       <c r="B276" t="s">
         <v>262</v>
@@ -21821,7 +21821,7 @@
     </row>
     <row r="277" spans="1:18">
       <c r="A277">
-        <v>6657</v>
+        <v>7048</v>
       </c>
       <c r="B277" t="s">
         <v>263</v>
@@ -21877,7 +21877,7 @@
     </row>
     <row r="278" spans="1:18">
       <c r="A278">
-        <v>6439</v>
+        <v>6830</v>
       </c>
       <c r="B278" t="s">
         <v>264</v>
@@ -21927,7 +21927,7 @@
     </row>
     <row r="279" spans="1:18">
       <c r="A279">
-        <v>6448</v>
+        <v>6839</v>
       </c>
       <c r="B279" t="s">
         <v>265</v>
@@ -21971,7 +21971,7 @@
     </row>
     <row r="280" spans="1:18">
       <c r="A280">
-        <v>6699</v>
+        <v>7090</v>
       </c>
       <c r="B280" t="s">
         <v>266</v>
@@ -22024,7 +22024,7 @@
     </row>
     <row r="281" spans="1:18">
       <c r="A281">
-        <v>6440</v>
+        <v>6831</v>
       </c>
       <c r="B281" t="s">
         <v>267</v>
@@ -22074,7 +22074,7 @@
     </row>
     <row r="282" spans="1:18">
       <c r="A282">
-        <v>6519</v>
+        <v>6910</v>
       </c>
       <c r="B282" t="s">
         <v>268</v>
@@ -22130,7 +22130,7 @@
     </row>
     <row r="283" spans="1:18">
       <c r="A283">
-        <v>6514</v>
+        <v>6905</v>
       </c>
       <c r="B283" t="s">
         <v>269</v>
@@ -22186,7 +22186,7 @@
     </row>
     <row r="284" spans="1:18">
       <c r="A284">
-        <v>6629</v>
+        <v>7020</v>
       </c>
       <c r="B284" t="s">
         <v>270</v>
@@ -22239,7 +22239,7 @@
     </row>
     <row r="285" spans="1:18">
       <c r="A285">
-        <v>6388</v>
+        <v>6779</v>
       </c>
       <c r="B285" t="s">
         <v>271</v>
@@ -22292,7 +22292,7 @@
     </row>
     <row r="286" spans="1:18">
       <c r="A286">
-        <v>6513</v>
+        <v>6904</v>
       </c>
       <c r="B286" t="s">
         <v>272</v>
@@ -22345,7 +22345,7 @@
     </row>
     <row r="287" spans="1:18">
       <c r="A287">
-        <v>6547</v>
+        <v>6938</v>
       </c>
       <c r="B287" t="s">
         <v>273</v>
@@ -22401,7 +22401,7 @@
     </row>
     <row r="288" spans="1:18">
       <c r="A288">
-        <v>6575</v>
+        <v>6966</v>
       </c>
       <c r="B288" t="s">
         <v>274</v>
@@ -22454,7 +22454,7 @@
     </row>
     <row r="289" spans="1:18">
       <c r="A289">
-        <v>6502</v>
+        <v>6893</v>
       </c>
       <c r="B289" t="s">
         <v>275</v>
@@ -22510,7 +22510,7 @@
     </row>
     <row r="290" spans="1:18">
       <c r="A290">
-        <v>6722</v>
+        <v>7113</v>
       </c>
       <c r="B290" t="s">
         <v>276</v>
@@ -22566,7 +22566,7 @@
     </row>
     <row r="291" spans="1:18">
       <c r="A291">
-        <v>6663</v>
+        <v>7054</v>
       </c>
       <c r="B291" t="s">
         <v>277</v>
@@ -22622,7 +22622,7 @@
     </row>
     <row r="292" spans="1:18">
       <c r="A292">
-        <v>6661</v>
+        <v>7052</v>
       </c>
       <c r="B292" t="s">
         <v>278</v>
@@ -22678,7 +22678,7 @@
     </row>
     <row r="293" spans="1:18">
       <c r="A293">
-        <v>6616</v>
+        <v>7007</v>
       </c>
       <c r="B293" t="s">
         <v>279</v>
@@ -22731,7 +22731,7 @@
     </row>
     <row r="294" spans="1:18">
       <c r="A294">
-        <v>6379</v>
+        <v>6770</v>
       </c>
       <c r="B294" t="s">
         <v>280</v>
@@ -22772,7 +22772,7 @@
     </row>
     <row r="295" spans="1:18">
       <c r="A295">
-        <v>6672</v>
+        <v>7063</v>
       </c>
       <c r="B295" t="s">
         <v>281</v>
@@ -22822,7 +22822,7 @@
     </row>
     <row r="296" spans="1:18">
       <c r="A296">
-        <v>6428</v>
+        <v>6819</v>
       </c>
       <c r="B296" t="s">
         <v>282</v>
@@ -22878,7 +22878,7 @@
     </row>
     <row r="297" spans="1:18">
       <c r="A297">
-        <v>6432</v>
+        <v>6823</v>
       </c>
       <c r="B297" t="s">
         <v>283</v>
@@ -22934,7 +22934,7 @@
     </row>
     <row r="298" spans="1:18">
       <c r="A298">
-        <v>6554</v>
+        <v>6945</v>
       </c>
       <c r="B298" t="s">
         <v>284</v>
@@ -22990,7 +22990,7 @@
     </row>
     <row r="299" spans="1:18">
       <c r="A299">
-        <v>6506</v>
+        <v>6897</v>
       </c>
       <c r="B299" t="s">
         <v>285</v>
@@ -23034,7 +23034,7 @@
     </row>
     <row r="300" spans="1:18">
       <c r="A300">
-        <v>6688</v>
+        <v>7079</v>
       </c>
       <c r="B300" t="s">
         <v>286</v>
@@ -23090,7 +23090,7 @@
     </row>
     <row r="301" spans="1:18">
       <c r="A301">
-        <v>6686</v>
+        <v>7077</v>
       </c>
       <c r="B301" t="s">
         <v>287</v>
@@ -23146,7 +23146,7 @@
     </row>
     <row r="302" spans="1:18">
       <c r="A302">
-        <v>6721</v>
+        <v>7112</v>
       </c>
       <c r="B302" t="s">
         <v>288</v>
@@ -23199,7 +23199,7 @@
     </row>
     <row r="303" spans="1:18">
       <c r="A303">
-        <v>6713</v>
+        <v>7104</v>
       </c>
       <c r="B303" t="s">
         <v>289</v>
@@ -23255,7 +23255,7 @@
     </row>
     <row r="304" spans="1:18">
       <c r="A304">
-        <v>6433</v>
+        <v>6824</v>
       </c>
       <c r="B304" t="s">
         <v>290</v>
@@ -23311,7 +23311,7 @@
     </row>
     <row r="305" spans="1:18">
       <c r="A305">
-        <v>6701</v>
+        <v>7092</v>
       </c>
       <c r="B305" t="s">
         <v>291</v>
@@ -23367,7 +23367,7 @@
     </row>
     <row r="306" spans="1:18">
       <c r="A306">
-        <v>6394</v>
+        <v>6785</v>
       </c>
       <c r="B306" t="s">
         <v>292</v>
@@ -23417,7 +23417,7 @@
     </row>
     <row r="307" spans="1:18">
       <c r="A307">
-        <v>6594</v>
+        <v>6985</v>
       </c>
       <c r="B307" t="s">
         <v>293</v>
@@ -23458,7 +23458,7 @@
     </row>
     <row r="308" spans="1:18">
       <c r="A308">
-        <v>6680</v>
+        <v>7071</v>
       </c>
       <c r="B308" t="s">
         <v>294</v>
@@ -23514,7 +23514,7 @@
     </row>
     <row r="309" spans="1:18">
       <c r="A309">
-        <v>6668</v>
+        <v>7059</v>
       </c>
       <c r="B309" t="s">
         <v>295</v>
@@ -23564,7 +23564,7 @@
     </row>
     <row r="310" spans="1:18">
       <c r="A310">
-        <v>6467</v>
+        <v>6858</v>
       </c>
       <c r="B310" t="s">
         <v>296</v>
@@ -23620,7 +23620,7 @@
     </row>
     <row r="311" spans="1:18">
       <c r="A311">
-        <v>6532</v>
+        <v>6923</v>
       </c>
       <c r="B311" t="s">
         <v>297</v>
@@ -23673,7 +23673,7 @@
     </row>
     <row r="312" spans="1:18">
       <c r="A312">
-        <v>6653</v>
+        <v>7044</v>
       </c>
       <c r="B312" t="s">
         <v>298</v>
@@ -23717,7 +23717,7 @@
     </row>
     <row r="313" spans="1:18">
       <c r="A313">
-        <v>6516</v>
+        <v>6907</v>
       </c>
       <c r="B313" t="s">
         <v>299</v>
@@ -23773,7 +23773,7 @@
     </row>
     <row r="314" spans="1:18">
       <c r="A314">
-        <v>6643</v>
+        <v>7034</v>
       </c>
       <c r="B314" t="s">
         <v>300</v>
@@ -23829,7 +23829,7 @@
     </row>
     <row r="315" spans="1:18">
       <c r="A315">
-        <v>6384</v>
+        <v>6775</v>
       </c>
       <c r="B315" t="s">
         <v>301</v>
@@ -23879,7 +23879,7 @@
     </row>
     <row r="316" spans="1:18">
       <c r="A316">
-        <v>6385</v>
+        <v>6776</v>
       </c>
       <c r="B316" t="s">
         <v>301</v>
@@ -23929,7 +23929,7 @@
     </row>
     <row r="317" spans="1:18">
       <c r="A317">
-        <v>6666</v>
+        <v>7057</v>
       </c>
       <c r="B317" t="s">
         <v>302</v>
@@ -23979,7 +23979,7 @@
     </row>
     <row r="318" spans="1:18">
       <c r="A318">
-        <v>6724</v>
+        <v>7115</v>
       </c>
       <c r="B318" t="s">
         <v>303</v>
@@ -24032,7 +24032,7 @@
     </row>
     <row r="319" spans="1:18">
       <c r="A319">
-        <v>6675</v>
+        <v>7066</v>
       </c>
       <c r="B319" t="s">
         <v>304</v>
@@ -24076,7 +24076,7 @@
     </row>
     <row r="320" spans="1:18">
       <c r="A320">
-        <v>6578</v>
+        <v>6969</v>
       </c>
       <c r="B320" t="s">
         <v>305</v>
@@ -24123,7 +24123,7 @@
     </row>
     <row r="321" spans="1:18">
       <c r="A321">
-        <v>6579</v>
+        <v>6970</v>
       </c>
       <c r="B321" t="s">
         <v>305</v>
@@ -24173,7 +24173,7 @@
     </row>
     <row r="322" spans="1:18">
       <c r="A322">
-        <v>6581</v>
+        <v>6972</v>
       </c>
       <c r="B322" t="s">
         <v>306</v>
@@ -24220,7 +24220,7 @@
     </row>
     <row r="323" spans="1:18">
       <c r="A323">
-        <v>6569</v>
+        <v>6960</v>
       </c>
       <c r="B323" t="s">
         <v>307</v>
@@ -24276,7 +24276,7 @@
     </row>
     <row r="324" spans="1:18">
       <c r="A324">
-        <v>6550</v>
+        <v>6941</v>
       </c>
       <c r="B324" t="s">
         <v>308</v>
@@ -24332,7 +24332,7 @@
     </row>
     <row r="325" spans="1:18">
       <c r="A325">
-        <v>6596</v>
+        <v>6987</v>
       </c>
       <c r="B325" t="s">
         <v>309</v>
@@ -24385,7 +24385,7 @@
     </row>
     <row r="326" spans="1:18">
       <c r="A326">
-        <v>6597</v>
+        <v>6988</v>
       </c>
       <c r="B326" t="s">
         <v>309</v>
@@ -24438,7 +24438,7 @@
     </row>
     <row r="327" spans="1:18">
       <c r="A327">
-        <v>6609</v>
+        <v>7000</v>
       </c>
       <c r="B327" t="s">
         <v>310</v>
@@ -24494,7 +24494,7 @@
     </row>
     <row r="328" spans="1:18">
       <c r="A328">
-        <v>6541</v>
+        <v>6932</v>
       </c>
       <c r="B328" t="s">
         <v>311</v>
@@ -24541,7 +24541,7 @@
     </row>
     <row r="329" spans="1:18">
       <c r="A329">
-        <v>6542</v>
+        <v>6933</v>
       </c>
       <c r="B329" t="s">
         <v>311</v>
@@ -24591,7 +24591,7 @@
     </row>
     <row r="330" spans="1:18">
       <c r="A330">
-        <v>6582</v>
+        <v>6973</v>
       </c>
       <c r="B330" t="s">
         <v>312</v>
@@ -24638,7 +24638,7 @@
     </row>
     <row r="331" spans="1:18">
       <c r="A331">
-        <v>6600</v>
+        <v>6991</v>
       </c>
       <c r="B331" t="s">
         <v>313</v>
@@ -24691,7 +24691,7 @@
     </row>
     <row r="332" spans="1:18">
       <c r="A332">
-        <v>6601</v>
+        <v>6992</v>
       </c>
       <c r="B332" t="s">
         <v>313</v>
@@ -24744,7 +24744,7 @@
     </row>
     <row r="333" spans="1:18">
       <c r="A333">
-        <v>6604</v>
+        <v>6995</v>
       </c>
       <c r="B333" t="s">
         <v>314</v>
@@ -24785,7 +24785,7 @@
     </row>
     <row r="334" spans="1:18">
       <c r="A334">
-        <v>6605</v>
+        <v>6996</v>
       </c>
       <c r="B334" t="s">
         <v>314</v>
@@ -24826,7 +24826,7 @@
     </row>
     <row r="335" spans="1:18">
       <c r="A335">
-        <v>6611</v>
+        <v>7002</v>
       </c>
       <c r="B335" t="s">
         <v>315</v>
@@ -24882,7 +24882,7 @@
     </row>
     <row r="336" spans="1:18">
       <c r="A336">
-        <v>6614</v>
+        <v>7005</v>
       </c>
       <c r="B336" t="s">
         <v>316</v>
@@ -24926,7 +24926,7 @@
     </row>
     <row r="337" spans="1:18">
       <c r="A337">
-        <v>6523</v>
+        <v>6914</v>
       </c>
       <c r="B337" t="s">
         <v>317</v>
@@ -24982,7 +24982,7 @@
     </row>
     <row r="338" spans="1:18">
       <c r="A338">
-        <v>6633</v>
+        <v>7024</v>
       </c>
       <c r="B338" t="s">
         <v>318</v>
@@ -25035,7 +25035,7 @@
     </row>
     <row r="339" spans="1:18">
       <c r="A339">
-        <v>6531</v>
+        <v>6922</v>
       </c>
       <c r="B339" t="s">
         <v>319</v>
@@ -25091,7 +25091,7 @@
     </row>
     <row r="340" spans="1:18">
       <c r="A340">
-        <v>6573</v>
+        <v>6964</v>
       </c>
       <c r="B340" t="s">
         <v>320</v>
@@ -25135,7 +25135,7 @@
     </row>
     <row r="341" spans="1:18">
       <c r="A341">
-        <v>6718</v>
+        <v>7109</v>
       </c>
       <c r="B341" t="s">
         <v>321</v>
@@ -25191,7 +25191,7 @@
     </row>
     <row r="342" spans="1:18">
       <c r="A342">
-        <v>6507</v>
+        <v>6898</v>
       </c>
       <c r="B342" t="s">
         <v>322</v>
@@ -25247,7 +25247,7 @@
     </row>
     <row r="343" spans="1:18">
       <c r="A343">
-        <v>6700</v>
+        <v>7091</v>
       </c>
       <c r="B343" t="s">
         <v>323</v>
@@ -25300,7 +25300,7 @@
     </row>
     <row r="344" spans="1:18">
       <c r="A344">
-        <v>6571</v>
+        <v>6962</v>
       </c>
       <c r="B344" t="s">
         <v>324</v>
@@ -25356,7 +25356,7 @@
     </row>
     <row r="345" spans="1:18">
       <c r="A345">
-        <v>6434</v>
+        <v>6825</v>
       </c>
       <c r="B345" t="s">
         <v>325</v>
@@ -25412,7 +25412,7 @@
     </row>
     <row r="346" spans="1:18">
       <c r="A346">
-        <v>6710</v>
+        <v>7101</v>
       </c>
       <c r="B346" t="s">
         <v>326</v>
@@ -25462,7 +25462,7 @@
     </row>
     <row r="347" spans="1:18">
       <c r="A347">
-        <v>6435</v>
+        <v>6826</v>
       </c>
       <c r="B347" t="s">
         <v>327</v>
@@ -25512,7 +25512,7 @@
     </row>
     <row r="348" spans="1:18">
       <c r="A348">
-        <v>6725</v>
+        <v>7116</v>
       </c>
       <c r="B348" t="s">
         <v>328</v>
@@ -25562,7 +25562,7 @@
     </row>
     <row r="349" spans="1:18">
       <c r="A349">
-        <v>6726</v>
+        <v>7117</v>
       </c>
       <c r="B349" t="s">
         <v>329</v>
@@ -25618,7 +25618,7 @@
     </row>
     <row r="350" spans="1:18">
       <c r="A350">
-        <v>6727</v>
+        <v>7118</v>
       </c>
       <c r="B350" t="s">
         <v>330</v>
@@ -25665,7 +25665,7 @@
     </row>
     <row r="351" spans="1:18">
       <c r="A351">
-        <v>6728</v>
+        <v>7119</v>
       </c>
       <c r="B351" t="s">
         <v>331</v>
@@ -25718,7 +25718,7 @@
     </row>
     <row r="352" spans="1:18">
       <c r="A352">
-        <v>6730</v>
+        <v>7121</v>
       </c>
       <c r="B352" t="s">
         <v>332</v>
@@ -25771,7 +25771,7 @@
     </row>
     <row r="353" spans="1:18">
       <c r="A353">
-        <v>6729</v>
+        <v>7120</v>
       </c>
       <c r="B353" t="s">
         <v>333</v>
@@ -25815,7 +25815,7 @@
     </row>
     <row r="354" spans="1:18">
       <c r="A354">
-        <v>6731</v>
+        <v>7122</v>
       </c>
       <c r="B354" t="s">
         <v>334</v>
@@ -25871,7 +25871,7 @@
     </row>
     <row r="355" spans="1:18">
       <c r="A355">
-        <v>6732</v>
+        <v>7123</v>
       </c>
       <c r="B355" t="s">
         <v>335</v>
@@ -25909,7 +25909,7 @@
     </row>
     <row r="356" spans="1:18">
       <c r="A356">
-        <v>6737</v>
+        <v>7128</v>
       </c>
       <c r="B356" t="s">
         <v>336</v>
@@ -25962,7 +25962,7 @@
     </row>
     <row r="357" spans="1:18">
       <c r="A357">
-        <v>6736</v>
+        <v>7127</v>
       </c>
       <c r="B357" t="s">
         <v>337</v>
@@ -26012,7 +26012,7 @@
     </row>
     <row r="358" spans="1:18">
       <c r="A358">
-        <v>6734</v>
+        <v>7125</v>
       </c>
       <c r="B358" t="s">
         <v>338</v>
@@ -26068,7 +26068,7 @@
     </row>
     <row r="359" spans="1:18">
       <c r="A359">
-        <v>6735</v>
+        <v>7126</v>
       </c>
       <c r="B359" t="s">
         <v>339</v>
@@ -26118,7 +26118,7 @@
     </row>
     <row r="360" spans="1:18">
       <c r="A360">
-        <v>6733</v>
+        <v>7124</v>
       </c>
       <c r="B360" t="s">
         <v>340</v>
@@ -26168,7 +26168,7 @@
     </row>
     <row r="361" spans="1:18">
       <c r="A361">
-        <v>6740</v>
+        <v>7131</v>
       </c>
       <c r="B361" t="s">
         <v>341</v>
@@ -26212,7 +26212,7 @@
     </row>
     <row r="362" spans="1:18">
       <c r="A362">
-        <v>6739</v>
+        <v>7130</v>
       </c>
       <c r="B362" t="s">
         <v>342</v>
@@ -26262,7 +26262,7 @@
     </row>
     <row r="363" spans="1:18">
       <c r="A363">
-        <v>6738</v>
+        <v>7129</v>
       </c>
       <c r="B363" t="s">
         <v>343</v>
@@ -26300,7 +26300,7 @@
     </row>
     <row r="364" spans="1:18">
       <c r="A364">
-        <v>6747</v>
+        <v>7138</v>
       </c>
       <c r="B364" t="s">
         <v>344</v>
@@ -26335,7 +26335,7 @@
     </row>
     <row r="365" spans="1:18">
       <c r="A365">
-        <v>6741</v>
+        <v>7132</v>
       </c>
       <c r="B365" t="s">
         <v>345</v>
@@ -26379,7 +26379,7 @@
     </row>
     <row r="366" spans="1:18">
       <c r="A366">
-        <v>6742</v>
+        <v>7133</v>
       </c>
       <c r="B366" t="s">
         <v>346</v>
@@ -26432,7 +26432,7 @@
     </row>
     <row r="367" spans="1:18">
       <c r="A367">
-        <v>6748</v>
+        <v>7139</v>
       </c>
       <c r="B367" t="s">
         <v>347</v>
@@ -26485,7 +26485,7 @@
     </row>
     <row r="368" spans="1:18">
       <c r="A368">
-        <v>6749</v>
+        <v>7140</v>
       </c>
       <c r="B368" t="s">
         <v>348</v>
@@ -26523,7 +26523,7 @@
     </row>
     <row r="369" spans="1:18">
       <c r="A369">
-        <v>6746</v>
+        <v>7137</v>
       </c>
       <c r="B369" t="s">
         <v>349</v>
@@ -26579,7 +26579,7 @@
     </row>
     <row r="370" spans="1:18">
       <c r="A370">
-        <v>6743</v>
+        <v>7134</v>
       </c>
       <c r="B370" t="s">
         <v>350</v>
@@ -26626,7 +26626,7 @@
     </row>
     <row r="371" spans="1:18">
       <c r="A371">
-        <v>6744</v>
+        <v>7135</v>
       </c>
       <c r="B371" t="s">
         <v>255</v>
@@ -26679,7 +26679,7 @@
     </row>
     <row r="372" spans="1:18">
       <c r="A372">
-        <v>6745</v>
+        <v>7136</v>
       </c>
       <c r="B372" t="s">
         <v>351</v>
@@ -26732,7 +26732,7 @@
     </row>
     <row r="373" spans="1:18">
       <c r="A373">
-        <v>6750</v>
+        <v>7141</v>
       </c>
       <c r="B373" t="s">
         <v>352</v>
@@ -26782,7 +26782,7 @@
     </row>
     <row r="374" spans="1:18">
       <c r="A374">
-        <v>6753</v>
+        <v>7144</v>
       </c>
       <c r="B374" t="s">
         <v>353</v>
@@ -26832,7 +26832,7 @@
     </row>
     <row r="375" spans="1:18">
       <c r="A375">
-        <v>6752</v>
+        <v>7143</v>
       </c>
       <c r="B375" t="s">
         <v>354</v>
@@ -26888,7 +26888,7 @@
     </row>
     <row r="376" spans="1:18">
       <c r="A376">
-        <v>6754</v>
+        <v>7145</v>
       </c>
       <c r="B376" t="s">
         <v>355</v>
@@ -26938,7 +26938,7 @@
     </row>
     <row r="377" spans="1:18">
       <c r="A377">
-        <v>6751</v>
+        <v>7142</v>
       </c>
       <c r="B377" t="s">
         <v>356</v>
@@ -26976,7 +26976,7 @@
     </row>
     <row r="378" spans="1:18">
       <c r="A378">
-        <v>6757</v>
+        <v>7148</v>
       </c>
       <c r="B378" t="s">
         <v>357</v>
@@ -27020,7 +27020,7 @@
     </row>
     <row r="379" spans="1:18">
       <c r="A379">
-        <v>6756</v>
+        <v>7147</v>
       </c>
       <c r="B379" t="s">
         <v>244</v>
@@ -27061,7 +27061,7 @@
     </row>
     <row r="380" spans="1:18">
       <c r="A380">
-        <v>6755</v>
+        <v>7146</v>
       </c>
       <c r="B380" t="s">
         <v>358</v>
@@ -27117,7 +27117,7 @@
     </row>
     <row r="381" spans="1:18">
       <c r="A381">
-        <v>6760</v>
+        <v>7151</v>
       </c>
       <c r="B381" t="s">
         <v>359</v>
@@ -27167,7 +27167,7 @@
     </row>
     <row r="382" spans="1:18">
       <c r="A382">
-        <v>6759</v>
+        <v>7150</v>
       </c>
       <c r="B382" t="s">
         <v>360</v>
@@ -27223,7 +27223,7 @@
     </row>
     <row r="383" spans="1:18">
       <c r="A383">
-        <v>6761</v>
+        <v>7152</v>
       </c>
       <c r="B383" t="s">
         <v>361</v>
@@ -27273,7 +27273,7 @@
     </row>
     <row r="384" spans="1:18">
       <c r="A384">
-        <v>6758</v>
+        <v>7149</v>
       </c>
       <c r="B384" t="s">
         <v>333</v>
@@ -27317,7 +27317,7 @@
     </row>
     <row r="385" spans="1:18">
       <c r="A385">
-        <v>6763</v>
+        <v>7154</v>
       </c>
       <c r="B385" t="s">
         <v>346</v>
@@ -27370,7 +27370,7 @@
     </row>
     <row r="386" spans="1:18">
       <c r="A386">
-        <v>6767</v>
+        <v>7158</v>
       </c>
       <c r="B386" t="s">
         <v>362</v>
@@ -27414,7 +27414,7 @@
     </row>
     <row r="387" spans="1:18">
       <c r="A387">
-        <v>6762</v>
+        <v>7153</v>
       </c>
       <c r="B387" t="s">
         <v>363</v>
@@ -27458,7 +27458,7 @@
     </row>
     <row r="388" spans="1:18">
       <c r="A388">
-        <v>6766</v>
+        <v>7157</v>
       </c>
       <c r="B388" t="s">
         <v>364</v>
@@ -27493,7 +27493,7 @@
     </row>
     <row r="389" spans="1:18">
       <c r="A389">
-        <v>6765</v>
+        <v>7156</v>
       </c>
       <c r="B389" t="s">
         <v>357</v>
@@ -27531,7 +27531,7 @@
     </row>
     <row r="390" spans="1:18">
       <c r="A390">
-        <v>6764</v>
+        <v>7155</v>
       </c>
       <c r="B390" t="s">
         <v>365</v>
@@ -27572,7 +27572,7 @@
     </row>
     <row r="391" spans="1:18">
       <c r="A391">
-        <v>6768</v>
+        <v>7159</v>
       </c>
       <c r="B391" t="s">
         <v>366</v>
@@ -27625,7 +27625,7 @@
     </row>
     <row r="392" spans="1:18">
       <c r="A392">
-        <v>6769</v>
+        <v>7160</v>
       </c>
       <c r="B392" t="s">
         <v>367</v>

</xml_diff>

<commit_message>
Add notable people review export
</commit_message>
<xml_diff>
--- a/data/exports/duplicate_candidates.xlsx
+++ b/data/exports/duplicate_candidates.xlsx
@@ -7420,7 +7420,7 @@
     </row>
     <row r="2" spans="1:18">
       <c r="A2">
-        <v>7036</v>
+        <v>7818</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
@@ -7476,7 +7476,7 @@
     </row>
     <row r="3" spans="1:18">
       <c r="A3">
-        <v>6948</v>
+        <v>7730</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
@@ -7526,7 +7526,7 @@
     </row>
     <row r="4" spans="1:18">
       <c r="A4">
-        <v>6913</v>
+        <v>7695</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -7582,7 +7582,7 @@
     </row>
     <row r="5" spans="1:18">
       <c r="A5">
-        <v>6803</v>
+        <v>7585</v>
       </c>
       <c r="B5" t="s">
         <v>21</v>
@@ -7638,7 +7638,7 @@
     </row>
     <row r="6" spans="1:18">
       <c r="A6">
-        <v>6821</v>
+        <v>7603</v>
       </c>
       <c r="B6" t="s">
         <v>22</v>
@@ -7694,7 +7694,7 @@
     </row>
     <row r="7" spans="1:18">
       <c r="A7">
-        <v>6866</v>
+        <v>7648</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
@@ -7744,7 +7744,7 @@
     </row>
     <row r="8" spans="1:18">
       <c r="A8">
-        <v>6878</v>
+        <v>7660</v>
       </c>
       <c r="B8" t="s">
         <v>24</v>
@@ -7800,7 +7800,7 @@
     </row>
     <row r="9" spans="1:18">
       <c r="A9">
-        <v>6846</v>
+        <v>7628</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>
@@ -7856,7 +7856,7 @@
     </row>
     <row r="10" spans="1:18">
       <c r="A10">
-        <v>6984</v>
+        <v>7766</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
@@ -7897,7 +7897,7 @@
     </row>
     <row r="11" spans="1:18">
       <c r="A11">
-        <v>6963</v>
+        <v>7745</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
@@ -7953,7 +7953,7 @@
     </row>
     <row r="12" spans="1:18">
       <c r="A12">
-        <v>6921</v>
+        <v>7703</v>
       </c>
       <c r="B12" t="s">
         <v>28</v>
@@ -8009,7 +8009,7 @@
     </row>
     <row r="13" spans="1:18">
       <c r="A13">
-        <v>7026</v>
+        <v>7808</v>
       </c>
       <c r="B13" t="s">
         <v>29</v>
@@ -8062,7 +8062,7 @@
     </row>
     <row r="14" spans="1:18">
       <c r="A14">
-        <v>7027</v>
+        <v>7809</v>
       </c>
       <c r="B14" t="s">
         <v>29</v>
@@ -8115,7 +8115,7 @@
     </row>
     <row r="15" spans="1:18">
       <c r="A15">
-        <v>7028</v>
+        <v>7810</v>
       </c>
       <c r="B15" t="s">
         <v>29</v>
@@ -8168,7 +8168,7 @@
     </row>
     <row r="16" spans="1:18">
       <c r="A16">
-        <v>7029</v>
+        <v>7811</v>
       </c>
       <c r="B16" t="s">
         <v>30</v>
@@ -8218,7 +8218,7 @@
     </row>
     <row r="17" spans="1:18">
       <c r="A17">
-        <v>7030</v>
+        <v>7812</v>
       </c>
       <c r="B17" t="s">
         <v>30</v>
@@ -8268,7 +8268,7 @@
     </row>
     <row r="18" spans="1:18">
       <c r="A18">
-        <v>7031</v>
+        <v>7813</v>
       </c>
       <c r="B18" t="s">
         <v>31</v>
@@ -8318,7 +8318,7 @@
     </row>
     <row r="19" spans="1:18">
       <c r="A19">
-        <v>6911</v>
+        <v>7693</v>
       </c>
       <c r="B19" t="s">
         <v>32</v>
@@ -8374,7 +8374,7 @@
     </row>
     <row r="20" spans="1:18">
       <c r="A20">
-        <v>6950</v>
+        <v>7732</v>
       </c>
       <c r="B20" t="s">
         <v>33</v>
@@ -8424,7 +8424,7 @@
     </row>
     <row r="21" spans="1:18">
       <c r="A21">
-        <v>7076</v>
+        <v>7858</v>
       </c>
       <c r="B21" t="s">
         <v>34</v>
@@ -8480,7 +8480,7 @@
     </row>
     <row r="22" spans="1:18">
       <c r="A22">
-        <v>6993</v>
+        <v>7775</v>
       </c>
       <c r="B22" t="s">
         <v>35</v>
@@ -8533,7 +8533,7 @@
     </row>
     <row r="23" spans="1:18">
       <c r="A23">
-        <v>6994</v>
+        <v>7776</v>
       </c>
       <c r="B23" t="s">
         <v>35</v>
@@ -8586,7 +8586,7 @@
     </row>
     <row r="24" spans="1:18">
       <c r="A24">
-        <v>7003</v>
+        <v>7785</v>
       </c>
       <c r="B24" t="s">
         <v>36</v>
@@ -8642,7 +8642,7 @@
     </row>
     <row r="25" spans="1:18">
       <c r="A25">
-        <v>6977</v>
+        <v>7759</v>
       </c>
       <c r="B25" t="s">
         <v>37</v>
@@ -8695,7 +8695,7 @@
     </row>
     <row r="26" spans="1:18">
       <c r="A26">
-        <v>6978</v>
+        <v>7760</v>
       </c>
       <c r="B26" t="s">
         <v>37</v>
@@ -8751,7 +8751,7 @@
     </row>
     <row r="27" spans="1:18">
       <c r="A27">
-        <v>6980</v>
+        <v>7762</v>
       </c>
       <c r="B27" t="s">
         <v>38</v>
@@ -8804,7 +8804,7 @@
     </row>
     <row r="28" spans="1:18">
       <c r="A28">
-        <v>6867</v>
+        <v>7649</v>
       </c>
       <c r="B28" t="s">
         <v>39</v>
@@ -8860,7 +8860,7 @@
     </row>
     <row r="29" spans="1:18">
       <c r="A29">
-        <v>6975</v>
+        <v>7757</v>
       </c>
       <c r="B29" t="s">
         <v>40</v>
@@ -8901,7 +8901,7 @@
     </row>
     <row r="30" spans="1:18">
       <c r="A30">
-        <v>6976</v>
+        <v>7758</v>
       </c>
       <c r="B30" t="s">
         <v>40</v>
@@ -8945,7 +8945,7 @@
     </row>
     <row r="31" spans="1:18">
       <c r="A31">
-        <v>6979</v>
+        <v>7761</v>
       </c>
       <c r="B31" t="s">
         <v>41</v>
@@ -8986,7 +8986,7 @@
     </row>
     <row r="32" spans="1:18">
       <c r="A32">
-        <v>7080</v>
+        <v>7862</v>
       </c>
       <c r="B32" t="s">
         <v>42</v>
@@ -9042,7 +9042,7 @@
     </row>
     <row r="33" spans="1:18">
       <c r="A33">
-        <v>6901</v>
+        <v>7683</v>
       </c>
       <c r="B33" t="s">
         <v>43</v>
@@ -9098,7 +9098,7 @@
     </row>
     <row r="34" spans="1:18">
       <c r="A34">
-        <v>6902</v>
+        <v>7684</v>
       </c>
       <c r="B34" t="s">
         <v>44</v>
@@ -9139,7 +9139,7 @@
     </row>
     <row r="35" spans="1:18">
       <c r="A35">
-        <v>6942</v>
+        <v>7724</v>
       </c>
       <c r="B35" t="s">
         <v>45</v>
@@ -9195,7 +9195,7 @@
     </row>
     <row r="36" spans="1:18">
       <c r="A36">
-        <v>6928</v>
+        <v>7710</v>
       </c>
       <c r="B36" t="s">
         <v>46</v>
@@ -9248,7 +9248,7 @@
     </row>
     <row r="37" spans="1:18">
       <c r="A37">
-        <v>6929</v>
+        <v>7711</v>
       </c>
       <c r="B37" t="s">
         <v>46</v>
@@ -9304,7 +9304,7 @@
     </row>
     <row r="38" spans="1:18">
       <c r="A38">
-        <v>6931</v>
+        <v>7713</v>
       </c>
       <c r="B38" t="s">
         <v>47</v>
@@ -9357,7 +9357,7 @@
     </row>
     <row r="39" spans="1:18">
       <c r="A39">
-        <v>6934</v>
+        <v>7716</v>
       </c>
       <c r="B39" t="s">
         <v>48</v>
@@ -9404,7 +9404,7 @@
     </row>
     <row r="40" spans="1:18">
       <c r="A40">
-        <v>6935</v>
+        <v>7717</v>
       </c>
       <c r="B40" t="s">
         <v>48</v>
@@ -9454,7 +9454,7 @@
     </row>
     <row r="41" spans="1:18">
       <c r="A41">
-        <v>6974</v>
+        <v>7756</v>
       </c>
       <c r="B41" t="s">
         <v>49</v>
@@ -9501,7 +9501,7 @@
     </row>
     <row r="42" spans="1:18">
       <c r="A42">
-        <v>6989</v>
+        <v>7771</v>
       </c>
       <c r="B42" t="s">
         <v>50</v>
@@ -9554,7 +9554,7 @@
     </row>
     <row r="43" spans="1:18">
       <c r="A43">
-        <v>6990</v>
+        <v>7772</v>
       </c>
       <c r="B43" t="s">
         <v>50</v>
@@ -9607,7 +9607,7 @@
     </row>
     <row r="44" spans="1:18">
       <c r="A44">
-        <v>7001</v>
+        <v>7783</v>
       </c>
       <c r="B44" t="s">
         <v>51</v>
@@ -9663,7 +9663,7 @@
     </row>
     <row r="45" spans="1:18">
       <c r="A45">
-        <v>6834</v>
+        <v>7616</v>
       </c>
       <c r="B45" t="s">
         <v>52</v>
@@ -9713,7 +9713,7 @@
     </row>
     <row r="46" spans="1:18">
       <c r="A46">
-        <v>7099</v>
+        <v>7881</v>
       </c>
       <c r="B46" t="s">
         <v>53</v>
@@ -9769,7 +9769,7 @@
     </row>
     <row r="47" spans="1:18">
       <c r="A47">
-        <v>6814</v>
+        <v>7596</v>
       </c>
       <c r="B47" t="s">
         <v>54</v>
@@ -9822,7 +9822,7 @@
     </row>
     <row r="48" spans="1:18">
       <c r="A48">
-        <v>6965</v>
+        <v>7747</v>
       </c>
       <c r="B48" t="s">
         <v>55</v>
@@ -9875,7 +9875,7 @@
     </row>
     <row r="49" spans="1:18">
       <c r="A49">
-        <v>6999</v>
+        <v>7781</v>
       </c>
       <c r="B49" t="s">
         <v>56</v>
@@ -9931,7 +9931,7 @@
     </row>
     <row r="50" spans="1:18">
       <c r="A50">
-        <v>6813</v>
+        <v>7595</v>
       </c>
       <c r="B50" t="s">
         <v>57</v>
@@ -9978,7 +9978,7 @@
     </row>
     <row r="51" spans="1:18">
       <c r="A51">
-        <v>7064</v>
+        <v>7846</v>
       </c>
       <c r="B51" t="s">
         <v>58</v>
@@ -10028,7 +10028,7 @@
     </row>
     <row r="52" spans="1:18">
       <c r="A52">
-        <v>6912</v>
+        <v>7694</v>
       </c>
       <c r="B52" t="s">
         <v>59</v>
@@ -10084,7 +10084,7 @@
     </row>
     <row r="53" spans="1:18">
       <c r="A53">
-        <v>7013</v>
+        <v>7795</v>
       </c>
       <c r="B53" t="s">
         <v>60</v>
@@ -10137,7 +10137,7 @@
     </row>
     <row r="54" spans="1:18">
       <c r="A54">
-        <v>7018</v>
+        <v>7800</v>
       </c>
       <c r="B54" t="s">
         <v>61</v>
@@ -10190,7 +10190,7 @@
     </row>
     <row r="55" spans="1:18">
       <c r="A55">
-        <v>7093</v>
+        <v>7875</v>
       </c>
       <c r="B55" t="s">
         <v>62</v>
@@ -10243,7 +10243,7 @@
     </row>
     <row r="56" spans="1:18">
       <c r="A56">
-        <v>6816</v>
+        <v>7598</v>
       </c>
       <c r="B56" t="s">
         <v>63</v>
@@ -10287,7 +10287,7 @@
     </row>
     <row r="57" spans="1:18">
       <c r="A57">
-        <v>6924</v>
+        <v>7706</v>
       </c>
       <c r="B57" t="s">
         <v>64</v>
@@ -10343,7 +10343,7 @@
     </row>
     <row r="58" spans="1:18">
       <c r="A58">
-        <v>7016</v>
+        <v>7798</v>
       </c>
       <c r="B58" t="s">
         <v>65</v>
@@ -10396,7 +10396,7 @@
     </row>
     <row r="59" spans="1:18">
       <c r="A59">
-        <v>6848</v>
+        <v>7630</v>
       </c>
       <c r="B59" t="s">
         <v>66</v>
@@ -10449,7 +10449,7 @@
     </row>
     <row r="60" spans="1:18">
       <c r="A60">
-        <v>6771</v>
+        <v>7553</v>
       </c>
       <c r="B60" t="s">
         <v>67</v>
@@ -10502,7 +10502,7 @@
     </row>
     <row r="61" spans="1:18">
       <c r="A61">
-        <v>7037</v>
+        <v>7819</v>
       </c>
       <c r="B61" t="s">
         <v>68</v>
@@ -10555,7 +10555,7 @@
     </row>
     <row r="62" spans="1:18">
       <c r="A62">
-        <v>7025</v>
+        <v>7807</v>
       </c>
       <c r="B62" t="s">
         <v>69</v>
@@ -10608,7 +10608,7 @@
     </row>
     <row r="63" spans="1:18">
       <c r="A63">
-        <v>6939</v>
+        <v>7721</v>
       </c>
       <c r="B63" t="s">
         <v>70</v>
@@ -10664,7 +10664,7 @@
     </row>
     <row r="64" spans="1:18">
       <c r="A64">
-        <v>6903</v>
+        <v>7685</v>
       </c>
       <c r="B64" t="s">
         <v>71</v>
@@ -10717,7 +10717,7 @@
     </row>
     <row r="65" spans="1:18">
       <c r="A65">
-        <v>6891</v>
+        <v>7673</v>
       </c>
       <c r="B65" t="s">
         <v>72</v>
@@ -10764,7 +10764,7 @@
     </row>
     <row r="66" spans="1:18">
       <c r="A66">
-        <v>6915</v>
+        <v>7697</v>
       </c>
       <c r="B66" t="s">
         <v>73</v>
@@ -10820,7 +10820,7 @@
     </row>
     <row r="67" spans="1:18">
       <c r="A67">
-        <v>6855</v>
+        <v>7637</v>
       </c>
       <c r="B67" t="s">
         <v>74</v>
@@ -10870,7 +10870,7 @@
     </row>
     <row r="68" spans="1:18">
       <c r="A68">
-        <v>7111</v>
+        <v>7893</v>
       </c>
       <c r="B68" t="s">
         <v>75</v>
@@ -10920,7 +10920,7 @@
     </row>
     <row r="69" spans="1:18">
       <c r="A69">
-        <v>6909</v>
+        <v>7691</v>
       </c>
       <c r="B69" t="s">
         <v>76</v>
@@ -10976,7 +10976,7 @@
     </row>
     <row r="70" spans="1:18">
       <c r="A70">
-        <v>7106</v>
+        <v>7888</v>
       </c>
       <c r="B70" t="s">
         <v>77</v>
@@ -11032,7 +11032,7 @@
     </row>
     <row r="71" spans="1:18">
       <c r="A71">
-        <v>6936</v>
+        <v>7718</v>
       </c>
       <c r="B71" t="s">
         <v>78</v>
@@ -11079,7 +11079,7 @@
     </row>
     <row r="72" spans="1:18">
       <c r="A72">
-        <v>6937</v>
+        <v>7719</v>
       </c>
       <c r="B72" t="s">
         <v>78</v>
@@ -11129,7 +11129,7 @@
     </row>
     <row r="73" spans="1:18">
       <c r="A73">
-        <v>6986</v>
+        <v>7768</v>
       </c>
       <c r="B73" t="s">
         <v>79</v>
@@ -11176,7 +11176,7 @@
     </row>
     <row r="74" spans="1:18">
       <c r="A74">
-        <v>7033</v>
+        <v>7815</v>
       </c>
       <c r="B74" t="s">
         <v>80</v>
@@ -11220,7 +11220,7 @@
     </row>
     <row r="75" spans="1:18">
       <c r="A75">
-        <v>7100</v>
+        <v>7882</v>
       </c>
       <c r="B75" t="s">
         <v>81</v>
@@ -11273,7 +11273,7 @@
     </row>
     <row r="76" spans="1:18">
       <c r="A76">
-        <v>6959</v>
+        <v>7741</v>
       </c>
       <c r="B76" t="s">
         <v>82</v>
@@ -11329,7 +11329,7 @@
     </row>
     <row r="77" spans="1:18">
       <c r="A77">
-        <v>6773</v>
+        <v>7555</v>
       </c>
       <c r="B77" t="s">
         <v>83</v>
@@ -11382,7 +11382,7 @@
     </row>
     <row r="78" spans="1:18">
       <c r="A78">
-        <v>6997</v>
+        <v>7779</v>
       </c>
       <c r="B78" t="s">
         <v>84</v>
@@ -11435,7 +11435,7 @@
     </row>
     <row r="79" spans="1:18">
       <c r="A79">
-        <v>6998</v>
+        <v>7780</v>
       </c>
       <c r="B79" t="s">
         <v>84</v>
@@ -11488,7 +11488,7 @@
     </row>
     <row r="80" spans="1:18">
       <c r="A80">
-        <v>7006</v>
+        <v>7788</v>
       </c>
       <c r="B80" t="s">
         <v>85</v>
@@ -11544,7 +11544,7 @@
     </row>
     <row r="81" spans="1:18">
       <c r="A81">
-        <v>6961</v>
+        <v>7743</v>
       </c>
       <c r="B81" t="s">
         <v>86</v>
@@ -11600,7 +11600,7 @@
     </row>
     <row r="82" spans="1:18">
       <c r="A82">
-        <v>6946</v>
+        <v>7728</v>
       </c>
       <c r="B82" t="s">
         <v>87</v>
@@ -11656,7 +11656,7 @@
     </row>
     <row r="83" spans="1:18">
       <c r="A83">
-        <v>6870</v>
+        <v>7652</v>
       </c>
       <c r="B83" t="s">
         <v>88</v>
@@ -11712,7 +11712,7 @@
     </row>
     <row r="84" spans="1:18">
       <c r="A84">
-        <v>6871</v>
+        <v>7653</v>
       </c>
       <c r="B84" t="s">
         <v>88</v>
@@ -11768,7 +11768,7 @@
     </row>
     <row r="85" spans="1:18">
       <c r="A85">
-        <v>6888</v>
+        <v>7670</v>
       </c>
       <c r="B85" t="s">
         <v>89</v>
@@ -11824,7 +11824,7 @@
     </row>
     <row r="86" spans="1:18">
       <c r="A86">
-        <v>7074</v>
+        <v>7856</v>
       </c>
       <c r="B86" t="s">
         <v>90</v>
@@ -11880,7 +11880,7 @@
     </row>
     <row r="87" spans="1:18">
       <c r="A87">
-        <v>6882</v>
+        <v>7664</v>
       </c>
       <c r="B87" t="s">
         <v>91</v>
@@ -11936,7 +11936,7 @@
     </row>
     <row r="88" spans="1:18">
       <c r="A88">
-        <v>7035</v>
+        <v>7817</v>
       </c>
       <c r="B88" t="s">
         <v>92</v>
@@ -11992,7 +11992,7 @@
     </row>
     <row r="89" spans="1:18">
       <c r="A89">
-        <v>6796</v>
+        <v>7578</v>
       </c>
       <c r="B89" t="s">
         <v>93</v>
@@ -12048,7 +12048,7 @@
     </row>
     <row r="90" spans="1:18">
       <c r="A90">
-        <v>6797</v>
+        <v>7579</v>
       </c>
       <c r="B90" t="s">
         <v>93</v>
@@ -12104,7 +12104,7 @@
     </row>
     <row r="91" spans="1:18">
       <c r="A91">
-        <v>6804</v>
+        <v>7586</v>
       </c>
       <c r="B91" t="s">
         <v>94</v>
@@ -12157,7 +12157,7 @@
     </row>
     <row r="92" spans="1:18">
       <c r="A92">
-        <v>6944</v>
+        <v>7726</v>
       </c>
       <c r="B92" t="s">
         <v>95</v>
@@ -12210,7 +12210,7 @@
     </row>
     <row r="93" spans="1:18">
       <c r="A93">
-        <v>6792</v>
+        <v>7574</v>
       </c>
       <c r="B93" t="s">
         <v>96</v>
@@ -12254,7 +12254,7 @@
     </row>
     <row r="94" spans="1:18">
       <c r="A94">
-        <v>7040</v>
+        <v>7822</v>
       </c>
       <c r="B94" t="s">
         <v>97</v>
@@ -12310,7 +12310,7 @@
     </row>
     <row r="95" spans="1:18">
       <c r="A95">
-        <v>6852</v>
+        <v>7634</v>
       </c>
       <c r="B95" t="s">
         <v>98</v>
@@ -12363,7 +12363,7 @@
     </row>
     <row r="96" spans="1:18">
       <c r="A96">
-        <v>7021</v>
+        <v>7803</v>
       </c>
       <c r="B96" t="s">
         <v>99</v>
@@ -12416,7 +12416,7 @@
     </row>
     <row r="97" spans="1:18">
       <c r="A97">
-        <v>7096</v>
+        <v>7878</v>
       </c>
       <c r="B97" t="s">
         <v>100</v>
@@ -12469,7 +12469,7 @@
     </row>
     <row r="98" spans="1:18">
       <c r="A98">
-        <v>6856</v>
+        <v>7638</v>
       </c>
       <c r="B98" t="s">
         <v>101</v>
@@ -12525,7 +12525,7 @@
     </row>
     <row r="99" spans="1:18">
       <c r="A99">
-        <v>6811</v>
+        <v>7593</v>
       </c>
       <c r="B99" t="s">
         <v>102</v>
@@ -12569,7 +12569,7 @@
     </row>
     <row r="100" spans="1:18">
       <c r="A100">
-        <v>6812</v>
+        <v>7594</v>
       </c>
       <c r="B100" t="s">
         <v>102</v>
@@ -12613,7 +12613,7 @@
     </row>
     <row r="101" spans="1:18">
       <c r="A101">
-        <v>6874</v>
+        <v>7656</v>
       </c>
       <c r="B101" t="s">
         <v>103</v>
@@ -12657,7 +12657,7 @@
     </row>
     <row r="102" spans="1:18">
       <c r="A102">
-        <v>7107</v>
+        <v>7889</v>
       </c>
       <c r="B102" t="s">
         <v>104</v>
@@ -12698,7 +12698,7 @@
     </row>
     <row r="103" spans="1:18">
       <c r="A103">
-        <v>6982</v>
+        <v>7764</v>
       </c>
       <c r="B103" t="s">
         <v>105</v>
@@ -12739,7 +12739,7 @@
     </row>
     <row r="104" spans="1:18">
       <c r="A104">
-        <v>6829</v>
+        <v>7611</v>
       </c>
       <c r="B104" t="s">
         <v>106</v>
@@ -12789,7 +12789,7 @@
     </row>
     <row r="105" spans="1:18">
       <c r="A105">
-        <v>6782</v>
+        <v>7564</v>
       </c>
       <c r="B105" t="s">
         <v>107</v>
@@ -12842,7 +12842,7 @@
     </row>
     <row r="106" spans="1:18">
       <c r="A106">
-        <v>7086</v>
+        <v>7868</v>
       </c>
       <c r="B106" t="s">
         <v>108</v>
@@ -12892,7 +12892,7 @@
     </row>
     <row r="107" spans="1:18">
       <c r="A107">
-        <v>7010</v>
+        <v>7792</v>
       </c>
       <c r="B107" t="s">
         <v>109</v>
@@ -12945,7 +12945,7 @@
     </row>
     <row r="108" spans="1:18">
       <c r="A108">
-        <v>7062</v>
+        <v>7844</v>
       </c>
       <c r="B108" t="s">
         <v>110</v>
@@ -12992,7 +12992,7 @@
     </row>
     <row r="109" spans="1:18">
       <c r="A109">
-        <v>7014</v>
+        <v>7796</v>
       </c>
       <c r="B109" t="s">
         <v>111</v>
@@ -13045,7 +13045,7 @@
     </row>
     <row r="110" spans="1:18">
       <c r="A110">
-        <v>7032</v>
+        <v>7814</v>
       </c>
       <c r="B110" t="s">
         <v>112</v>
@@ -13083,7 +13083,7 @@
     </row>
     <row r="111" spans="1:18">
       <c r="A111">
-        <v>6895</v>
+        <v>7677</v>
       </c>
       <c r="B111" t="s">
         <v>113</v>
@@ -13139,7 +13139,7 @@
     </row>
     <row r="112" spans="1:18">
       <c r="A112">
-        <v>6809</v>
+        <v>7591</v>
       </c>
       <c r="B112" t="s">
         <v>114</v>
@@ -13189,7 +13189,7 @@
     </row>
     <row r="113" spans="1:18">
       <c r="A113">
-        <v>6810</v>
+        <v>7592</v>
       </c>
       <c r="B113" t="s">
         <v>114</v>
@@ -13239,7 +13239,7 @@
     </row>
     <row r="114" spans="1:18">
       <c r="A114">
-        <v>6873</v>
+        <v>7655</v>
       </c>
       <c r="B114" t="s">
         <v>115</v>
@@ -13289,7 +13289,7 @@
     </row>
     <row r="115" spans="1:18">
       <c r="A115">
-        <v>6799</v>
+        <v>7581</v>
       </c>
       <c r="B115" t="s">
         <v>116</v>
@@ -13333,7 +13333,7 @@
     </row>
     <row r="116" spans="1:18">
       <c r="A116">
-        <v>6800</v>
+        <v>7582</v>
       </c>
       <c r="B116" t="s">
         <v>116</v>
@@ -13377,7 +13377,7 @@
     </row>
     <row r="117" spans="1:18">
       <c r="A117">
-        <v>6872</v>
+        <v>7654</v>
       </c>
       <c r="B117" t="s">
         <v>117</v>
@@ -13421,7 +13421,7 @@
     </row>
     <row r="118" spans="1:18">
       <c r="A118">
-        <v>7058</v>
+        <v>7840</v>
       </c>
       <c r="B118" t="s">
         <v>118</v>
@@ -13471,7 +13471,7 @@
     </row>
     <row r="119" spans="1:18">
       <c r="A119">
-        <v>6836</v>
+        <v>7618</v>
       </c>
       <c r="B119" t="s">
         <v>119</v>
@@ -13521,7 +13521,7 @@
     </row>
     <row r="120" spans="1:18">
       <c r="A120">
-        <v>6847</v>
+        <v>7629</v>
       </c>
       <c r="B120" t="s">
         <v>120</v>
@@ -13577,7 +13577,7 @@
     </row>
     <row r="121" spans="1:18">
       <c r="A121">
-        <v>6860</v>
+        <v>7642</v>
       </c>
       <c r="B121" t="s">
         <v>121</v>
@@ -13615,7 +13615,7 @@
     </row>
     <row r="122" spans="1:18">
       <c r="A122">
-        <v>6951</v>
+        <v>7733</v>
       </c>
       <c r="B122" t="s">
         <v>122</v>
@@ -13671,7 +13671,7 @@
     </row>
     <row r="123" spans="1:18">
       <c r="A123">
-        <v>6954</v>
+        <v>7736</v>
       </c>
       <c r="B123" t="s">
         <v>123</v>
@@ -13727,7 +13727,7 @@
     </row>
     <row r="124" spans="1:18">
       <c r="A124">
-        <v>7008</v>
+        <v>7790</v>
       </c>
       <c r="B124" t="s">
         <v>124</v>
@@ -13780,7 +13780,7 @@
     </row>
     <row r="125" spans="1:18">
       <c r="A125">
-        <v>7061</v>
+        <v>7843</v>
       </c>
       <c r="B125" t="s">
         <v>125</v>
@@ -13830,7 +13830,7 @@
     </row>
     <row r="126" spans="1:18">
       <c r="A126">
-        <v>7009</v>
+        <v>7791</v>
       </c>
       <c r="B126" t="s">
         <v>126</v>
@@ -13883,7 +13883,7 @@
     </row>
     <row r="127" spans="1:18">
       <c r="A127">
-        <v>6786</v>
+        <v>7568</v>
       </c>
       <c r="B127" t="s">
         <v>127</v>
@@ -13936,7 +13936,7 @@
     </row>
     <row r="128" spans="1:18">
       <c r="A128">
-        <v>6835</v>
+        <v>7617</v>
       </c>
       <c r="B128" t="s">
         <v>128</v>
@@ -13980,7 +13980,7 @@
     </row>
     <row r="129" spans="1:18">
       <c r="A129">
-        <v>7073</v>
+        <v>7855</v>
       </c>
       <c r="B129" t="s">
         <v>129</v>
@@ -14036,7 +14036,7 @@
     </row>
     <row r="130" spans="1:18">
       <c r="A130">
-        <v>6908</v>
+        <v>7690</v>
       </c>
       <c r="B130" t="s">
         <v>130</v>
@@ -14092,7 +14092,7 @@
     </row>
     <row r="131" spans="1:18">
       <c r="A131">
-        <v>6916</v>
+        <v>7698</v>
       </c>
       <c r="B131" t="s">
         <v>131</v>
@@ -14148,7 +14148,7 @@
     </row>
     <row r="132" spans="1:18">
       <c r="A132">
-        <v>6894</v>
+        <v>7676</v>
       </c>
       <c r="B132" t="s">
         <v>132</v>
@@ -14204,7 +14204,7 @@
     </row>
     <row r="133" spans="1:18">
       <c r="A133">
-        <v>7022</v>
+        <v>7804</v>
       </c>
       <c r="B133" t="s">
         <v>133</v>
@@ -14257,7 +14257,7 @@
     </row>
     <row r="134" spans="1:18">
       <c r="A134">
-        <v>6892</v>
+        <v>7674</v>
       </c>
       <c r="B134" t="s">
         <v>134</v>
@@ -14313,7 +14313,7 @@
     </row>
     <row r="135" spans="1:18">
       <c r="A135">
-        <v>7053</v>
+        <v>7835</v>
       </c>
       <c r="B135" t="s">
         <v>135</v>
@@ -14369,7 +14369,7 @@
     </row>
     <row r="136" spans="1:18">
       <c r="A136">
-        <v>6838</v>
+        <v>7620</v>
       </c>
       <c r="B136" t="s">
         <v>136</v>
@@ -14413,7 +14413,7 @@
     </row>
     <row r="137" spans="1:18">
       <c r="A137">
-        <v>7065</v>
+        <v>7847</v>
       </c>
       <c r="B137" t="s">
         <v>137</v>
@@ -14463,7 +14463,7 @@
     </row>
     <row r="138" spans="1:18">
       <c r="A138">
-        <v>6833</v>
+        <v>7615</v>
       </c>
       <c r="B138" t="s">
         <v>138</v>
@@ -14513,7 +14513,7 @@
     </row>
     <row r="139" spans="1:18">
       <c r="A139">
-        <v>6853</v>
+        <v>7635</v>
       </c>
       <c r="B139" t="s">
         <v>139</v>
@@ -14569,7 +14569,7 @@
     </row>
     <row r="140" spans="1:18">
       <c r="A140">
-        <v>6943</v>
+        <v>7725</v>
       </c>
       <c r="B140" t="s">
         <v>140</v>
@@ -14625,7 +14625,7 @@
     </row>
     <row r="141" spans="1:18">
       <c r="A141">
-        <v>6832</v>
+        <v>7614</v>
       </c>
       <c r="B141" t="s">
         <v>141</v>
@@ -14663,7 +14663,7 @@
     </row>
     <row r="142" spans="1:18">
       <c r="A142">
-        <v>7098</v>
+        <v>7880</v>
       </c>
       <c r="B142" t="s">
         <v>142</v>
@@ -14716,7 +14716,7 @@
     </row>
     <row r="143" spans="1:18">
       <c r="A143">
-        <v>6859</v>
+        <v>7641</v>
       </c>
       <c r="B143" t="s">
         <v>143</v>
@@ -14769,7 +14769,7 @@
     </row>
     <row r="144" spans="1:18">
       <c r="A144">
-        <v>6789</v>
+        <v>7571</v>
       </c>
       <c r="B144" t="s">
         <v>144</v>
@@ -14822,7 +14822,7 @@
     </row>
     <row r="145" spans="1:18">
       <c r="A145">
-        <v>6956</v>
+        <v>7738</v>
       </c>
       <c r="B145" t="s">
         <v>145</v>
@@ -14878,7 +14878,7 @@
     </row>
     <row r="146" spans="1:18">
       <c r="A146">
-        <v>6957</v>
+        <v>7739</v>
       </c>
       <c r="B146" t="s">
         <v>145</v>
@@ -14934,7 +14934,7 @@
     </row>
     <row r="147" spans="1:18">
       <c r="A147">
-        <v>6958</v>
+        <v>7740</v>
       </c>
       <c r="B147" t="s">
         <v>146</v>
@@ -14990,7 +14990,7 @@
     </row>
     <row r="148" spans="1:18">
       <c r="A148">
-        <v>7083</v>
+        <v>7865</v>
       </c>
       <c r="B148" t="s">
         <v>147</v>
@@ -15046,7 +15046,7 @@
     </row>
     <row r="149" spans="1:18">
       <c r="A149">
-        <v>7055</v>
+        <v>7837</v>
       </c>
       <c r="B149" t="s">
         <v>148</v>
@@ -15102,7 +15102,7 @@
     </row>
     <row r="150" spans="1:18">
       <c r="A150">
-        <v>6971</v>
+        <v>7753</v>
       </c>
       <c r="B150" t="s">
         <v>149</v>
@@ -15155,7 +15155,7 @@
     </row>
     <row r="151" spans="1:18">
       <c r="A151">
-        <v>6886</v>
+        <v>7668</v>
       </c>
       <c r="B151" t="s">
         <v>150</v>
@@ -15211,7 +15211,7 @@
     </row>
     <row r="152" spans="1:18">
       <c r="A152">
-        <v>6884</v>
+        <v>7666</v>
       </c>
       <c r="B152" t="s">
         <v>151</v>
@@ -15267,7 +15267,7 @@
     </row>
     <row r="153" spans="1:18">
       <c r="A153">
-        <v>7017</v>
+        <v>7799</v>
       </c>
       <c r="B153" t="s">
         <v>152</v>
@@ -15320,7 +15320,7 @@
     </row>
     <row r="154" spans="1:18">
       <c r="A154">
-        <v>6863</v>
+        <v>7645</v>
       </c>
       <c r="B154" t="s">
         <v>153</v>
@@ -15376,7 +15376,7 @@
     </row>
     <row r="155" spans="1:18">
       <c r="A155">
-        <v>7075</v>
+        <v>7857</v>
       </c>
       <c r="B155" t="s">
         <v>154</v>
@@ -15432,7 +15432,7 @@
     </row>
     <row r="156" spans="1:18">
       <c r="A156">
-        <v>6949</v>
+        <v>7731</v>
       </c>
       <c r="B156" t="s">
         <v>155</v>
@@ -15482,7 +15482,7 @@
     </row>
     <row r="157" spans="1:18">
       <c r="A157">
-        <v>6883</v>
+        <v>7665</v>
       </c>
       <c r="B157" t="s">
         <v>156</v>
@@ -15538,7 +15538,7 @@
     </row>
     <row r="158" spans="1:18">
       <c r="A158">
-        <v>6983</v>
+        <v>7765</v>
       </c>
       <c r="B158" t="s">
         <v>157</v>
@@ -15579,7 +15579,7 @@
     </row>
     <row r="159" spans="1:18">
       <c r="A159">
-        <v>7004</v>
+        <v>7786</v>
       </c>
       <c r="B159" t="s">
         <v>158</v>
@@ -15629,7 +15629,7 @@
     </row>
     <row r="160" spans="1:18">
       <c r="A160">
-        <v>7114</v>
+        <v>7896</v>
       </c>
       <c r="B160" t="s">
         <v>159</v>
@@ -15685,7 +15685,7 @@
     </row>
     <row r="161" spans="1:18">
       <c r="A161">
-        <v>6798</v>
+        <v>7580</v>
       </c>
       <c r="B161" t="s">
         <v>160</v>
@@ -15741,7 +15741,7 @@
     </row>
     <row r="162" spans="1:18">
       <c r="A162">
-        <v>6981</v>
+        <v>7763</v>
       </c>
       <c r="B162" t="s">
         <v>161</v>
@@ -15794,7 +15794,7 @@
     </row>
     <row r="163" spans="1:18">
       <c r="A163">
-        <v>7015</v>
+        <v>7797</v>
       </c>
       <c r="B163" t="s">
         <v>162</v>
@@ -15847,7 +15847,7 @@
     </row>
     <row r="164" spans="1:18">
       <c r="A164">
-        <v>6828</v>
+        <v>7610</v>
       </c>
       <c r="B164" t="s">
         <v>163</v>
@@ -15885,7 +15885,7 @@
     </row>
     <row r="165" spans="1:18">
       <c r="A165">
-        <v>7072</v>
+        <v>7854</v>
       </c>
       <c r="B165" t="s">
         <v>164</v>
@@ -15941,7 +15941,7 @@
     </row>
     <row r="166" spans="1:18">
       <c r="A166">
-        <v>6854</v>
+        <v>7636</v>
       </c>
       <c r="B166" t="s">
         <v>165</v>
@@ -15997,7 +15997,7 @@
     </row>
     <row r="167" spans="1:18">
       <c r="A167">
-        <v>6861</v>
+        <v>7643</v>
       </c>
       <c r="B167" t="s">
         <v>166</v>
@@ -16050,7 +16050,7 @@
     </row>
     <row r="168" spans="1:18">
       <c r="A168">
-        <v>6849</v>
+        <v>7631</v>
       </c>
       <c r="B168" t="s">
         <v>167</v>
@@ -16103,7 +16103,7 @@
     </row>
     <row r="169" spans="1:18">
       <c r="A169">
-        <v>6896</v>
+        <v>7678</v>
       </c>
       <c r="B169" t="s">
         <v>168</v>
@@ -16147,7 +16147,7 @@
     </row>
     <row r="170" spans="1:18">
       <c r="A170">
-        <v>6790</v>
+        <v>7572</v>
       </c>
       <c r="B170" t="s">
         <v>169</v>
@@ -16203,7 +16203,7 @@
     </row>
     <row r="171" spans="1:18">
       <c r="A171">
-        <v>7078</v>
+        <v>7860</v>
       </c>
       <c r="B171" t="s">
         <v>170</v>
@@ -16259,7 +16259,7 @@
     </row>
     <row r="172" spans="1:18">
       <c r="A172">
-        <v>6967</v>
+        <v>7749</v>
       </c>
       <c r="B172" t="s">
         <v>171</v>
@@ -16312,7 +16312,7 @@
     </row>
     <row r="173" spans="1:18">
       <c r="A173">
-        <v>7085</v>
+        <v>7867</v>
       </c>
       <c r="B173" t="s">
         <v>172</v>
@@ -16368,7 +16368,7 @@
     </row>
     <row r="174" spans="1:18">
       <c r="A174">
-        <v>7088</v>
+        <v>7870</v>
       </c>
       <c r="B174" t="s">
         <v>173</v>
@@ -16421,7 +16421,7 @@
     </row>
     <row r="175" spans="1:18">
       <c r="A175">
-        <v>6920</v>
+        <v>7702</v>
       </c>
       <c r="B175" t="s">
         <v>174</v>
@@ -16471,7 +16471,7 @@
     </row>
     <row r="176" spans="1:18">
       <c r="A176">
-        <v>6899</v>
+        <v>7681</v>
       </c>
       <c r="B176" t="s">
         <v>175</v>
@@ -16527,7 +16527,7 @@
     </row>
     <row r="177" spans="1:18">
       <c r="A177">
-        <v>7081</v>
+        <v>7863</v>
       </c>
       <c r="B177" t="s">
         <v>176</v>
@@ -16571,7 +16571,7 @@
     </row>
     <row r="178" spans="1:18">
       <c r="A178">
-        <v>7011</v>
+        <v>7793</v>
       </c>
       <c r="B178" t="s">
         <v>177</v>
@@ -16627,7 +16627,7 @@
     </row>
     <row r="179" spans="1:18">
       <c r="A179">
-        <v>7082</v>
+        <v>7864</v>
       </c>
       <c r="B179" t="s">
         <v>178</v>
@@ -16683,7 +16683,7 @@
     </row>
     <row r="180" spans="1:18">
       <c r="A180">
-        <v>6880</v>
+        <v>7662</v>
       </c>
       <c r="B180" t="s">
         <v>179</v>
@@ -16739,7 +16739,7 @@
     </row>
     <row r="181" spans="1:18">
       <c r="A181">
-        <v>6781</v>
+        <v>7563</v>
       </c>
       <c r="B181" t="s">
         <v>180</v>
@@ -16789,7 +16789,7 @@
     </row>
     <row r="182" spans="1:18">
       <c r="A182">
-        <v>6778</v>
+        <v>7560</v>
       </c>
       <c r="B182" t="s">
         <v>181</v>
@@ -16842,7 +16842,7 @@
     </row>
     <row r="183" spans="1:18">
       <c r="A183">
-        <v>6774</v>
+        <v>7556</v>
       </c>
       <c r="B183" t="s">
         <v>182</v>
@@ -16892,7 +16892,7 @@
     </row>
     <row r="184" spans="1:18">
       <c r="A184">
-        <v>6843</v>
+        <v>7625</v>
       </c>
       <c r="B184" t="s">
         <v>183</v>
@@ -16942,7 +16942,7 @@
     </row>
     <row r="185" spans="1:18">
       <c r="A185">
-        <v>7103</v>
+        <v>7885</v>
       </c>
       <c r="B185" t="s">
         <v>184</v>
@@ -16998,7 +16998,7 @@
     </row>
     <row r="186" spans="1:18">
       <c r="A186">
-        <v>6917</v>
+        <v>7699</v>
       </c>
       <c r="B186" t="s">
         <v>185</v>
@@ -17054,7 +17054,7 @@
     </row>
     <row r="187" spans="1:18">
       <c r="A187">
-        <v>6918</v>
+        <v>7700</v>
       </c>
       <c r="B187" t="s">
         <v>186</v>
@@ -17110,7 +17110,7 @@
     </row>
     <row r="188" spans="1:18">
       <c r="A188">
-        <v>7108</v>
+        <v>7890</v>
       </c>
       <c r="B188" t="s">
         <v>187</v>
@@ -17166,7 +17166,7 @@
     </row>
     <row r="189" spans="1:18">
       <c r="A189">
-        <v>6806</v>
+        <v>7588</v>
       </c>
       <c r="B189" t="s">
         <v>188</v>
@@ -17219,7 +17219,7 @@
     </row>
     <row r="190" spans="1:18">
       <c r="A190">
-        <v>6807</v>
+        <v>7589</v>
       </c>
       <c r="B190" t="s">
         <v>188</v>
@@ -17272,7 +17272,7 @@
     </row>
     <row r="191" spans="1:18">
       <c r="A191">
-        <v>7056</v>
+        <v>7838</v>
       </c>
       <c r="B191" t="s">
         <v>189</v>
@@ -17328,7 +17328,7 @@
     </row>
     <row r="192" spans="1:18">
       <c r="A192">
-        <v>7051</v>
+        <v>7833</v>
       </c>
       <c r="B192" t="s">
         <v>190</v>
@@ -17384,7 +17384,7 @@
     </row>
     <row r="193" spans="1:18">
       <c r="A193">
-        <v>6919</v>
+        <v>7701</v>
       </c>
       <c r="B193" t="s">
         <v>191</v>
@@ -17440,7 +17440,7 @@
     </row>
     <row r="194" spans="1:18">
       <c r="A194">
-        <v>7038</v>
+        <v>7820</v>
       </c>
       <c r="B194" t="s">
         <v>192</v>
@@ -17493,7 +17493,7 @@
     </row>
     <row r="195" spans="1:18">
       <c r="A195">
-        <v>7039</v>
+        <v>7821</v>
       </c>
       <c r="B195" t="s">
         <v>192</v>
@@ -17546,7 +17546,7 @@
     </row>
     <row r="196" spans="1:18">
       <c r="A196">
-        <v>7084</v>
+        <v>7866</v>
       </c>
       <c r="B196" t="s">
         <v>193</v>
@@ -17596,7 +17596,7 @@
     </row>
     <row r="197" spans="1:18">
       <c r="A197">
-        <v>6952</v>
+        <v>7734</v>
       </c>
       <c r="B197" t="s">
         <v>194</v>
@@ -17652,7 +17652,7 @@
     </row>
     <row r="198" spans="1:18">
       <c r="A198">
-        <v>7110</v>
+        <v>7892</v>
       </c>
       <c r="B198" t="s">
         <v>195</v>
@@ -17708,7 +17708,7 @@
     </row>
     <row r="199" spans="1:18">
       <c r="A199">
-        <v>7087</v>
+        <v>7869</v>
       </c>
       <c r="B199" t="s">
         <v>196</v>
@@ -17761,7 +17761,7 @@
     </row>
     <row r="200" spans="1:18">
       <c r="A200">
-        <v>6793</v>
+        <v>7575</v>
       </c>
       <c r="B200" t="s">
         <v>197</v>
@@ -17817,7 +17817,7 @@
     </row>
     <row r="201" spans="1:18">
       <c r="A201">
-        <v>6794</v>
+        <v>7576</v>
       </c>
       <c r="B201" t="s">
         <v>197</v>
@@ -17873,7 +17873,7 @@
     </row>
     <row r="202" spans="1:18">
       <c r="A202">
-        <v>6795</v>
+        <v>7577</v>
       </c>
       <c r="B202" t="s">
         <v>197</v>
@@ -17929,7 +17929,7 @@
     </row>
     <row r="203" spans="1:18">
       <c r="A203">
-        <v>6868</v>
+        <v>7650</v>
       </c>
       <c r="B203" t="s">
         <v>198</v>
@@ -17985,7 +17985,7 @@
     </row>
     <row r="204" spans="1:18">
       <c r="A204">
-        <v>6869</v>
+        <v>7651</v>
       </c>
       <c r="B204" t="s">
         <v>198</v>
@@ -18041,7 +18041,7 @@
     </row>
     <row r="205" spans="1:18">
       <c r="A205">
-        <v>6887</v>
+        <v>7669</v>
       </c>
       <c r="B205" t="s">
         <v>199</v>
@@ -18097,7 +18097,7 @@
     </row>
     <row r="206" spans="1:18">
       <c r="A206">
-        <v>6780</v>
+        <v>7562</v>
       </c>
       <c r="B206" t="s">
         <v>200</v>
@@ -18144,7 +18144,7 @@
     </row>
     <row r="207" spans="1:18">
       <c r="A207">
-        <v>7094</v>
+        <v>7876</v>
       </c>
       <c r="B207" t="s">
         <v>201</v>
@@ -18200,7 +18200,7 @@
     </row>
     <row r="208" spans="1:18">
       <c r="A208">
-        <v>7095</v>
+        <v>7877</v>
       </c>
       <c r="B208" t="s">
         <v>201</v>
@@ -18256,7 +18256,7 @@
     </row>
     <row r="209" spans="1:18">
       <c r="A209">
-        <v>7097</v>
+        <v>7879</v>
       </c>
       <c r="B209" t="s">
         <v>202</v>
@@ -18312,7 +18312,7 @@
     </row>
     <row r="210" spans="1:18">
       <c r="A210">
-        <v>6841</v>
+        <v>7623</v>
       </c>
       <c r="B210" t="s">
         <v>203</v>
@@ -18362,7 +18362,7 @@
     </row>
     <row r="211" spans="1:18">
       <c r="A211">
-        <v>7105</v>
+        <v>7887</v>
       </c>
       <c r="B211" t="s">
         <v>204</v>
@@ -18388,7 +18388,7 @@
     </row>
     <row r="212" spans="1:18">
       <c r="A212">
-        <v>6906</v>
+        <v>7688</v>
       </c>
       <c r="B212" t="s">
         <v>205</v>
@@ -18444,7 +18444,7 @@
     </row>
     <row r="213" spans="1:18">
       <c r="A213">
-        <v>6851</v>
+        <v>7633</v>
       </c>
       <c r="B213" t="s">
         <v>206</v>
@@ -18500,7 +18500,7 @@
     </row>
     <row r="214" spans="1:18">
       <c r="A214">
-        <v>6844</v>
+        <v>7626</v>
       </c>
       <c r="B214" t="s">
         <v>207</v>
@@ -18550,7 +18550,7 @@
     </row>
     <row r="215" spans="1:18">
       <c r="A215">
-        <v>6862</v>
+        <v>7644</v>
       </c>
       <c r="B215" t="s">
         <v>208</v>
@@ -18603,7 +18603,7 @@
     </row>
     <row r="216" spans="1:18">
       <c r="A216">
-        <v>7049</v>
+        <v>7831</v>
       </c>
       <c r="B216" t="s">
         <v>209</v>
@@ -18659,7 +18659,7 @@
     </row>
     <row r="217" spans="1:18">
       <c r="A217">
-        <v>6850</v>
+        <v>7632</v>
       </c>
       <c r="B217" t="s">
         <v>210</v>
@@ -18715,7 +18715,7 @@
     </row>
     <row r="218" spans="1:18">
       <c r="A218">
-        <v>6837</v>
+        <v>7619</v>
       </c>
       <c r="B218" t="s">
         <v>211</v>
@@ -18765,7 +18765,7 @@
     </row>
     <row r="219" spans="1:18">
       <c r="A219">
-        <v>6777</v>
+        <v>7559</v>
       </c>
       <c r="B219" t="s">
         <v>212</v>
@@ -18818,7 +18818,7 @@
     </row>
     <row r="220" spans="1:18">
       <c r="A220">
-        <v>7089</v>
+        <v>7871</v>
       </c>
       <c r="B220" t="s">
         <v>213</v>
@@ -18871,7 +18871,7 @@
     </row>
     <row r="221" spans="1:18">
       <c r="A221">
-        <v>7070</v>
+        <v>7852</v>
       </c>
       <c r="B221" t="s">
         <v>214</v>
@@ -18927,7 +18927,7 @@
     </row>
     <row r="222" spans="1:18">
       <c r="A222">
-        <v>6877</v>
+        <v>7659</v>
       </c>
       <c r="B222" t="s">
         <v>215</v>
@@ -18983,7 +18983,7 @@
     </row>
     <row r="223" spans="1:18">
       <c r="A223">
-        <v>6900</v>
+        <v>7682</v>
       </c>
       <c r="B223" t="s">
         <v>216</v>
@@ -19039,7 +19039,7 @@
     </row>
     <row r="224" spans="1:18">
       <c r="A224">
-        <v>6955</v>
+        <v>7737</v>
       </c>
       <c r="B224" t="s">
         <v>217</v>
@@ -19095,7 +19095,7 @@
     </row>
     <row r="225" spans="1:18">
       <c r="A225">
-        <v>7102</v>
+        <v>7884</v>
       </c>
       <c r="B225" t="s">
         <v>218</v>
@@ -19151,7 +19151,7 @@
     </row>
     <row r="226" spans="1:18">
       <c r="A226">
-        <v>6827</v>
+        <v>7609</v>
       </c>
       <c r="B226" t="s">
         <v>219</v>
@@ -19201,7 +19201,7 @@
     </row>
     <row r="227" spans="1:18">
       <c r="A227">
-        <v>6940</v>
+        <v>7722</v>
       </c>
       <c r="B227" t="s">
         <v>220</v>
@@ -19257,7 +19257,7 @@
     </row>
     <row r="228" spans="1:18">
       <c r="A228">
-        <v>6787</v>
+        <v>7569</v>
       </c>
       <c r="B228" t="s">
         <v>221</v>
@@ -19310,7 +19310,7 @@
     </row>
     <row r="229" spans="1:18">
       <c r="A229">
-        <v>6879</v>
+        <v>7661</v>
       </c>
       <c r="B229" t="s">
         <v>222</v>
@@ -19366,7 +19366,7 @@
     </row>
     <row r="230" spans="1:18">
       <c r="A230">
-        <v>6820</v>
+        <v>7602</v>
       </c>
       <c r="B230" t="s">
         <v>223</v>
@@ -19419,7 +19419,7 @@
     </row>
     <row r="231" spans="1:18">
       <c r="A231">
-        <v>6818</v>
+        <v>7600</v>
       </c>
       <c r="B231" t="s">
         <v>224</v>
@@ -19475,7 +19475,7 @@
     </row>
     <row r="232" spans="1:18">
       <c r="A232">
-        <v>6815</v>
+        <v>7597</v>
       </c>
       <c r="B232" t="s">
         <v>225</v>
@@ -19528,7 +19528,7 @@
     </row>
     <row r="233" spans="1:18">
       <c r="A233">
-        <v>6772</v>
+        <v>7554</v>
       </c>
       <c r="B233" t="s">
         <v>226</v>
@@ -19581,7 +19581,7 @@
     </row>
     <row r="234" spans="1:18">
       <c r="A234">
-        <v>7012</v>
+        <v>7794</v>
       </c>
       <c r="B234" t="s">
         <v>227</v>
@@ -19634,7 +19634,7 @@
     </row>
     <row r="235" spans="1:18">
       <c r="A235">
-        <v>6845</v>
+        <v>7627</v>
       </c>
       <c r="B235" t="s">
         <v>228</v>
@@ -19672,7 +19672,7 @@
     </row>
     <row r="236" spans="1:18">
       <c r="A236">
-        <v>6840</v>
+        <v>7622</v>
       </c>
       <c r="B236" t="s">
         <v>229</v>
@@ -19725,7 +19725,7 @@
     </row>
     <row r="237" spans="1:18">
       <c r="A237">
-        <v>6947</v>
+        <v>7729</v>
       </c>
       <c r="B237" t="s">
         <v>230</v>
@@ -19775,7 +19775,7 @@
     </row>
     <row r="238" spans="1:18">
       <c r="A238">
-        <v>6842</v>
+        <v>7624</v>
       </c>
       <c r="B238" t="s">
         <v>231</v>
@@ -19825,7 +19825,7 @@
     </row>
     <row r="239" spans="1:18">
       <c r="A239">
-        <v>6783</v>
+        <v>7565</v>
       </c>
       <c r="B239" t="s">
         <v>232</v>
@@ -19878,7 +19878,7 @@
     </row>
     <row r="240" spans="1:18">
       <c r="A240">
-        <v>6784</v>
+        <v>7566</v>
       </c>
       <c r="B240" t="s">
         <v>232</v>
@@ -19931,7 +19931,7 @@
     </row>
     <row r="241" spans="1:18">
       <c r="A241">
-        <v>6885</v>
+        <v>7667</v>
       </c>
       <c r="B241" t="s">
         <v>233</v>
@@ -19987,7 +19987,7 @@
     </row>
     <row r="242" spans="1:18">
       <c r="A242">
-        <v>6788</v>
+        <v>7570</v>
       </c>
       <c r="B242" t="s">
         <v>234</v>
@@ -20040,7 +20040,7 @@
     </row>
     <row r="243" spans="1:18">
       <c r="A243">
-        <v>7067</v>
+        <v>7849</v>
       </c>
       <c r="B243" t="s">
         <v>235</v>
@@ -20096,7 +20096,7 @@
     </row>
     <row r="244" spans="1:18">
       <c r="A244">
-        <v>6822</v>
+        <v>7604</v>
       </c>
       <c r="B244" t="s">
         <v>236</v>
@@ -20146,7 +20146,7 @@
     </row>
     <row r="245" spans="1:18">
       <c r="A245">
-        <v>6817</v>
+        <v>7599</v>
       </c>
       <c r="B245" t="s">
         <v>237</v>
@@ -20202,7 +20202,7 @@
     </row>
     <row r="246" spans="1:18">
       <c r="A246">
-        <v>7069</v>
+        <v>7851</v>
       </c>
       <c r="B246" t="s">
         <v>238</v>
@@ -20258,7 +20258,7 @@
     </row>
     <row r="247" spans="1:18">
       <c r="A247">
-        <v>7068</v>
+        <v>7850</v>
       </c>
       <c r="B247" t="s">
         <v>239</v>
@@ -20314,7 +20314,7 @@
     </row>
     <row r="248" spans="1:18">
       <c r="A248">
-        <v>6791</v>
+        <v>7573</v>
       </c>
       <c r="B248" t="s">
         <v>240</v>
@@ -20370,7 +20370,7 @@
     </row>
     <row r="249" spans="1:18">
       <c r="A249">
-        <v>6865</v>
+        <v>7647</v>
       </c>
       <c r="B249" t="s">
         <v>241</v>
@@ -20420,7 +20420,7 @@
     </row>
     <row r="250" spans="1:18">
       <c r="A250">
-        <v>6925</v>
+        <v>7707</v>
       </c>
       <c r="B250" t="s">
         <v>242</v>
@@ -20470,7 +20470,7 @@
     </row>
     <row r="251" spans="1:18">
       <c r="A251">
-        <v>7019</v>
+        <v>7801</v>
       </c>
       <c r="B251" t="s">
         <v>243</v>
@@ -20523,7 +20523,7 @@
     </row>
     <row r="252" spans="1:18">
       <c r="A252">
-        <v>6968</v>
+        <v>7750</v>
       </c>
       <c r="B252" t="s">
         <v>244</v>
@@ -20567,7 +20567,7 @@
     </row>
     <row r="253" spans="1:18">
       <c r="A253">
-        <v>6926</v>
+        <v>7708</v>
       </c>
       <c r="B253" t="s">
         <v>245</v>
@@ -20620,7 +20620,7 @@
     </row>
     <row r="254" spans="1:18">
       <c r="A254">
-        <v>6927</v>
+        <v>7709</v>
       </c>
       <c r="B254" t="s">
         <v>245</v>
@@ -20676,7 +20676,7 @@
     </row>
     <row r="255" spans="1:18">
       <c r="A255">
-        <v>6930</v>
+        <v>7712</v>
       </c>
       <c r="B255" t="s">
         <v>246</v>
@@ -20729,7 +20729,7 @@
     </row>
     <row r="256" spans="1:18">
       <c r="A256">
-        <v>6889</v>
+        <v>7671</v>
       </c>
       <c r="B256" t="s">
         <v>247</v>
@@ -20773,7 +20773,7 @@
     </row>
     <row r="257" spans="1:18">
       <c r="A257">
-        <v>6801</v>
+        <v>7583</v>
       </c>
       <c r="B257" t="s">
         <v>248</v>
@@ -20826,7 +20826,7 @@
     </row>
     <row r="258" spans="1:18">
       <c r="A258">
-        <v>6802</v>
+        <v>7584</v>
       </c>
       <c r="B258" t="s">
         <v>248</v>
@@ -20879,7 +20879,7 @@
     </row>
     <row r="259" spans="1:18">
       <c r="A259">
-        <v>6808</v>
+        <v>7590</v>
       </c>
       <c r="B259" t="s">
         <v>249</v>
@@ -20935,7 +20935,7 @@
     </row>
     <row r="260" spans="1:18">
       <c r="A260">
-        <v>7041</v>
+        <v>7823</v>
       </c>
       <c r="B260" t="s">
         <v>250</v>
@@ -20991,7 +20991,7 @@
     </row>
     <row r="261" spans="1:18">
       <c r="A261">
-        <v>7042</v>
+        <v>7824</v>
       </c>
       <c r="B261" t="s">
         <v>250</v>
@@ -21047,7 +21047,7 @@
     </row>
     <row r="262" spans="1:18">
       <c r="A262">
-        <v>7043</v>
+        <v>7825</v>
       </c>
       <c r="B262" t="s">
         <v>250</v>
@@ -21103,7 +21103,7 @@
     </row>
     <row r="263" spans="1:18">
       <c r="A263">
-        <v>7047</v>
+        <v>7829</v>
       </c>
       <c r="B263" t="s">
         <v>251</v>
@@ -21159,7 +21159,7 @@
     </row>
     <row r="264" spans="1:18">
       <c r="A264">
-        <v>7045</v>
+        <v>7827</v>
       </c>
       <c r="B264" t="s">
         <v>252</v>
@@ -21215,7 +21215,7 @@
     </row>
     <row r="265" spans="1:18">
       <c r="A265">
-        <v>7046</v>
+        <v>7828</v>
       </c>
       <c r="B265" t="s">
         <v>252</v>
@@ -21271,7 +21271,7 @@
     </row>
     <row r="266" spans="1:18">
       <c r="A266">
-        <v>6953</v>
+        <v>7735</v>
       </c>
       <c r="B266" t="s">
         <v>253</v>
@@ -21327,7 +21327,7 @@
     </row>
     <row r="267" spans="1:18">
       <c r="A267">
-        <v>6881</v>
+        <v>7663</v>
       </c>
       <c r="B267" t="s">
         <v>254</v>
@@ -21383,7 +21383,7 @@
     </row>
     <row r="268" spans="1:18">
       <c r="A268">
-        <v>6864</v>
+        <v>7646</v>
       </c>
       <c r="B268" t="s">
         <v>255</v>
@@ -21439,7 +21439,7 @@
     </row>
     <row r="269" spans="1:18">
       <c r="A269">
-        <v>6857</v>
+        <v>7639</v>
       </c>
       <c r="B269" t="s">
         <v>256</v>
@@ -21495,7 +21495,7 @@
     </row>
     <row r="270" spans="1:18">
       <c r="A270">
-        <v>6805</v>
+        <v>7587</v>
       </c>
       <c r="B270" t="s">
         <v>257</v>
@@ -21548,7 +21548,7 @@
     </row>
     <row r="271" spans="1:18">
       <c r="A271">
-        <v>7060</v>
+        <v>7842</v>
       </c>
       <c r="B271" t="s">
         <v>258</v>
@@ -21598,7 +21598,7 @@
     </row>
     <row r="272" spans="1:18">
       <c r="A272">
-        <v>7050</v>
+        <v>7832</v>
       </c>
       <c r="B272" t="s">
         <v>259</v>
@@ -21654,7 +21654,7 @@
     </row>
     <row r="273" spans="1:18">
       <c r="A273">
-        <v>6875</v>
+        <v>7657</v>
       </c>
       <c r="B273" t="s">
         <v>260</v>
@@ -21692,7 +21692,7 @@
     </row>
     <row r="274" spans="1:18">
       <c r="A274">
-        <v>6876</v>
+        <v>7658</v>
       </c>
       <c r="B274" t="s">
         <v>260</v>
@@ -21730,7 +21730,7 @@
     </row>
     <row r="275" spans="1:18">
       <c r="A275">
-        <v>6890</v>
+        <v>7672</v>
       </c>
       <c r="B275" t="s">
         <v>261</v>
@@ -21768,7 +21768,7 @@
     </row>
     <row r="276" spans="1:18">
       <c r="A276">
-        <v>7023</v>
+        <v>7805</v>
       </c>
       <c r="B276" t="s">
         <v>262</v>
@@ -21821,7 +21821,7 @@
     </row>
     <row r="277" spans="1:18">
       <c r="A277">
-        <v>7048</v>
+        <v>7830</v>
       </c>
       <c r="B277" t="s">
         <v>263</v>
@@ -21877,7 +21877,7 @@
     </row>
     <row r="278" spans="1:18">
       <c r="A278">
-        <v>6830</v>
+        <v>7612</v>
       </c>
       <c r="B278" t="s">
         <v>264</v>
@@ -21927,7 +21927,7 @@
     </row>
     <row r="279" spans="1:18">
       <c r="A279">
-        <v>6839</v>
+        <v>7621</v>
       </c>
       <c r="B279" t="s">
         <v>265</v>
@@ -21971,7 +21971,7 @@
     </row>
     <row r="280" spans="1:18">
       <c r="A280">
-        <v>7090</v>
+        <v>7872</v>
       </c>
       <c r="B280" t="s">
         <v>266</v>
@@ -22024,7 +22024,7 @@
     </row>
     <row r="281" spans="1:18">
       <c r="A281">
-        <v>6831</v>
+        <v>7613</v>
       </c>
       <c r="B281" t="s">
         <v>267</v>
@@ -22074,7 +22074,7 @@
     </row>
     <row r="282" spans="1:18">
       <c r="A282">
-        <v>6910</v>
+        <v>7692</v>
       </c>
       <c r="B282" t="s">
         <v>268</v>
@@ -22130,7 +22130,7 @@
     </row>
     <row r="283" spans="1:18">
       <c r="A283">
-        <v>6905</v>
+        <v>7687</v>
       </c>
       <c r="B283" t="s">
         <v>269</v>
@@ -22186,7 +22186,7 @@
     </row>
     <row r="284" spans="1:18">
       <c r="A284">
-        <v>7020</v>
+        <v>7802</v>
       </c>
       <c r="B284" t="s">
         <v>270</v>
@@ -22239,7 +22239,7 @@
     </row>
     <row r="285" spans="1:18">
       <c r="A285">
-        <v>6779</v>
+        <v>7561</v>
       </c>
       <c r="B285" t="s">
         <v>271</v>
@@ -22292,7 +22292,7 @@
     </row>
     <row r="286" spans="1:18">
       <c r="A286">
-        <v>6904</v>
+        <v>7686</v>
       </c>
       <c r="B286" t="s">
         <v>272</v>
@@ -22345,7 +22345,7 @@
     </row>
     <row r="287" spans="1:18">
       <c r="A287">
-        <v>6938</v>
+        <v>7720</v>
       </c>
       <c r="B287" t="s">
         <v>273</v>
@@ -22401,7 +22401,7 @@
     </row>
     <row r="288" spans="1:18">
       <c r="A288">
-        <v>6966</v>
+        <v>7748</v>
       </c>
       <c r="B288" t="s">
         <v>274</v>
@@ -22454,7 +22454,7 @@
     </row>
     <row r="289" spans="1:18">
       <c r="A289">
-        <v>6893</v>
+        <v>7675</v>
       </c>
       <c r="B289" t="s">
         <v>275</v>
@@ -22510,7 +22510,7 @@
     </row>
     <row r="290" spans="1:18">
       <c r="A290">
-        <v>7113</v>
+        <v>7895</v>
       </c>
       <c r="B290" t="s">
         <v>276</v>
@@ -22566,7 +22566,7 @@
     </row>
     <row r="291" spans="1:18">
       <c r="A291">
-        <v>7054</v>
+        <v>7836</v>
       </c>
       <c r="B291" t="s">
         <v>277</v>
@@ -22622,7 +22622,7 @@
     </row>
     <row r="292" spans="1:18">
       <c r="A292">
-        <v>7052</v>
+        <v>7834</v>
       </c>
       <c r="B292" t="s">
         <v>278</v>
@@ -22678,7 +22678,7 @@
     </row>
     <row r="293" spans="1:18">
       <c r="A293">
-        <v>7007</v>
+        <v>7789</v>
       </c>
       <c r="B293" t="s">
         <v>279</v>
@@ -22731,7 +22731,7 @@
     </row>
     <row r="294" spans="1:18">
       <c r="A294">
-        <v>6770</v>
+        <v>7552</v>
       </c>
       <c r="B294" t="s">
         <v>280</v>
@@ -22772,7 +22772,7 @@
     </row>
     <row r="295" spans="1:18">
       <c r="A295">
-        <v>7063</v>
+        <v>7845</v>
       </c>
       <c r="B295" t="s">
         <v>281</v>
@@ -22822,7 +22822,7 @@
     </row>
     <row r="296" spans="1:18">
       <c r="A296">
-        <v>6819</v>
+        <v>7601</v>
       </c>
       <c r="B296" t="s">
         <v>282</v>
@@ -22878,7 +22878,7 @@
     </row>
     <row r="297" spans="1:18">
       <c r="A297">
-        <v>6823</v>
+        <v>7605</v>
       </c>
       <c r="B297" t="s">
         <v>283</v>
@@ -22934,7 +22934,7 @@
     </row>
     <row r="298" spans="1:18">
       <c r="A298">
-        <v>6945</v>
+        <v>7727</v>
       </c>
       <c r="B298" t="s">
         <v>284</v>
@@ -22990,7 +22990,7 @@
     </row>
     <row r="299" spans="1:18">
       <c r="A299">
-        <v>6897</v>
+        <v>7679</v>
       </c>
       <c r="B299" t="s">
         <v>285</v>
@@ -23034,7 +23034,7 @@
     </row>
     <row r="300" spans="1:18">
       <c r="A300">
-        <v>7079</v>
+        <v>7861</v>
       </c>
       <c r="B300" t="s">
         <v>286</v>
@@ -23090,7 +23090,7 @@
     </row>
     <row r="301" spans="1:18">
       <c r="A301">
-        <v>7077</v>
+        <v>7859</v>
       </c>
       <c r="B301" t="s">
         <v>287</v>
@@ -23146,7 +23146,7 @@
     </row>
     <row r="302" spans="1:18">
       <c r="A302">
-        <v>7112</v>
+        <v>7894</v>
       </c>
       <c r="B302" t="s">
         <v>288</v>
@@ -23199,7 +23199,7 @@
     </row>
     <row r="303" spans="1:18">
       <c r="A303">
-        <v>7104</v>
+        <v>7886</v>
       </c>
       <c r="B303" t="s">
         <v>289</v>
@@ -23255,7 +23255,7 @@
     </row>
     <row r="304" spans="1:18">
       <c r="A304">
-        <v>6824</v>
+        <v>7606</v>
       </c>
       <c r="B304" t="s">
         <v>290</v>
@@ -23311,7 +23311,7 @@
     </row>
     <row r="305" spans="1:18">
       <c r="A305">
-        <v>7092</v>
+        <v>7874</v>
       </c>
       <c r="B305" t="s">
         <v>291</v>
@@ -23367,7 +23367,7 @@
     </row>
     <row r="306" spans="1:18">
       <c r="A306">
-        <v>6785</v>
+        <v>7567</v>
       </c>
       <c r="B306" t="s">
         <v>292</v>
@@ -23417,7 +23417,7 @@
     </row>
     <row r="307" spans="1:18">
       <c r="A307">
-        <v>6985</v>
+        <v>7767</v>
       </c>
       <c r="B307" t="s">
         <v>293</v>
@@ -23458,7 +23458,7 @@
     </row>
     <row r="308" spans="1:18">
       <c r="A308">
-        <v>7071</v>
+        <v>7853</v>
       </c>
       <c r="B308" t="s">
         <v>294</v>
@@ -23514,7 +23514,7 @@
     </row>
     <row r="309" spans="1:18">
       <c r="A309">
-        <v>7059</v>
+        <v>7841</v>
       </c>
       <c r="B309" t="s">
         <v>295</v>
@@ -23564,7 +23564,7 @@
     </row>
     <row r="310" spans="1:18">
       <c r="A310">
-        <v>6858</v>
+        <v>7640</v>
       </c>
       <c r="B310" t="s">
         <v>296</v>
@@ -23620,7 +23620,7 @@
     </row>
     <row r="311" spans="1:18">
       <c r="A311">
-        <v>6923</v>
+        <v>7705</v>
       </c>
       <c r="B311" t="s">
         <v>297</v>
@@ -23673,7 +23673,7 @@
     </row>
     <row r="312" spans="1:18">
       <c r="A312">
-        <v>7044</v>
+        <v>7826</v>
       </c>
       <c r="B312" t="s">
         <v>298</v>
@@ -23717,7 +23717,7 @@
     </row>
     <row r="313" spans="1:18">
       <c r="A313">
-        <v>6907</v>
+        <v>7689</v>
       </c>
       <c r="B313" t="s">
         <v>299</v>
@@ -23773,7 +23773,7 @@
     </row>
     <row r="314" spans="1:18">
       <c r="A314">
-        <v>7034</v>
+        <v>7816</v>
       </c>
       <c r="B314" t="s">
         <v>300</v>
@@ -23829,7 +23829,7 @@
     </row>
     <row r="315" spans="1:18">
       <c r="A315">
-        <v>6775</v>
+        <v>7557</v>
       </c>
       <c r="B315" t="s">
         <v>301</v>
@@ -23879,7 +23879,7 @@
     </row>
     <row r="316" spans="1:18">
       <c r="A316">
-        <v>6776</v>
+        <v>7558</v>
       </c>
       <c r="B316" t="s">
         <v>301</v>
@@ -23929,7 +23929,7 @@
     </row>
     <row r="317" spans="1:18">
       <c r="A317">
-        <v>7057</v>
+        <v>7839</v>
       </c>
       <c r="B317" t="s">
         <v>302</v>
@@ -23979,7 +23979,7 @@
     </row>
     <row r="318" spans="1:18">
       <c r="A318">
-        <v>7115</v>
+        <v>7897</v>
       </c>
       <c r="B318" t="s">
         <v>303</v>
@@ -24032,7 +24032,7 @@
     </row>
     <row r="319" spans="1:18">
       <c r="A319">
-        <v>7066</v>
+        <v>7848</v>
       </c>
       <c r="B319" t="s">
         <v>304</v>
@@ -24076,7 +24076,7 @@
     </row>
     <row r="320" spans="1:18">
       <c r="A320">
-        <v>6969</v>
+        <v>7751</v>
       </c>
       <c r="B320" t="s">
         <v>305</v>
@@ -24123,7 +24123,7 @@
     </row>
     <row r="321" spans="1:18">
       <c r="A321">
-        <v>6970</v>
+        <v>7752</v>
       </c>
       <c r="B321" t="s">
         <v>305</v>
@@ -24173,7 +24173,7 @@
     </row>
     <row r="322" spans="1:18">
       <c r="A322">
-        <v>6972</v>
+        <v>7754</v>
       </c>
       <c r="B322" t="s">
         <v>306</v>
@@ -24220,7 +24220,7 @@
     </row>
     <row r="323" spans="1:18">
       <c r="A323">
-        <v>6960</v>
+        <v>7742</v>
       </c>
       <c r="B323" t="s">
         <v>307</v>
@@ -24276,7 +24276,7 @@
     </row>
     <row r="324" spans="1:18">
       <c r="A324">
-        <v>6941</v>
+        <v>7723</v>
       </c>
       <c r="B324" t="s">
         <v>308</v>
@@ -24332,7 +24332,7 @@
     </row>
     <row r="325" spans="1:18">
       <c r="A325">
-        <v>6987</v>
+        <v>7769</v>
       </c>
       <c r="B325" t="s">
         <v>309</v>
@@ -24385,7 +24385,7 @@
     </row>
     <row r="326" spans="1:18">
       <c r="A326">
-        <v>6988</v>
+        <v>7770</v>
       </c>
       <c r="B326" t="s">
         <v>309</v>
@@ -24438,7 +24438,7 @@
     </row>
     <row r="327" spans="1:18">
       <c r="A327">
-        <v>7000</v>
+        <v>7782</v>
       </c>
       <c r="B327" t="s">
         <v>310</v>
@@ -24494,7 +24494,7 @@
     </row>
     <row r="328" spans="1:18">
       <c r="A328">
-        <v>6932</v>
+        <v>7714</v>
       </c>
       <c r="B328" t="s">
         <v>311</v>
@@ -24541,7 +24541,7 @@
     </row>
     <row r="329" spans="1:18">
       <c r="A329">
-        <v>6933</v>
+        <v>7715</v>
       </c>
       <c r="B329" t="s">
         <v>311</v>
@@ -24591,7 +24591,7 @@
     </row>
     <row r="330" spans="1:18">
       <c r="A330">
-        <v>6973</v>
+        <v>7755</v>
       </c>
       <c r="B330" t="s">
         <v>312</v>
@@ -24638,7 +24638,7 @@
     </row>
     <row r="331" spans="1:18">
       <c r="A331">
-        <v>6991</v>
+        <v>7773</v>
       </c>
       <c r="B331" t="s">
         <v>313</v>
@@ -24691,7 +24691,7 @@
     </row>
     <row r="332" spans="1:18">
       <c r="A332">
-        <v>6992</v>
+        <v>7774</v>
       </c>
       <c r="B332" t="s">
         <v>313</v>
@@ -24744,7 +24744,7 @@
     </row>
     <row r="333" spans="1:18">
       <c r="A333">
-        <v>6995</v>
+        <v>7777</v>
       </c>
       <c r="B333" t="s">
         <v>314</v>
@@ -24785,7 +24785,7 @@
     </row>
     <row r="334" spans="1:18">
       <c r="A334">
-        <v>6996</v>
+        <v>7778</v>
       </c>
       <c r="B334" t="s">
         <v>314</v>
@@ -24826,7 +24826,7 @@
     </row>
     <row r="335" spans="1:18">
       <c r="A335">
-        <v>7002</v>
+        <v>7784</v>
       </c>
       <c r="B335" t="s">
         <v>315</v>
@@ -24882,7 +24882,7 @@
     </row>
     <row r="336" spans="1:18">
       <c r="A336">
-        <v>7005</v>
+        <v>7787</v>
       </c>
       <c r="B336" t="s">
         <v>316</v>
@@ -24926,7 +24926,7 @@
     </row>
     <row r="337" spans="1:18">
       <c r="A337">
-        <v>6914</v>
+        <v>7696</v>
       </c>
       <c r="B337" t="s">
         <v>317</v>
@@ -24982,7 +24982,7 @@
     </row>
     <row r="338" spans="1:18">
       <c r="A338">
-        <v>7024</v>
+        <v>7806</v>
       </c>
       <c r="B338" t="s">
         <v>318</v>
@@ -25035,7 +25035,7 @@
     </row>
     <row r="339" spans="1:18">
       <c r="A339">
-        <v>6922</v>
+        <v>7704</v>
       </c>
       <c r="B339" t="s">
         <v>319</v>
@@ -25091,7 +25091,7 @@
     </row>
     <row r="340" spans="1:18">
       <c r="A340">
-        <v>6964</v>
+        <v>7746</v>
       </c>
       <c r="B340" t="s">
         <v>320</v>
@@ -25135,7 +25135,7 @@
     </row>
     <row r="341" spans="1:18">
       <c r="A341">
-        <v>7109</v>
+        <v>7891</v>
       </c>
       <c r="B341" t="s">
         <v>321</v>
@@ -25191,7 +25191,7 @@
     </row>
     <row r="342" spans="1:18">
       <c r="A342">
-        <v>6898</v>
+        <v>7680</v>
       </c>
       <c r="B342" t="s">
         <v>322</v>
@@ -25247,7 +25247,7 @@
     </row>
     <row r="343" spans="1:18">
       <c r="A343">
-        <v>7091</v>
+        <v>7873</v>
       </c>
       <c r="B343" t="s">
         <v>323</v>
@@ -25300,7 +25300,7 @@
     </row>
     <row r="344" spans="1:18">
       <c r="A344">
-        <v>6962</v>
+        <v>7744</v>
       </c>
       <c r="B344" t="s">
         <v>324</v>
@@ -25356,7 +25356,7 @@
     </row>
     <row r="345" spans="1:18">
       <c r="A345">
-        <v>6825</v>
+        <v>7607</v>
       </c>
       <c r="B345" t="s">
         <v>325</v>
@@ -25412,7 +25412,7 @@
     </row>
     <row r="346" spans="1:18">
       <c r="A346">
-        <v>7101</v>
+        <v>7883</v>
       </c>
       <c r="B346" t="s">
         <v>326</v>
@@ -25462,7 +25462,7 @@
     </row>
     <row r="347" spans="1:18">
       <c r="A347">
-        <v>6826</v>
+        <v>7608</v>
       </c>
       <c r="B347" t="s">
         <v>327</v>
@@ -25512,7 +25512,7 @@
     </row>
     <row r="348" spans="1:18">
       <c r="A348">
-        <v>7116</v>
+        <v>7898</v>
       </c>
       <c r="B348" t="s">
         <v>328</v>
@@ -25562,7 +25562,7 @@
     </row>
     <row r="349" spans="1:18">
       <c r="A349">
-        <v>7117</v>
+        <v>7899</v>
       </c>
       <c r="B349" t="s">
         <v>329</v>
@@ -25618,7 +25618,7 @@
     </row>
     <row r="350" spans="1:18">
       <c r="A350">
-        <v>7118</v>
+        <v>7900</v>
       </c>
       <c r="B350" t="s">
         <v>330</v>
@@ -25665,7 +25665,7 @@
     </row>
     <row r="351" spans="1:18">
       <c r="A351">
-        <v>7119</v>
+        <v>7901</v>
       </c>
       <c r="B351" t="s">
         <v>331</v>
@@ -25718,7 +25718,7 @@
     </row>
     <row r="352" spans="1:18">
       <c r="A352">
-        <v>7121</v>
+        <v>7903</v>
       </c>
       <c r="B352" t="s">
         <v>332</v>
@@ -25771,7 +25771,7 @@
     </row>
     <row r="353" spans="1:18">
       <c r="A353">
-        <v>7120</v>
+        <v>7902</v>
       </c>
       <c r="B353" t="s">
         <v>333</v>
@@ -25815,7 +25815,7 @@
     </row>
     <row r="354" spans="1:18">
       <c r="A354">
-        <v>7122</v>
+        <v>7904</v>
       </c>
       <c r="B354" t="s">
         <v>334</v>
@@ -25871,7 +25871,7 @@
     </row>
     <row r="355" spans="1:18">
       <c r="A355">
-        <v>7123</v>
+        <v>7905</v>
       </c>
       <c r="B355" t="s">
         <v>335</v>
@@ -25909,7 +25909,7 @@
     </row>
     <row r="356" spans="1:18">
       <c r="A356">
-        <v>7128</v>
+        <v>7910</v>
       </c>
       <c r="B356" t="s">
         <v>336</v>
@@ -25962,7 +25962,7 @@
     </row>
     <row r="357" spans="1:18">
       <c r="A357">
-        <v>7127</v>
+        <v>7909</v>
       </c>
       <c r="B357" t="s">
         <v>337</v>
@@ -26012,7 +26012,7 @@
     </row>
     <row r="358" spans="1:18">
       <c r="A358">
-        <v>7125</v>
+        <v>7907</v>
       </c>
       <c r="B358" t="s">
         <v>338</v>
@@ -26068,7 +26068,7 @@
     </row>
     <row r="359" spans="1:18">
       <c r="A359">
-        <v>7126</v>
+        <v>7908</v>
       </c>
       <c r="B359" t="s">
         <v>339</v>
@@ -26118,7 +26118,7 @@
     </row>
     <row r="360" spans="1:18">
       <c r="A360">
-        <v>7124</v>
+        <v>7906</v>
       </c>
       <c r="B360" t="s">
         <v>340</v>
@@ -26168,7 +26168,7 @@
     </row>
     <row r="361" spans="1:18">
       <c r="A361">
-        <v>7131</v>
+        <v>7913</v>
       </c>
       <c r="B361" t="s">
         <v>341</v>
@@ -26212,7 +26212,7 @@
     </row>
     <row r="362" spans="1:18">
       <c r="A362">
-        <v>7130</v>
+        <v>7912</v>
       </c>
       <c r="B362" t="s">
         <v>342</v>
@@ -26262,7 +26262,7 @@
     </row>
     <row r="363" spans="1:18">
       <c r="A363">
-        <v>7129</v>
+        <v>7911</v>
       </c>
       <c r="B363" t="s">
         <v>343</v>
@@ -26300,7 +26300,7 @@
     </row>
     <row r="364" spans="1:18">
       <c r="A364">
-        <v>7138</v>
+        <v>7920</v>
       </c>
       <c r="B364" t="s">
         <v>344</v>
@@ -26335,7 +26335,7 @@
     </row>
     <row r="365" spans="1:18">
       <c r="A365">
-        <v>7132</v>
+        <v>7914</v>
       </c>
       <c r="B365" t="s">
         <v>345</v>
@@ -26379,7 +26379,7 @@
     </row>
     <row r="366" spans="1:18">
       <c r="A366">
-        <v>7133</v>
+        <v>7915</v>
       </c>
       <c r="B366" t="s">
         <v>346</v>
@@ -26432,7 +26432,7 @@
     </row>
     <row r="367" spans="1:18">
       <c r="A367">
-        <v>7139</v>
+        <v>7921</v>
       </c>
       <c r="B367" t="s">
         <v>347</v>
@@ -26485,7 +26485,7 @@
     </row>
     <row r="368" spans="1:18">
       <c r="A368">
-        <v>7140</v>
+        <v>7922</v>
       </c>
       <c r="B368" t="s">
         <v>348</v>
@@ -26523,7 +26523,7 @@
     </row>
     <row r="369" spans="1:18">
       <c r="A369">
-        <v>7137</v>
+        <v>7919</v>
       </c>
       <c r="B369" t="s">
         <v>349</v>
@@ -26579,7 +26579,7 @@
     </row>
     <row r="370" spans="1:18">
       <c r="A370">
-        <v>7134</v>
+        <v>7916</v>
       </c>
       <c r="B370" t="s">
         <v>350</v>
@@ -26626,7 +26626,7 @@
     </row>
     <row r="371" spans="1:18">
       <c r="A371">
-        <v>7135</v>
+        <v>7917</v>
       </c>
       <c r="B371" t="s">
         <v>255</v>
@@ -26679,7 +26679,7 @@
     </row>
     <row r="372" spans="1:18">
       <c r="A372">
-        <v>7136</v>
+        <v>7918</v>
       </c>
       <c r="B372" t="s">
         <v>351</v>
@@ -26732,7 +26732,7 @@
     </row>
     <row r="373" spans="1:18">
       <c r="A373">
-        <v>7141</v>
+        <v>7923</v>
       </c>
       <c r="B373" t="s">
         <v>352</v>
@@ -26782,7 +26782,7 @@
     </row>
     <row r="374" spans="1:18">
       <c r="A374">
-        <v>7144</v>
+        <v>7926</v>
       </c>
       <c r="B374" t="s">
         <v>353</v>
@@ -26832,7 +26832,7 @@
     </row>
     <row r="375" spans="1:18">
       <c r="A375">
-        <v>7143</v>
+        <v>7925</v>
       </c>
       <c r="B375" t="s">
         <v>354</v>
@@ -26888,7 +26888,7 @@
     </row>
     <row r="376" spans="1:18">
       <c r="A376">
-        <v>7145</v>
+        <v>7927</v>
       </c>
       <c r="B376" t="s">
         <v>355</v>
@@ -26938,7 +26938,7 @@
     </row>
     <row r="377" spans="1:18">
       <c r="A377">
-        <v>7142</v>
+        <v>7924</v>
       </c>
       <c r="B377" t="s">
         <v>356</v>
@@ -26976,7 +26976,7 @@
     </row>
     <row r="378" spans="1:18">
       <c r="A378">
-        <v>7148</v>
+        <v>7930</v>
       </c>
       <c r="B378" t="s">
         <v>357</v>
@@ -27020,7 +27020,7 @@
     </row>
     <row r="379" spans="1:18">
       <c r="A379">
-        <v>7147</v>
+        <v>7929</v>
       </c>
       <c r="B379" t="s">
         <v>244</v>
@@ -27061,7 +27061,7 @@
     </row>
     <row r="380" spans="1:18">
       <c r="A380">
-        <v>7146</v>
+        <v>7928</v>
       </c>
       <c r="B380" t="s">
         <v>358</v>
@@ -27117,7 +27117,7 @@
     </row>
     <row r="381" spans="1:18">
       <c r="A381">
-        <v>7151</v>
+        <v>7933</v>
       </c>
       <c r="B381" t="s">
         <v>359</v>
@@ -27167,7 +27167,7 @@
     </row>
     <row r="382" spans="1:18">
       <c r="A382">
-        <v>7150</v>
+        <v>7932</v>
       </c>
       <c r="B382" t="s">
         <v>360</v>
@@ -27223,7 +27223,7 @@
     </row>
     <row r="383" spans="1:18">
       <c r="A383">
-        <v>7152</v>
+        <v>7934</v>
       </c>
       <c r="B383" t="s">
         <v>361</v>
@@ -27273,7 +27273,7 @@
     </row>
     <row r="384" spans="1:18">
       <c r="A384">
-        <v>7149</v>
+        <v>7931</v>
       </c>
       <c r="B384" t="s">
         <v>333</v>
@@ -27317,7 +27317,7 @@
     </row>
     <row r="385" spans="1:18">
       <c r="A385">
-        <v>7154</v>
+        <v>7936</v>
       </c>
       <c r="B385" t="s">
         <v>346</v>
@@ -27370,7 +27370,7 @@
     </row>
     <row r="386" spans="1:18">
       <c r="A386">
-        <v>7158</v>
+        <v>7940</v>
       </c>
       <c r="B386" t="s">
         <v>362</v>
@@ -27414,7 +27414,7 @@
     </row>
     <row r="387" spans="1:18">
       <c r="A387">
-        <v>7153</v>
+        <v>7935</v>
       </c>
       <c r="B387" t="s">
         <v>363</v>
@@ -27458,7 +27458,7 @@
     </row>
     <row r="388" spans="1:18">
       <c r="A388">
-        <v>7157</v>
+        <v>7939</v>
       </c>
       <c r="B388" t="s">
         <v>364</v>
@@ -27493,7 +27493,7 @@
     </row>
     <row r="389" spans="1:18">
       <c r="A389">
-        <v>7156</v>
+        <v>7938</v>
       </c>
       <c r="B389" t="s">
         <v>357</v>
@@ -27531,7 +27531,7 @@
     </row>
     <row r="390" spans="1:18">
       <c r="A390">
-        <v>7155</v>
+        <v>7937</v>
       </c>
       <c r="B390" t="s">
         <v>365</v>
@@ -27572,7 +27572,7 @@
     </row>
     <row r="391" spans="1:18">
       <c r="A391">
-        <v>7159</v>
+        <v>7941</v>
       </c>
       <c r="B391" t="s">
         <v>366</v>
@@ -27625,7 +27625,7 @@
     </row>
     <row r="392" spans="1:18">
       <c r="A392">
-        <v>7160</v>
+        <v>7942</v>
       </c>
       <c r="B392" t="s">
         <v>367</v>

</xml_diff>